<commit_message>
Dati: Girone D, anticipo due gare alle 20:00
Rigenerato da Calend Bocce 2026 (1).xlsx via tools/build_data.py.
- mer 24/06: Il Boccino della Discordia vs Tironi di Bocce 22:00 -> 20:00
- gio 25/06: Mirkae vs Tironi di Bocce 21:30 -> 20:00
Classifiche invariate. Nessuna sovrapposizione di slot (campo unico).
Cache-busting asset: v=202606201207.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="221">
   <si>
     <t>data e ora</t>
   </si>
@@ -238,6 +238,9 @@
     <t>Apostadores</t>
   </si>
   <si>
+    <t>mercoledì 24/06 20:00</t>
+  </si>
+  <si>
     <t>mercoledì 24/06 20:30</t>
   </si>
   <si>
@@ -260,6 +263,9 @@
   </si>
   <si>
     <t>mercoledì 24/06 23:00</t>
+  </si>
+  <si>
+    <t>giovedì 25/06 20:00</t>
   </si>
   <si>
     <t>giovedì 25/06 20:30</t>
@@ -923,10 +929,10 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="7" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1896,128 +1902,122 @@
       <c r="A37" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C37" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="D37" s="10" t="s">
-        <v>75</v>
+      <c r="B37" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>47</v>
       </c>
       <c r="E37" s="24"/>
       <c r="F37" s="24"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D38" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B38" s="21" t="s">
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B39" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="C38" s="21" t="s">
+      <c r="C39" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="D38" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="E38" s="6"/>
-      <c r="F38" s="6"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="11" t="s">
+      <c r="D39" s="21" t="s">
         <v>78</v>
-      </c>
-      <c r="B39" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="C39" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="D39" s="17" t="s">
-        <v>44</v>
       </c>
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="B40" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C40" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>47</v>
+      <c r="B40" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C40" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D40" s="17" t="s">
+        <v>44</v>
       </c>
       <c r="E40" s="6"/>
       <c r="F40" s="6"/>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="s">
+      <c r="A41" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="B41" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C41" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D41" s="10" t="s">
-        <v>75</v>
-      </c>
+      <c r="B41" s="23"/>
+      <c r="C41" s="23"/>
+      <c r="D41" s="23"/>
       <c r="E41" s="6"/>
       <c r="F41" s="6"/>
     </row>
     <row r="42">
-      <c r="A42" s="25" t="s">
+      <c r="A42" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="B42" s="23"/>
-      <c r="C42" s="23"/>
-      <c r="D42" s="23"/>
-      <c r="E42" s="24"/>
-      <c r="F42" s="24"/>
+      <c r="B42" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
     </row>
     <row r="43">
-      <c r="A43" s="14"/>
-      <c r="B43" s="26"/>
-      <c r="C43" s="26"/>
-      <c r="D43" s="26"/>
-      <c r="E43" s="20"/>
-      <c r="F43" s="20"/>
+      <c r="A43" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="B43" s="23"/>
+      <c r="C43" s="23"/>
+      <c r="D43" s="23"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B44" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C44" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="D44" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E44" s="24"/>
-      <c r="F44" s="24"/>
+      <c r="A44" s="14"/>
+      <c r="B44" s="26"/>
+      <c r="C44" s="26"/>
+      <c r="D44" s="26"/>
+      <c r="E44" s="20"/>
+      <c r="F44" s="20"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="B45" s="13" t="s">
-        <v>26</v>
+      <c r="B45" s="27" t="s">
+        <v>15</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>73</v>
+        <v>30</v>
       </c>
       <c r="D45" s="27" t="s">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="E45" s="24"/>
       <c r="F45" s="24"/>
@@ -2026,17 +2026,17 @@
       <c r="A46" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B46" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="C46" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="D46" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="E46" s="6"/>
-      <c r="F46" s="6"/>
+      <c r="B46" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C46" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="D46" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="E46" s="24"/>
+      <c r="F46" s="24"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="s">
@@ -2045,99 +2045,93 @@
       <c r="B47" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C47" s="13" t="s">
+      <c r="C47" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="D47" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E47" s="6"/>
-      <c r="F47" s="6"/>
+      <c r="D47" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="E47" s="24"/>
+      <c r="F47" s="24"/>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B48" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C48" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>13</v>
-      </c>
+      <c r="B48" s="23"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="23"/>
       <c r="E48" s="6"/>
       <c r="F48" s="6"/>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="s">
+      <c r="A49" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B49" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="C49" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="D49" s="19" t="s">
-        <v>56</v>
+      <c r="B49" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C49" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D49" s="13" t="s">
+        <v>40</v>
       </c>
       <c r="E49" s="6"/>
       <c r="F49" s="6"/>
     </row>
     <row r="50">
-      <c r="A50" s="14"/>
-      <c r="B50" s="15"/>
-      <c r="C50" s="15"/>
-      <c r="D50" s="15"/>
-      <c r="E50" s="20"/>
-      <c r="F50" s="20"/>
+      <c r="A50" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E50" s="6"/>
+      <c r="F50" s="6"/>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="B51" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C51" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="D51" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E51" s="24"/>
-      <c r="F51" s="24"/>
+      <c r="A51" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="B51" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C51" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="D51" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="E51" s="6"/>
+      <c r="F51" s="6"/>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B52" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C52" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D52" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="E52" s="24"/>
-      <c r="F52" s="24"/>
+      <c r="A52" s="14"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="15"/>
+      <c r="D52" s="15"/>
+      <c r="E52" s="20"/>
+      <c r="F52" s="20"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B53" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D53" s="5" t="s">
-        <v>63</v>
+      <c r="B53" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C53" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="D53" s="21" t="s">
+        <v>51</v>
       </c>
       <c r="E53" s="24"/>
       <c r="F53" s="24"/>
@@ -2146,97 +2140,103 @@
       <c r="A54" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B54" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="C54" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="D54" s="19" t="s">
-        <v>38</v>
+      <c r="B54" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C54" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D54" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="E54" s="24"/>
       <c r="F54" s="24"/>
     </row>
     <row r="55">
-      <c r="A55" s="11" t="s">
+      <c r="A55" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B55" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>24</v>
+      <c r="B55" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>63</v>
       </c>
       <c r="E55" s="24"/>
       <c r="F55" s="24"/>
     </row>
     <row r="56">
-      <c r="A56" s="11" t="s">
+      <c r="A56" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B56" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C56" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D56" s="13" t="s">
-        <v>40</v>
+      <c r="B56" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C56" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D56" s="19" t="s">
+        <v>38</v>
       </c>
       <c r="E56" s="24"/>
       <c r="F56" s="24"/>
     </row>
     <row r="57">
-      <c r="A57" s="14"/>
-      <c r="B57" s="26"/>
-      <c r="C57" s="26"/>
-      <c r="D57" s="26"/>
-      <c r="E57" s="29"/>
-      <c r="F57" s="29"/>
+      <c r="A57" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E57" s="24"/>
+      <c r="F57" s="24"/>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B58" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="C58" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="D58" s="19" t="s">
-        <v>38</v>
+      <c r="A58" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B58" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C58" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D58" s="13" t="s">
+        <v>40</v>
       </c>
       <c r="E58" s="24"/>
       <c r="F58" s="24"/>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="B59" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C59" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="D59" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="E59" s="24"/>
-      <c r="F59" s="24"/>
+      <c r="A59" s="14"/>
+      <c r="B59" s="26"/>
+      <c r="C59" s="26"/>
+      <c r="D59" s="26"/>
+      <c r="E59" s="29"/>
+      <c r="F59" s="29"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B60" s="23"/>
-      <c r="C60" s="23"/>
-      <c r="D60" s="23"/>
+      <c r="B60" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C60" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="D60" s="19" t="s">
+        <v>38</v>
+      </c>
       <c r="E60" s="24"/>
       <c r="F60" s="24"/>
     </row>
@@ -2244,66 +2244,68 @@
       <c r="A61" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B61" s="30"/>
-      <c r="C61" s="30"/>
-      <c r="D61" s="30"/>
+      <c r="B61" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C61" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D61" s="21" t="s">
+        <v>78</v>
+      </c>
       <c r="E61" s="24"/>
       <c r="F61" s="24"/>
     </row>
     <row r="62">
-      <c r="A62" s="11" t="s">
+      <c r="A62" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B62" s="9"/>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
+      <c r="B62" s="23"/>
+      <c r="C62" s="23"/>
+      <c r="D62" s="23"/>
       <c r="E62" s="24"/>
       <c r="F62" s="24"/>
     </row>
     <row r="63">
-      <c r="A63" s="11" t="s">
+      <c r="A63" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B63" s="9"/>
-      <c r="C63" s="9"/>
-      <c r="D63" s="9"/>
+      <c r="B63" s="30"/>
+      <c r="C63" s="30"/>
+      <c r="D63" s="30"/>
       <c r="E63" s="24"/>
       <c r="F63" s="24"/>
     </row>
-    <row r="64"/>
-    <row r="65"/>
+    <row r="64">
+      <c r="A64" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="B64" s="9"/>
+      <c r="C64" s="9"/>
+      <c r="D64" s="9"/>
+      <c r="E64" s="24"/>
+      <c r="F64" s="24"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="B65" s="9"/>
+      <c r="C65" s="9"/>
+      <c r="D65" s="9"/>
+      <c r="E65" s="24"/>
+      <c r="F65" s="24"/>
+    </row>
     <row r="66"/>
     <row r="67"/>
-    <row r="68">
-      <c r="A68" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B68" s="31" t="s">
-        <v>101</v>
-      </c>
-      <c r="C68" s="32"/>
-      <c r="D68" s="32"/>
-      <c r="E68" s="33"/>
-      <c r="F68" s="33"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="B69" s="31" t="s">
-        <v>101</v>
-      </c>
-      <c r="C69" s="32"/>
-      <c r="D69" s="32"/>
-      <c r="E69" s="33"/>
-      <c r="F69" s="33"/>
-    </row>
+    <row r="68"/>
+    <row r="69"/>
     <row r="70">
       <c r="A70" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B70" s="31" t="s">
         <v>103</v>
-      </c>
-      <c r="B70" s="31" t="s">
-        <v>101</v>
       </c>
       <c r="C70" s="32"/>
       <c r="D70" s="32"/>
@@ -2315,53 +2317,53 @@
         <v>104</v>
       </c>
       <c r="B71" s="31" t="s">
-        <v>101</v>
-      </c>
-      <c r="C71" s="34"/>
-      <c r="D71" s="34"/>
+        <v>103</v>
+      </c>
+      <c r="C71" s="32"/>
+      <c r="D71" s="32"/>
       <c r="E71" s="33"/>
       <c r="F71" s="33"/>
     </row>
     <row r="72">
-      <c r="B72" s="35"/>
-      <c r="C72" s="15"/>
-      <c r="D72" s="15"/>
-      <c r="E72" s="29"/>
-      <c r="F72" s="29"/>
+      <c r="A72" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B72" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="C72" s="32"/>
+      <c r="D72" s="32"/>
+      <c r="E72" s="33"/>
+      <c r="F72" s="33"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B73" s="31" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C73" s="34"/>
       <c r="D73" s="34"/>
-      <c r="E73" s="36"/>
-      <c r="F73" s="36"/>
+      <c r="E73" s="33"/>
+      <c r="F73" s="33"/>
     </row>
     <row r="74">
-      <c r="A74" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B74" s="31" t="s">
-        <v>101</v>
-      </c>
-      <c r="C74" s="32"/>
-      <c r="D74" s="32"/>
-      <c r="E74" s="36"/>
-      <c r="F74" s="36"/>
+      <c r="B74" s="35"/>
+      <c r="C74" s="15"/>
+      <c r="D74" s="15"/>
+      <c r="E74" s="29"/>
+      <c r="F74" s="29"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="s">
         <v>107</v>
       </c>
       <c r="B75" s="31" t="s">
-        <v>101</v>
-      </c>
-      <c r="C75" s="32"/>
-      <c r="D75" s="32"/>
+        <v>103</v>
+      </c>
+      <c r="C75" s="34"/>
+      <c r="D75" s="34"/>
       <c r="E75" s="36"/>
       <c r="F75" s="36"/>
     </row>
@@ -2370,7 +2372,7 @@
         <v>108</v>
       </c>
       <c r="B76" s="31" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C76" s="32"/>
       <c r="D76" s="32"/>
@@ -2378,46 +2380,50 @@
       <c r="F76" s="36"/>
     </row>
     <row r="77">
-      <c r="B77" s="26"/>
-      <c r="C77" s="37"/>
-      <c r="D77" s="37"/>
-      <c r="E77" s="29"/>
-      <c r="F77" s="29"/>
+      <c r="A77" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B77" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="C77" s="32"/>
+      <c r="D77" s="32"/>
+      <c r="E77" s="36"/>
+      <c r="F77" s="36"/>
     </row>
     <row r="78">
-      <c r="A78" s="4"/>
-      <c r="B78" s="38" t="s">
-        <v>109</v>
+      <c r="A78" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B78" s="31" t="s">
+        <v>103</v>
       </c>
       <c r="C78" s="32"/>
       <c r="D78" s="32"/>
-      <c r="E78" s="39"/>
-      <c r="F78" s="39"/>
+      <c r="E78" s="36"/>
+      <c r="F78" s="36"/>
     </row>
     <row r="79">
-      <c r="A79" s="4"/>
-      <c r="B79" s="38" t="s">
-        <v>109</v>
-      </c>
-      <c r="C79" s="32"/>
-      <c r="D79" s="32"/>
-      <c r="E79" s="39"/>
-      <c r="F79" s="39"/>
+      <c r="B79" s="26"/>
+      <c r="C79" s="37"/>
+      <c r="D79" s="37"/>
+      <c r="E79" s="29"/>
+      <c r="F79" s="29"/>
     </row>
     <row r="80">
       <c r="A80" s="4"/>
       <c r="B80" s="38" t="s">
-        <v>109</v>
-      </c>
-      <c r="C80" s="34"/>
-      <c r="D80" s="34"/>
+        <v>111</v>
+      </c>
+      <c r="C80" s="32"/>
+      <c r="D80" s="32"/>
       <c r="E80" s="39"/>
       <c r="F80" s="39"/>
     </row>
     <row r="81">
       <c r="A81" s="4"/>
       <c r="B81" s="38" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C81" s="32"/>
       <c r="D81" s="32"/>
@@ -2425,16 +2431,19 @@
       <c r="F81" s="39"/>
     </row>
     <row r="82">
-      <c r="B82" s="26"/>
-      <c r="C82" s="37"/>
-      <c r="D82" s="37"/>
-      <c r="E82" s="29"/>
-      <c r="F82" s="29"/>
+      <c r="A82" s="4"/>
+      <c r="B82" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="C82" s="34"/>
+      <c r="D82" s="34"/>
+      <c r="E82" s="39"/>
+      <c r="F82" s="39"/>
     </row>
     <row r="83">
       <c r="A83" s="4"/>
       <c r="B83" s="38" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C83" s="32"/>
       <c r="D83" s="32"/>
@@ -2442,55 +2451,58 @@
       <c r="F83" s="39"/>
     </row>
     <row r="84">
-      <c r="A84" s="4"/>
-      <c r="B84" s="38" t="s">
-        <v>110</v>
-      </c>
-      <c r="C84" s="32"/>
-      <c r="D84" s="32"/>
-      <c r="E84" s="39"/>
-      <c r="F84" s="39"/>
+      <c r="B84" s="26"/>
+      <c r="C84" s="37"/>
+      <c r="D84" s="37"/>
+      <c r="E84" s="29"/>
+      <c r="F84" s="29"/>
     </row>
     <row r="85">
-      <c r="B85" s="26"/>
-      <c r="C85" s="37"/>
-      <c r="D85" s="37"/>
-      <c r="E85" s="29"/>
-      <c r="F85" s="29"/>
+      <c r="A85" s="4"/>
+      <c r="B85" s="38" t="s">
+        <v>112</v>
+      </c>
+      <c r="C85" s="32"/>
+      <c r="D85" s="32"/>
+      <c r="E85" s="39"/>
+      <c r="F85" s="39"/>
     </row>
     <row r="86">
       <c r="A86" s="4"/>
-      <c r="B86" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="C86" s="40"/>
-      <c r="D86" s="40"/>
-      <c r="E86" s="4"/>
-      <c r="F86" s="4"/>
+      <c r="B86" s="38" t="s">
+        <v>112</v>
+      </c>
+      <c r="C86" s="32"/>
+      <c r="D86" s="32"/>
+      <c r="E86" s="39"/>
+      <c r="F86" s="39"/>
     </row>
     <row r="87">
-      <c r="A87" s="4"/>
-      <c r="B87" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C87" s="40"/>
-      <c r="D87" s="40"/>
-      <c r="E87" s="4"/>
-      <c r="F87" s="4"/>
+      <c r="B87" s="26"/>
+      <c r="C87" s="37"/>
+      <c r="D87" s="37"/>
+      <c r="E87" s="29"/>
+      <c r="F87" s="29"/>
     </row>
     <row r="88">
-      <c r="B88" s="26"/>
-      <c r="C88" s="26"/>
-      <c r="D88" s="26"/>
-      <c r="E88" s="29"/>
-      <c r="F88" s="29"/>
+      <c r="A88" s="4"/>
+      <c r="B88" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C88" s="40"/>
+      <c r="D88" s="40"/>
+      <c r="E88" s="4"/>
+      <c r="F88" s="4"/>
     </row>
     <row r="89">
-      <c r="B89" s="26"/>
-      <c r="C89" s="26"/>
-      <c r="D89" s="26"/>
-      <c r="E89" s="29"/>
-      <c r="F89" s="29"/>
+      <c r="A89" s="4"/>
+      <c r="B89" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C89" s="40"/>
+      <c r="D89" s="40"/>
+      <c r="E89" s="4"/>
+      <c r="F89" s="4"/>
     </row>
     <row r="90">
       <c r="B90" s="26"/>
@@ -8826,6 +8838,20 @@
       <c r="D994" s="26"/>
       <c r="E994" s="29"/>
       <c r="F994" s="29"/>
+    </row>
+    <row r="995">
+      <c r="B995" s="26"/>
+      <c r="C995" s="26"/>
+      <c r="D995" s="26"/>
+      <c r="E995" s="29"/>
+      <c r="F995" s="29"/>
+    </row>
+    <row r="996">
+      <c r="B996" s="26"/>
+      <c r="C996" s="26"/>
+      <c r="D996" s="26"/>
+      <c r="E996" s="29"/>
+      <c r="F996" s="29"/>
     </row>
   </sheetData>
   <printOptions/>
@@ -8850,28 +8876,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="41" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B1" s="42" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C1" s="43" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D1" s="44" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E1" s="45" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F1" s="46" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G1" s="47" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H1" s="48" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2">
@@ -8934,7 +8960,7 @@
         <v>28</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D4" s="50" t="s">
         <v>17</v>
@@ -8954,7 +8980,7 @@
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B5" s="49" t="s">
         <v>40</v>
@@ -9034,10 +9060,10 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B2" s="57" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C2" s="57" t="s">
         <v>21</v>
@@ -9054,16 +9080,16 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B3" s="59" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C3" s="59" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D3" s="59" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E3" s="58">
         <v>9.0</v>
@@ -9074,13 +9100,13 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B4" s="60" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C4" s="60" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D4" s="60" t="s">
         <v>40</v>
@@ -9094,16 +9120,16 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B5" s="61" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C5" s="61" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D5" s="61" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E5" s="58">
         <v>11.0</v>
@@ -9114,16 +9140,16 @@
     </row>
     <row r="6">
       <c r="A6" s="11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B6" s="62" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C6" s="62" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D6" s="62" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E6" s="58">
         <v>4.0</v>
@@ -9135,16 +9161,16 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B7" s="61" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C7" s="61" t="s">
         <v>47</v>
       </c>
       <c r="D7" s="61" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E7" s="58">
         <v>11.0</v>
@@ -9160,16 +9186,16 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B9" s="61" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C9" s="61" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D9" s="61" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E9" s="58">
         <v>6.0</v>
@@ -9180,13 +9206,13 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B10" s="57" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C10" s="57" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D10" s="57" t="s">
         <v>21</v>
@@ -9201,16 +9227,16 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B11" s="59" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C11" s="59" t="s">
         <v>37</v>
       </c>
       <c r="D11" s="59" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E11" s="58">
         <v>10.0</v>
@@ -9221,13 +9247,13 @@
     </row>
     <row r="12">
       <c r="A12" s="11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B12" s="57" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C12" s="57" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D12" s="57" t="s">
         <v>21</v>
@@ -9241,16 +9267,16 @@
     </row>
     <row r="13">
       <c r="A13" s="64" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B13" s="62" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C13" s="62" t="s">
         <v>63</v>
       </c>
       <c r="D13" s="62" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E13" s="58">
         <v>6.0</v>
@@ -9261,10 +9287,10 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B14" s="65" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C14" s="65" t="s">
         <v>30</v>
@@ -9288,16 +9314,16 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B16" s="65" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C16" s="65" t="s">
         <v>30</v>
       </c>
       <c r="D16" s="65" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E16" s="58">
         <v>8.0</v>
@@ -9308,16 +9334,16 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B17" s="61" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C17" s="61" t="s">
         <v>47</v>
       </c>
       <c r="D17" s="61" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E17" s="58">
         <v>7.0</v>
@@ -9328,16 +9354,16 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B18" s="60" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C18" s="60" t="s">
         <v>40</v>
       </c>
       <c r="D18" s="60" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E18" s="58">
         <v>7.0</v>
@@ -9348,16 +9374,16 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B19" s="61" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C19" s="61" t="s">
         <v>47</v>
       </c>
       <c r="D19" s="61" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E19" s="58">
         <v>9.0</v>
@@ -9368,16 +9394,16 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B20" s="60" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C20" s="60" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D20" s="60" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E20" s="58">
         <v>6.0</v>
@@ -9388,16 +9414,16 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B21" s="60" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C21" s="60" t="s">
+        <v>162</v>
+      </c>
+      <c r="D21" s="60" t="s">
         <v>160</v>
-      </c>
-      <c r="D21" s="60" t="s">
-        <v>158</v>
       </c>
       <c r="E21" s="58">
         <v>7.0</v>
@@ -9413,32 +9439,32 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B23" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C23" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D23" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E23" s="33"/>
       <c r="F23" s="33"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B24" s="59" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C24" s="59" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D24" s="59" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E24" s="58">
         <v>5.0</v>
@@ -9449,13 +9475,13 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B25" s="57" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C25" s="57" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D25" s="57" t="s">
         <v>59</v>
@@ -9469,16 +9495,16 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B26" s="60" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C26" s="60" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D26" s="60" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E26" s="58">
         <v>8.0</v>
@@ -9489,16 +9515,16 @@
     </row>
     <row r="27">
       <c r="A27" s="64" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B27" s="62" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C27" s="62" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D27" s="62" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E27" s="58">
         <v>8.0</v>
@@ -9509,16 +9535,16 @@
     </row>
     <row r="28">
       <c r="A28" s="64" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B28" s="62" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C28" s="62" t="s">
         <v>63</v>
       </c>
       <c r="D28" s="62" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E28" s="58">
         <v>9.0</v>
@@ -9534,13 +9560,13 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B30" s="59" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C30" s="59" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D30" s="59" t="s">
         <v>37</v>
@@ -9554,16 +9580,16 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B31" s="61" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C31" s="61" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D31" s="61" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E31" s="58">
         <v>5.0</v>
@@ -9574,16 +9600,16 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B32" s="60" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C32" s="60" t="s">
         <v>40</v>
       </c>
       <c r="D32" s="60" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E32" s="58">
         <v>5.0</v>
@@ -9594,10 +9620,10 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B33" s="65" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C33" s="65" t="s">
         <v>30</v>
@@ -9614,16 +9640,16 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B34" s="61" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C34" s="61" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D34" s="61" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E34" s="58">
         <v>9.0</v>
@@ -9634,16 +9660,16 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B35" s="65" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C35" s="65" t="s">
         <v>27</v>
       </c>
       <c r="D35" s="65" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E35" s="58">
         <v>2.0</v>
@@ -9659,32 +9685,32 @@
     </row>
     <row r="37">
       <c r="A37" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B37" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C37" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D37" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E37" s="33"/>
       <c r="F37" s="33"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B38" s="62" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C38" s="62" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D38" s="62" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E38" s="58">
         <v>8.0</v>
@@ -9695,13 +9721,13 @@
     </row>
     <row r="39">
       <c r="A39" s="64" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B39" s="65" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C39" s="65" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D39" s="65" t="s">
         <v>51</v>
@@ -9715,16 +9741,16 @@
     </row>
     <row r="40">
       <c r="A40" s="4" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B40" s="57" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C40" s="57" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D40" s="57" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E40" s="58">
         <v>1.0</v>
@@ -9735,13 +9761,13 @@
     </row>
     <row r="41">
       <c r="A41" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B41" s="59" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C41" s="59" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D41" s="59" t="s">
         <v>37</v>
@@ -9755,16 +9781,16 @@
     </row>
     <row r="42">
       <c r="A42" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B42" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C42" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D42" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E42" s="33"/>
       <c r="F42" s="33"/>
@@ -9776,48 +9802,48 @@
     </row>
     <row r="44">
       <c r="A44" s="4" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B44" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C44" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D44" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E44" s="33"/>
       <c r="F44" s="33"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B45" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C45" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D45" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E45" s="33"/>
       <c r="F45" s="33"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B46" s="62" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C46" s="62" t="s">
         <v>63</v>
       </c>
       <c r="D46" s="62" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E46" s="58">
         <v>7.0</v>
@@ -9828,16 +9854,16 @@
     </row>
     <row r="47">
       <c r="A47" s="4" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B47" s="60" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C47" s="60" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D47" s="60" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E47" s="58">
         <v>4.0</v>
@@ -9848,10 +9874,10 @@
     </row>
     <row r="48">
       <c r="A48" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B48" s="65" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C48" s="65" t="s">
         <v>51</v>
@@ -9868,16 +9894,16 @@
     </row>
     <row r="49">
       <c r="A49" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B49" s="61" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C49" s="61" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D49" s="61" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E49" s="58">
         <v>6.0</v>
@@ -9893,61 +9919,61 @@
     </row>
     <row r="51">
       <c r="A51" s="4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B51" s="60" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C51" s="60" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D51" s="60" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E51" s="33"/>
       <c r="F51" s="33"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B52" s="59" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C52" s="59" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D52" s="59" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E52" s="33"/>
       <c r="F52" s="33"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B53" s="60" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C53" s="60" t="s">
         <v>40</v>
       </c>
       <c r="D53" s="60" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E53" s="33"/>
       <c r="F53" s="33"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B54" s="61" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C54" s="61" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D54" s="61" t="s">
         <v>47</v>
@@ -9957,32 +9983,32 @@
     </row>
     <row r="55">
       <c r="A55" s="11" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B55" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C55" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D55" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E55" s="33"/>
       <c r="F55" s="33"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B56" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C56" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D56" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E56" s="33"/>
       <c r="F56" s="33"/>
@@ -9994,29 +10020,29 @@
     </row>
     <row r="58">
       <c r="A58" s="4" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B58" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C58" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D58" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E58" s="33"/>
       <c r="F58" s="33"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B59" s="57" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C59" s="57" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D59" s="57" t="s">
         <v>59</v>
@@ -10026,64 +10052,64 @@
     </row>
     <row r="60">
       <c r="A60" s="4" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B60" s="61" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C60" s="61" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D60" s="61" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E60" s="33"/>
       <c r="F60" s="33"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B61" s="60" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C61" s="60" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D61" s="60" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E61" s="33"/>
       <c r="F61" s="33"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B62" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C62" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D62" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E62" s="33"/>
       <c r="F62" s="33"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B63" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C63" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D63" s="66" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E63" s="33"/>
       <c r="F63" s="33"/>
@@ -10094,10 +10120,10 @@
     </row>
     <row r="65">
       <c r="A65" s="4" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B65" s="31" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C65" s="61" t="s">
         <v>21</v>
@@ -10110,13 +10136,13 @@
     </row>
     <row r="66">
       <c r="A66" s="4" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B66" s="31" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C66" s="60" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D66" s="60" t="s">
         <v>59</v>
@@ -10126,13 +10152,13 @@
     </row>
     <row r="67">
       <c r="A67" s="4" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B67" s="31" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C67" s="60" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D67" s="60" t="s">
         <v>63</v>
@@ -10142,16 +10168,16 @@
     </row>
     <row r="68">
       <c r="A68" s="4" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B68" s="31" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C68" s="59" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D68" s="59" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E68" s="33"/>
       <c r="F68" s="33"/>
@@ -10165,13 +10191,13 @@
     </row>
     <row r="70">
       <c r="A70" s="4" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B70" s="31" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C70" s="59" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D70" s="59" t="s">
         <v>51</v>
@@ -10181,13 +10207,13 @@
     </row>
     <row r="71">
       <c r="A71" s="4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B71" s="31" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C71" s="65" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D71" s="65" t="s">
         <v>53</v>
@@ -10197,13 +10223,13 @@
     </row>
     <row r="72">
       <c r="A72" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B72" s="31" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C72" s="65" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D72" s="65" t="s">
         <v>30</v>
@@ -10213,16 +10239,16 @@
     </row>
     <row r="73">
       <c r="A73" s="4" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B73" s="31" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C73" s="61" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D73" s="61" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E73" s="36"/>
       <c r="F73" s="36"/>
@@ -10234,10 +10260,10 @@
     </row>
     <row r="75">
       <c r="A75" s="4" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B75" s="38" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C75" s="61"/>
       <c r="D75" s="61"/>
@@ -10246,10 +10272,10 @@
     </row>
     <row r="76">
       <c r="A76" s="4" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B76" s="38" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C76" s="60"/>
       <c r="D76" s="60"/>
@@ -10258,10 +10284,10 @@
     </row>
     <row r="77">
       <c r="A77" s="4" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B77" s="38" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C77" s="59"/>
       <c r="D77" s="59"/>
@@ -10270,10 +10296,10 @@
     </row>
     <row r="78">
       <c r="A78" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B78" s="38" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C78" s="65"/>
       <c r="D78" s="65"/>
@@ -10286,10 +10312,10 @@
     </row>
     <row r="80">
       <c r="A80" s="4" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B80" s="38" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C80" s="60"/>
       <c r="D80" s="68"/>
@@ -10298,10 +10324,10 @@
     </row>
     <row r="81">
       <c r="A81" s="4" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B81" s="38" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C81" s="65"/>
       <c r="D81" s="61"/>
@@ -10314,10 +10340,10 @@
     </row>
     <row r="83">
       <c r="A83" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C83" s="4"/>
       <c r="D83" s="4"/>
@@ -10326,10 +10352,10 @@
     </row>
     <row r="84">
       <c r="A84" s="4" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C84" s="4"/>
       <c r="D84" s="4"/>
@@ -14017,42 +14043,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="69" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B1" s="42" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C1" s="43" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D1" s="44" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E1" s="45" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F1" s="46" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="61" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B2" s="60" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C2" s="57" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D2" s="70" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E2" s="65" t="s">
         <v>30</v>
       </c>
       <c r="F2" s="71" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3">
@@ -14066,27 +14092,27 @@
         <v>104.0</v>
       </c>
       <c r="D3" s="70" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E3" s="65" t="s">
         <v>51</v>
       </c>
       <c r="F3" s="71" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="61" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B4" s="60" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C4" s="57" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="70" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E4" s="65" t="s">
         <v>27</v>
@@ -14097,30 +14123,30 @@
     </row>
     <row r="5">
       <c r="A5" s="61" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B5" s="60" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C5" s="57" t="s">
         <v>59</v>
       </c>
       <c r="D5" s="70" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E5" s="65" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F5" s="71" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="61" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B6" s="60" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>

</xml_diff>

<commit_message>
Dati: Girone B/C, riprogrammazione orari 23/06 e 25/06
Rigenerato da Calend Bocce 2026 (1).xlsx via tools/build_data.py.
- mar 23/06: I Toghini vs Apostadores 23:00 -> 20:00
- gio 25/06: Apostadores vs The Doctors 21:00 -> 20:30
- gio 25/06: 0Sbat vs I Cugini 20:30 -> 21:00
Classifiche invariate. Nessuna sovrapposizione di slot (campo unico).
Cache-busting asset: v=202606211011.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -214,6 +214,12 @@
     <t>lunedì 22/06 23:00</t>
   </si>
   <si>
+    <t>martedì 23/06 20:00</t>
+  </si>
+  <si>
+    <t>Apostadores</t>
+  </si>
+  <si>
     <t>martedì 23/06 20:30</t>
   </si>
   <si>
@@ -230,12 +236,6 @@
   </si>
   <si>
     <t>I Masalén</t>
-  </si>
-  <si>
-    <t>martedì 23/06 23:00</t>
-  </si>
-  <si>
-    <t>Apostadores</t>
   </si>
   <si>
     <t>mercoledì 24/06 20:00</t>
@@ -1795,81 +1795,81 @@
       <c r="F29" s="20"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B30" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C30" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="D30" s="10" t="s">
-        <v>21</v>
+      <c r="B30" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>67</v>
       </c>
       <c r="E30" s="6"/>
       <c r="F30" s="6"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B31" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="C31" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="D31" s="17" t="s">
-        <v>44</v>
+        <v>68</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>21</v>
       </c>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>53</v>
+        <v>69</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C32" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" s="17" t="s">
+        <v>44</v>
       </c>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>12</v>
+        <v>70</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>53</v>
       </c>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="B34" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="C34" s="19" t="s">
+      <c r="A34" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D34" s="19" t="s">
-        <v>37</v>
+      <c r="B34" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>12</v>
       </c>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
@@ -1878,14 +1878,14 @@
       <c r="A35" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B35" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D35" s="13" t="s">
+      <c r="B35" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C35" s="19" t="s">
         <v>73</v>
+      </c>
+      <c r="D35" s="19" t="s">
+        <v>37</v>
       </c>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
@@ -2026,14 +2026,14 @@
       <c r="A46" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B46" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C46" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="D46" s="21" t="s">
-        <v>51</v>
+      <c r="B46" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C46" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="D46" s="28" t="s">
+        <v>28</v>
       </c>
       <c r="E46" s="24"/>
       <c r="F46" s="24"/>
@@ -2042,14 +2042,14 @@
       <c r="A47" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B47" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C47" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="D47" s="28" t="s">
-        <v>28</v>
+      <c r="B47" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C47" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="D47" s="21" t="s">
+        <v>51</v>
       </c>
       <c r="E47" s="24"/>
       <c r="F47" s="24"/>
@@ -2072,7 +2072,7 @@
         <v>26</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D49" s="13" t="s">
         <v>40</v>
@@ -2104,7 +2104,7 @@
         <v>36</v>
       </c>
       <c r="C51" s="19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D51" s="19" t="s">
         <v>56</v>
@@ -2232,7 +2232,7 @@
         <v>36</v>
       </c>
       <c r="C60" s="19" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D60" s="19" t="s">
         <v>38</v>
@@ -8920,7 +8920,7 @@
         <v>33</v>
       </c>
       <c r="G2" s="53" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H2" s="54" t="s">
         <v>23</v>
@@ -8931,7 +8931,7 @@
         <v>42</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C3" s="21" t="s">
         <v>50</v>

</xml_diff>

<commit_message>
Dati: Girone A, compattata serata 24/06 (chiuso buco 22:00)
Rigenerato da Calend Bocce 2026 (1).xlsx via tools/build_data.py.
- mer 24/06: Gli Allenati vs Wood&Beton 22:30 -> 22:00
Serata 24/06 ora compatta 20:00->22:00, senza buchi.
Classifiche invariate. Nessuna sovrapposizione di slot (campo unico).
Cache-busting asset: v=202606211026.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -1963,28 +1963,28 @@
       <c r="F40" s="6"/>
     </row>
     <row r="41">
-      <c r="A41" s="22" t="s">
+      <c r="A41" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B41" s="23"/>
-      <c r="C41" s="23"/>
-      <c r="D41" s="23"/>
+      <c r="B41" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>76</v>
+      </c>
       <c r="E41" s="6"/>
       <c r="F41" s="6"/>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="s">
+      <c r="A42" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="B42" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C42" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D42" s="10" t="s">
-        <v>76</v>
-      </c>
+      <c r="B42" s="23"/>
+      <c r="C42" s="23"/>
+      <c r="D42" s="23"/>
       <c r="E42" s="6"/>
       <c r="F42" s="6"/>
     </row>

</xml_diff>

<commit_message>
Dati: 5 risultati e 2 rinvii; baseline verifica da tutti i risultati
Rigenerato da Calend Bocce 2026 (1).xlsx via tools/build_data.py.

Risultati (giocate 17 -> 22):
- C: 0Sbat 8-6 Chocolate Starfishes
- D: Mirkae 9-1 BocciAli
- E: Le Cognate 6-5 Ricci di Mare
- F: Zaccaria 7-4 A&M
- F: A&M 8-6 T alla seconda

Calendario (rinvii dal 23/06, campo unico, nessuna sovrapposizione):
- T alla seconda vs I Cavalli: 23/06 21:00 -> 30/06 21:30
- Le Cognate vs Bad Boys: 23/06 21:30 -> 25/06 21:30

Classifiche cambiate: C, D, E, F (A/B/G/H invariate).

tools/build_data.py: il baseline di verifica ora riflette le classifiche
calcolate da tutti i risultati, non piu' la lista iniziale del PDF.
Cache-busting v=202606230936.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -1703,8 +1703,12 @@
       <c r="D23" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
+      <c r="E23" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="F23" s="6">
+        <v>6.0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="s">
@@ -1719,8 +1723,12 @@
       <c r="D24" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
+      <c r="E24" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="F24" s="6">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="s">
@@ -1735,8 +1743,12 @@
       <c r="D25" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
+      <c r="E25" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="F25" s="6">
+        <v>4.0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="s">
@@ -1751,8 +1763,12 @@
       <c r="D26" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
+      <c r="E26" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="F26" s="6">
+        <v>5.0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="s">
@@ -1767,8 +1783,12 @@
       <c r="D27" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
+      <c r="E27" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="F27" s="6">
+        <v>8.0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="s">
@@ -1827,34 +1847,22 @@
       <c r="F31" s="6"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="B32" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="C32" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="D32" s="17" t="s">
-        <v>44</v>
-      </c>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>53</v>
-      </c>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
     </row>
@@ -2055,12 +2063,18 @@
       <c r="F47" s="24"/>
     </row>
     <row r="48">
-      <c r="A48" s="22" t="s">
+      <c r="A48" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B48" s="23"/>
-      <c r="C48" s="23"/>
-      <c r="D48" s="23"/>
+      <c r="B48" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="E48" s="6"/>
       <c r="F48" s="6"/>
     </row>
@@ -2260,9 +2274,15 @@
       <c r="A62" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B62" s="23"/>
-      <c r="C62" s="23"/>
-      <c r="D62" s="23"/>
+      <c r="B62" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C62" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D62" s="17" t="s">
+        <v>44</v>
+      </c>
       <c r="E62" s="24"/>
       <c r="F62" s="24"/>
     </row>

</xml_diff>

<commit_message>
Dati: 10 risultati e 4 rinvii; baseline classifiche aggiornato
Rigenerato da Calend Bocce 2026 (1).xlsx via tools/build_data.py.

Risultati (giocate 22 -> 32):
- A: Gli Zebis 2-11 Gli Allenati; Gli Zebis 9-1 Wood&Beton; Gli Allenati 10-2 Wood&Beton
- B: I Toghini 9-3 Apostadores
- C: 0Sbat 6-3 La Coppia
- D: Il Boccino 6-5 Tironi; Mirkae 8-1 Tironi
- F: Zaccaria 4-7 I Cavalli
- G: I Masalen 5-9 I Diavoli
- H: Atletico Cavalclown 2.0 7-6 Ghirarda

Calendario (consolidamento mar 30/06):
- I Masalen vs Bocce da Urlo 20:30 -> 21:00
- Chocolate Starfishes vs La Coppia 21:00 -> 21:30
- T alla seconda vs I Cavalli 21:30 -> 22:00
- I Masalen vs Gli Hummarell: gio 25/06 23:00 -> mar 30/06 22:30

Ordine cambiato: A, B, C, D, H -> baseline 'expected' aggiornato in build_data.py.
Nessuna sovrapposizione di slot (campo unico). Cache-busting v=202606251048.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -855,7 +855,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="71">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -922,12 +922,12 @@
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="7" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -935,9 +935,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -1827,8 +1824,12 @@
       <c r="D30" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
+      <c r="E30" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="F30" s="6">
+        <v>3.0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="s">
@@ -1843,8 +1844,12 @@
       <c r="D31" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
+      <c r="E31" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="F31" s="6">
+        <v>11.0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="22" t="s">
@@ -1879,8 +1884,12 @@
       <c r="D34" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
+      <c r="E34" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="F34" s="6">
+        <v>6.0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="s">
@@ -1895,8 +1904,12 @@
       <c r="D35" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
+      <c r="E35" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="F35" s="6">
+        <v>9.0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="14"/>
@@ -1919,8 +1932,12 @@
       <c r="D37" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E37" s="24"/>
-      <c r="F37" s="24"/>
+      <c r="E37" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="F37" s="6">
+        <v>5.0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="s">
@@ -1935,8 +1952,12 @@
       <c r="D38" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="E38" s="24"/>
-      <c r="F38" s="24"/>
+      <c r="E38" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="F38" s="6">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="s">
@@ -1951,8 +1972,12 @@
       <c r="D39" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="E39" s="6"/>
-      <c r="F39" s="6"/>
+      <c r="E39" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="F39" s="6">
+        <v>3.0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="11" t="s">
@@ -1967,8 +1992,12 @@
       <c r="D40" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="E40" s="6"/>
-      <c r="F40" s="6"/>
+      <c r="E40" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="F40" s="6">
+        <v>7.0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="s">
@@ -1983,34 +2012,42 @@
       <c r="D41" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="E41" s="6"/>
-      <c r="F41" s="6"/>
+      <c r="E41" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="F41" s="6">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="B42" s="25" t="s">
+      <c r="B42" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="C42" s="25" t="s">
+      <c r="C42" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="D42" s="25" t="s">
+      <c r="D42" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
+      <c r="E42" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="F42" s="6">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="26" t="s">
+      <c r="A43" s="25" t="s">
         <v>82</v>
       </c>
       <c r="B43" s="23"/>
       <c r="C43" s="23"/>
       <c r="D43" s="23"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="24"/>
+      <c r="E43" s="26"/>
+      <c r="F43" s="26"/>
     </row>
     <row r="44">
       <c r="A44" s="14"/>
@@ -2027,8 +2064,8 @@
       <c r="B45" s="23"/>
       <c r="C45" s="23"/>
       <c r="D45" s="23"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="24"/>
+      <c r="E45" s="26"/>
+      <c r="F45" s="26"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="s">
@@ -2043,8 +2080,8 @@
       <c r="D46" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="E46" s="24"/>
-      <c r="F46" s="24"/>
+      <c r="E46" s="26"/>
+      <c r="F46" s="26"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="s">
@@ -2059,8 +2096,8 @@
       <c r="D47" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="E47" s="24"/>
-      <c r="F47" s="24"/>
+      <c r="E47" s="26"/>
+      <c r="F47" s="26"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="s">
@@ -2111,18 +2148,12 @@
       <c r="F50" s="6"/>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="s">
+      <c r="A51" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="B51" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="C51" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="D51" s="19" t="s">
-        <v>56</v>
-      </c>
+      <c r="B51" s="23"/>
+      <c r="C51" s="23"/>
+      <c r="D51" s="23"/>
       <c r="E51" s="6"/>
       <c r="F51" s="6"/>
     </row>
@@ -2147,8 +2178,8 @@
       <c r="D53" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="E53" s="24"/>
-      <c r="F53" s="24"/>
+      <c r="E53" s="26"/>
+      <c r="F53" s="26"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="s">
@@ -2163,8 +2194,8 @@
       <c r="D54" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="E54" s="24"/>
-      <c r="F54" s="24"/>
+      <c r="E54" s="26"/>
+      <c r="F54" s="26"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="s">
@@ -2179,8 +2210,8 @@
       <c r="D55" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E55" s="24"/>
-      <c r="F55" s="24"/>
+      <c r="E55" s="26"/>
+      <c r="F55" s="26"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="s">
@@ -2195,8 +2226,8 @@
       <c r="D56" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="E56" s="24"/>
-      <c r="F56" s="24"/>
+      <c r="E56" s="26"/>
+      <c r="F56" s="26"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="s">
@@ -2211,8 +2242,8 @@
       <c r="D57" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E57" s="24"/>
-      <c r="F57" s="24"/>
+      <c r="E57" s="26"/>
+      <c r="F57" s="26"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="s">
@@ -2227,8 +2258,8 @@
       <c r="D58" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E58" s="24"/>
-      <c r="F58" s="24"/>
+      <c r="E58" s="26"/>
+      <c r="F58" s="26"/>
     </row>
     <row r="59">
       <c r="A59" s="14"/>
@@ -2239,82 +2270,88 @@
       <c r="F59" s="29"/>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="s">
+      <c r="A60" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="B60" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="C60" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="D60" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="E60" s="24"/>
-      <c r="F60" s="24"/>
+      <c r="B60" s="23"/>
+      <c r="C60" s="23"/>
+      <c r="D60" s="23"/>
+      <c r="E60" s="26"/>
+      <c r="F60" s="26"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B61" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C61" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="D61" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="E61" s="24"/>
-      <c r="F61" s="24"/>
+      <c r="B61" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C61" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D61" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="E61" s="26"/>
+      <c r="F61" s="26"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B62" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="C62" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="D62" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="E62" s="24"/>
-      <c r="F62" s="24"/>
+      <c r="B62" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C62" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D62" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="E62" s="26"/>
+      <c r="F62" s="26"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B63" s="30"/>
-      <c r="C63" s="30"/>
-      <c r="D63" s="30"/>
-      <c r="E63" s="24"/>
-      <c r="F63" s="24"/>
+      <c r="B63" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C63" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D63" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E63" s="26"/>
+      <c r="F63" s="26"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="B64" s="9"/>
-      <c r="C64" s="9"/>
-      <c r="D64" s="9"/>
-      <c r="E64" s="24"/>
-      <c r="F64" s="24"/>
+      <c r="B64" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C64" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D64" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="E64" s="26"/>
+      <c r="F64" s="26"/>
     </row>
     <row r="65">
-      <c r="A65" s="11" t="s">
+      <c r="A65" s="25" t="s">
         <v>101</v>
       </c>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
       <c r="D65" s="9"/>
-      <c r="E65" s="24"/>
-      <c r="F65" s="24"/>
+      <c r="E65" s="26"/>
+      <c r="F65" s="26"/>
     </row>
     <row r="66"/>
     <row r="67"/>
@@ -2324,52 +2361,52 @@
       <c r="A70" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B70" s="31" t="s">
+      <c r="B70" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C70" s="32"/>
-      <c r="D70" s="32"/>
-      <c r="E70" s="33"/>
-      <c r="F70" s="33"/>
+      <c r="C70" s="31"/>
+      <c r="D70" s="31"/>
+      <c r="E70" s="32"/>
+      <c r="F70" s="32"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B71" s="31" t="s">
+      <c r="B71" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C71" s="32"/>
-      <c r="D71" s="32"/>
-      <c r="E71" s="33"/>
-      <c r="F71" s="33"/>
+      <c r="C71" s="31"/>
+      <c r="D71" s="31"/>
+      <c r="E71" s="32"/>
+      <c r="F71" s="32"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B72" s="31" t="s">
+      <c r="B72" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C72" s="32"/>
-      <c r="D72" s="32"/>
-      <c r="E72" s="33"/>
-      <c r="F72" s="33"/>
+      <c r="C72" s="31"/>
+      <c r="D72" s="31"/>
+      <c r="E72" s="32"/>
+      <c r="F72" s="32"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B73" s="31" t="s">
+      <c r="B73" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C73" s="34"/>
-      <c r="D73" s="34"/>
-      <c r="E73" s="33"/>
-      <c r="F73" s="33"/>
+      <c r="C73" s="33"/>
+      <c r="D73" s="33"/>
+      <c r="E73" s="32"/>
+      <c r="F73" s="32"/>
     </row>
     <row r="74">
-      <c r="B74" s="35"/>
+      <c r="B74" s="34"/>
       <c r="C74" s="15"/>
       <c r="D74" s="15"/>
       <c r="E74" s="29"/>
@@ -2379,128 +2416,128 @@
       <c r="A75" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B75" s="31" t="s">
+      <c r="B75" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C75" s="34"/>
-      <c r="D75" s="34"/>
-      <c r="E75" s="36"/>
-      <c r="F75" s="36"/>
+      <c r="C75" s="33"/>
+      <c r="D75" s="33"/>
+      <c r="E75" s="35"/>
+      <c r="F75" s="35"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B76" s="31" t="s">
+      <c r="B76" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C76" s="32"/>
-      <c r="D76" s="32"/>
-      <c r="E76" s="36"/>
-      <c r="F76" s="36"/>
+      <c r="C76" s="31"/>
+      <c r="D76" s="31"/>
+      <c r="E76" s="35"/>
+      <c r="F76" s="35"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="B77" s="31" t="s">
+      <c r="B77" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C77" s="32"/>
-      <c r="D77" s="32"/>
-      <c r="E77" s="36"/>
-      <c r="F77" s="36"/>
+      <c r="C77" s="31"/>
+      <c r="D77" s="31"/>
+      <c r="E77" s="35"/>
+      <c r="F77" s="35"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B78" s="31" t="s">
+      <c r="B78" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C78" s="32"/>
-      <c r="D78" s="32"/>
-      <c r="E78" s="36"/>
-      <c r="F78" s="36"/>
+      <c r="C78" s="31"/>
+      <c r="D78" s="31"/>
+      <c r="E78" s="35"/>
+      <c r="F78" s="35"/>
     </row>
     <row r="79">
       <c r="B79" s="27"/>
-      <c r="C79" s="37"/>
-      <c r="D79" s="37"/>
+      <c r="C79" s="36"/>
+      <c r="D79" s="36"/>
       <c r="E79" s="29"/>
       <c r="F79" s="29"/>
     </row>
     <row r="80">
       <c r="A80" s="4"/>
-      <c r="B80" s="38" t="s">
+      <c r="B80" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="C80" s="32"/>
-      <c r="D80" s="32"/>
-      <c r="E80" s="39"/>
-      <c r="F80" s="39"/>
+      <c r="C80" s="31"/>
+      <c r="D80" s="31"/>
+      <c r="E80" s="38"/>
+      <c r="F80" s="38"/>
     </row>
     <row r="81">
       <c r="A81" s="4"/>
-      <c r="B81" s="38" t="s">
+      <c r="B81" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="C81" s="32"/>
-      <c r="D81" s="32"/>
-      <c r="E81" s="39"/>
-      <c r="F81" s="39"/>
+      <c r="C81" s="31"/>
+      <c r="D81" s="31"/>
+      <c r="E81" s="38"/>
+      <c r="F81" s="38"/>
     </row>
     <row r="82">
       <c r="A82" s="4"/>
-      <c r="B82" s="38" t="s">
+      <c r="B82" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="C82" s="34"/>
-      <c r="D82" s="34"/>
-      <c r="E82" s="39"/>
-      <c r="F82" s="39"/>
+      <c r="C82" s="33"/>
+      <c r="D82" s="33"/>
+      <c r="E82" s="38"/>
+      <c r="F82" s="38"/>
     </row>
     <row r="83">
       <c r="A83" s="4"/>
-      <c r="B83" s="38" t="s">
+      <c r="B83" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="C83" s="32"/>
-      <c r="D83" s="32"/>
-      <c r="E83" s="39"/>
-      <c r="F83" s="39"/>
+      <c r="C83" s="31"/>
+      <c r="D83" s="31"/>
+      <c r="E83" s="38"/>
+      <c r="F83" s="38"/>
     </row>
     <row r="84">
       <c r="B84" s="27"/>
-      <c r="C84" s="37"/>
-      <c r="D84" s="37"/>
+      <c r="C84" s="36"/>
+      <c r="D84" s="36"/>
       <c r="E84" s="29"/>
       <c r="F84" s="29"/>
     </row>
     <row r="85">
       <c r="A85" s="4"/>
-      <c r="B85" s="38" t="s">
+      <c r="B85" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="C85" s="32"/>
-      <c r="D85" s="32"/>
-      <c r="E85" s="39"/>
-      <c r="F85" s="39"/>
+      <c r="C85" s="31"/>
+      <c r="D85" s="31"/>
+      <c r="E85" s="38"/>
+      <c r="F85" s="38"/>
     </row>
     <row r="86">
       <c r="A86" s="4"/>
-      <c r="B86" s="38" t="s">
+      <c r="B86" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="C86" s="32"/>
-      <c r="D86" s="32"/>
-      <c r="E86" s="39"/>
-      <c r="F86" s="39"/>
+      <c r="C86" s="31"/>
+      <c r="D86" s="31"/>
+      <c r="E86" s="38"/>
+      <c r="F86" s="38"/>
     </row>
     <row r="87">
       <c r="B87" s="27"/>
-      <c r="C87" s="37"/>
-      <c r="D87" s="37"/>
+      <c r="C87" s="36"/>
+      <c r="D87" s="36"/>
       <c r="E87" s="29"/>
       <c r="F87" s="29"/>
     </row>
@@ -2509,8 +2546,8 @@
       <c r="B88" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C88" s="40"/>
-      <c r="D88" s="40"/>
+      <c r="C88" s="39"/>
+      <c r="D88" s="39"/>
       <c r="E88" s="4"/>
       <c r="F88" s="4"/>
     </row>
@@ -2519,8 +2556,8 @@
       <c r="B89" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="C89" s="40"/>
-      <c r="D89" s="40"/>
+      <c r="C89" s="39"/>
+      <c r="D89" s="39"/>
       <c r="E89" s="4"/>
       <c r="F89" s="4"/>
     </row>
@@ -8895,28 +8932,28 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="40" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="41" t="s">
         <v>116</v>
       </c>
-      <c r="C1" s="43" t="s">
+      <c r="C1" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="43" t="s">
         <v>118</v>
       </c>
-      <c r="E1" s="45" t="s">
+      <c r="E1" s="44" t="s">
         <v>119</v>
       </c>
-      <c r="F1" s="46" t="s">
+      <c r="F1" s="45" t="s">
         <v>120</v>
       </c>
-      <c r="G1" s="47" t="s">
+      <c r="G1" s="46" t="s">
         <v>121</v>
       </c>
-      <c r="H1" s="48" t="s">
+      <c r="H1" s="47" t="s">
         <v>122</v>
       </c>
     </row>
@@ -8924,25 +8961,25 @@
       <c r="A2" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="49" t="s">
+      <c r="B2" s="48" t="s">
         <v>27</v>
       </c>
       <c r="C2" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="D2" s="50" t="s">
+      <c r="D2" s="49" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="51" t="s">
+      <c r="E2" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="52" t="s">
+      <c r="F2" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="G2" s="53" t="s">
+      <c r="G2" s="52" t="s">
         <v>73</v>
       </c>
-      <c r="H2" s="54" t="s">
+      <c r="H2" s="53" t="s">
         <v>23</v>
       </c>
     </row>
@@ -8950,25 +8987,25 @@
       <c r="A3" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="48" t="s">
         <v>67</v>
       </c>
       <c r="C3" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="51" t="s">
+      <c r="E3" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="52" t="s">
+      <c r="F3" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="G3" s="53" t="s">
+      <c r="G3" s="52" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="54" t="s">
+      <c r="H3" s="53" t="s">
         <v>12</v>
       </c>
     </row>
@@ -8976,25 +9013,25 @@
       <c r="A4" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="49" t="s">
+      <c r="B4" s="48" t="s">
         <v>28</v>
       </c>
       <c r="C4" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="50" t="s">
+      <c r="D4" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="51" t="s">
+      <c r="E4" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="52" t="s">
+      <c r="F4" s="51" t="s">
         <v>44</v>
       </c>
-      <c r="G4" s="53" t="s">
+      <c r="G4" s="52" t="s">
         <v>56</v>
       </c>
-      <c r="H4" s="54" t="s">
+      <c r="H4" s="53" t="s">
         <v>24</v>
       </c>
     </row>
@@ -9002,22 +9039,22 @@
       <c r="A5" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B5" s="49" t="s">
+      <c r="B5" s="48" t="s">
         <v>40</v>
       </c>
       <c r="C5" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="50" t="s">
+      <c r="D5" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="51" t="s">
+      <c r="E5" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="F5" s="52" t="s">
+      <c r="F5" s="51" t="s">
         <v>45</v>
       </c>
-      <c r="G5" s="53" t="s">
+      <c r="G5" s="52" t="s">
         <v>38</v>
       </c>
       <c r="H5" s="8" t="s">
@@ -9025,8 +9062,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="55"/>
-      <c r="B6" s="55"/>
+      <c r="A6" s="54"/>
+      <c r="B6" s="54"/>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
       <c r="E6" s="12"/>
@@ -9070,10 +9107,10 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="56" t="s">
+      <c r="E1" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="56" t="s">
+      <c r="F1" s="55" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="3"/>
@@ -9082,19 +9119,19 @@
       <c r="A2" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="56" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="57" t="s">
+      <c r="C2" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="57" t="s">
+      <c r="D2" s="56" t="s">
         <v>59</v>
       </c>
-      <c r="E2" s="58">
+      <c r="E2" s="57">
         <v>10.0</v>
       </c>
-      <c r="F2" s="58">
+      <c r="F2" s="57">
         <v>2.0</v>
       </c>
     </row>
@@ -9102,19 +9139,19 @@
       <c r="A3" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="C3" s="59" t="s">
+      <c r="C3" s="58" t="s">
         <v>127</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="D3" s="58" t="s">
         <v>128</v>
       </c>
-      <c r="E3" s="58">
+      <c r="E3" s="57">
         <v>9.0</v>
       </c>
-      <c r="F3" s="58">
+      <c r="F3" s="57">
         <v>3.0</v>
       </c>
     </row>
@@ -9122,19 +9159,19 @@
       <c r="A4" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B4" s="60" t="s">
+      <c r="B4" s="59" t="s">
         <v>130</v>
       </c>
-      <c r="C4" s="60" t="s">
+      <c r="C4" s="59" t="s">
         <v>131</v>
       </c>
-      <c r="D4" s="60" t="s">
+      <c r="D4" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="58">
+      <c r="E4" s="57">
         <v>2.0</v>
       </c>
-      <c r="F4" s="58">
+      <c r="F4" s="57">
         <v>10.0</v>
       </c>
     </row>
@@ -9142,19 +9179,19 @@
       <c r="A5" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B5" s="61" t="s">
+      <c r="B5" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="C5" s="61" t="s">
+      <c r="C5" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="D5" s="61" t="s">
+      <c r="D5" s="60" t="s">
         <v>135</v>
       </c>
-      <c r="E5" s="58">
+      <c r="E5" s="57">
         <v>11.0</v>
       </c>
-      <c r="F5" s="58">
+      <c r="F5" s="57">
         <v>0.0</v>
       </c>
     </row>
@@ -9162,19 +9199,19 @@
       <c r="A6" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="61" t="s">
         <v>137</v>
       </c>
-      <c r="C6" s="62" t="s">
+      <c r="C6" s="61" t="s">
         <v>138</v>
       </c>
-      <c r="D6" s="62" t="s">
+      <c r="D6" s="61" t="s">
         <v>139</v>
       </c>
-      <c r="E6" s="58">
+      <c r="E6" s="57">
         <v>4.0</v>
       </c>
-      <c r="F6" s="58">
+      <c r="F6" s="57">
         <v>5.0</v>
       </c>
       <c r="N6" s="12"/>
@@ -9183,44 +9220,44 @@
       <c r="A7" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="B7" s="61" t="s">
+      <c r="B7" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="C7" s="61" t="s">
+      <c r="C7" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="61" t="s">
+      <c r="D7" s="60" t="s">
         <v>141</v>
       </c>
-      <c r="E7" s="58">
+      <c r="E7" s="57">
         <v>11.0</v>
       </c>
-      <c r="F7" s="58">
+      <c r="F7" s="57">
         <v>3.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14"/>
-      <c r="E8" s="63"/>
-      <c r="F8" s="63"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B9" s="61" t="s">
+      <c r="B9" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="C9" s="61" t="s">
+      <c r="C9" s="60" t="s">
         <v>76</v>
       </c>
-      <c r="D9" s="61" t="s">
+      <c r="D9" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="E9" s="58">
+      <c r="E9" s="57">
         <v>6.0</v>
       </c>
-      <c r="F9" s="58">
+      <c r="F9" s="57">
         <v>7.0</v>
       </c>
     </row>
@@ -9228,19 +9265,19 @@
       <c r="A10" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B10" s="57" t="s">
+      <c r="B10" s="56" t="s">
         <v>124</v>
       </c>
-      <c r="C10" s="57" t="s">
+      <c r="C10" s="56" t="s">
         <v>144</v>
       </c>
-      <c r="D10" s="57" t="s">
+      <c r="D10" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="58">
+      <c r="E10" s="57">
         <v>4.0</v>
       </c>
-      <c r="F10" s="58">
+      <c r="F10" s="57">
         <v>11.0</v>
       </c>
       <c r="H10" s="18"/>
@@ -9249,19 +9286,19 @@
       <c r="A11" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="B11" s="59" t="s">
+      <c r="B11" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="C11" s="59" t="s">
+      <c r="C11" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="59" t="s">
+      <c r="D11" s="58" t="s">
         <v>146</v>
       </c>
-      <c r="E11" s="58">
+      <c r="E11" s="57">
         <v>10.0</v>
       </c>
-      <c r="F11" s="58">
+      <c r="F11" s="57">
         <v>0.0</v>
       </c>
     </row>
@@ -9269,39 +9306,39 @@
       <c r="A12" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="B12" s="57" t="s">
+      <c r="B12" s="56" t="s">
         <v>124</v>
       </c>
-      <c r="C12" s="57" t="s">
+      <c r="C12" s="56" t="s">
         <v>148</v>
       </c>
-      <c r="D12" s="57" t="s">
+      <c r="D12" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="58">
+      <c r="E12" s="57">
         <v>2.0</v>
       </c>
-      <c r="F12" s="58">
+      <c r="F12" s="57">
         <v>11.0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="64" t="s">
+      <c r="A13" s="63" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="62" t="s">
+      <c r="B13" s="61" t="s">
         <v>137</v>
       </c>
-      <c r="C13" s="62" t="s">
+      <c r="C13" s="61" t="s">
         <v>63</v>
       </c>
-      <c r="D13" s="62" t="s">
+      <c r="D13" s="61" t="s">
         <v>150</v>
       </c>
-      <c r="E13" s="58">
+      <c r="E13" s="57">
         <v>6.0</v>
       </c>
-      <c r="F13" s="58">
+      <c r="F13" s="57">
         <v>5.0</v>
       </c>
     </row>
@@ -9309,19 +9346,19 @@
       <c r="A14" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B14" s="65" t="s">
+      <c r="B14" s="64" t="s">
         <v>152</v>
       </c>
-      <c r="C14" s="65" t="s">
+      <c r="C14" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="65" t="s">
+      <c r="D14" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="58">
+      <c r="E14" s="57">
         <v>10.0</v>
       </c>
-      <c r="F14" s="58">
+      <c r="F14" s="57">
         <v>3.0</v>
       </c>
       <c r="H14" s="18"/>
@@ -9336,19 +9373,19 @@
       <c r="A16" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="B16" s="65" t="s">
+      <c r="B16" s="64" t="s">
         <v>152</v>
       </c>
-      <c r="C16" s="65" t="s">
+      <c r="C16" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="65" t="s">
+      <c r="D16" s="64" t="s">
         <v>154</v>
       </c>
-      <c r="E16" s="58">
+      <c r="E16" s="57">
         <v>8.0</v>
       </c>
-      <c r="F16" s="58">
+      <c r="F16" s="57">
         <v>5.0</v>
       </c>
     </row>
@@ -9356,19 +9393,19 @@
       <c r="A17" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="B17" s="61" t="s">
+      <c r="B17" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="C17" s="61" t="s">
+      <c r="C17" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="61" t="s">
+      <c r="D17" s="60" t="s">
         <v>135</v>
       </c>
-      <c r="E17" s="58">
+      <c r="E17" s="57">
         <v>7.0</v>
       </c>
-      <c r="F17" s="58">
+      <c r="F17" s="57">
         <v>4.0</v>
       </c>
     </row>
@@ -9376,19 +9413,19 @@
       <c r="A18" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="B18" s="60" t="s">
+      <c r="B18" s="59" t="s">
         <v>130</v>
       </c>
-      <c r="C18" s="60" t="s">
+      <c r="C18" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="60" t="s">
+      <c r="D18" s="59" t="s">
         <v>157</v>
       </c>
-      <c r="E18" s="58">
+      <c r="E18" s="57">
         <v>7.0</v>
       </c>
-      <c r="F18" s="58">
+      <c r="F18" s="57">
         <v>5.0</v>
       </c>
     </row>
@@ -9396,19 +9433,19 @@
       <c r="A19" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="61" t="s">
+      <c r="D19" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="E19" s="58">
+      <c r="E19" s="57">
         <v>9.0</v>
       </c>
-      <c r="F19" s="58">
+      <c r="F19" s="57">
         <v>5.0</v>
       </c>
     </row>
@@ -9416,19 +9453,19 @@
       <c r="A20" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="B20" s="60" t="s">
+      <c r="B20" s="59" t="s">
         <v>130</v>
       </c>
-      <c r="C20" s="60" t="s">
+      <c r="C20" s="59" t="s">
         <v>131</v>
       </c>
-      <c r="D20" s="60" t="s">
+      <c r="D20" s="59" t="s">
         <v>160</v>
       </c>
-      <c r="E20" s="58">
+      <c r="E20" s="57">
         <v>6.0</v>
       </c>
-      <c r="F20" s="58">
+      <c r="F20" s="57">
         <v>8.0</v>
       </c>
     </row>
@@ -9436,19 +9473,19 @@
       <c r="A21" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="B21" s="60" t="s">
+      <c r="B21" s="59" t="s">
         <v>130</v>
       </c>
-      <c r="C21" s="60" t="s">
+      <c r="C21" s="59" t="s">
         <v>162</v>
       </c>
-      <c r="D21" s="60" t="s">
+      <c r="D21" s="59" t="s">
         <v>160</v>
       </c>
-      <c r="E21" s="58">
+      <c r="E21" s="57">
         <v>7.0</v>
       </c>
-      <c r="F21" s="58">
+      <c r="F21" s="57">
         <v>3.0</v>
       </c>
     </row>
@@ -9461,35 +9498,35 @@
       <c r="A23" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="B23" s="66" t="s">
+      <c r="B23" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="C23" s="66" t="s">
+      <c r="C23" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="D23" s="66" t="s">
+      <c r="D23" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="E23" s="33"/>
-      <c r="F23" s="33"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="B24" s="59" t="s">
+      <c r="B24" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="C24" s="59" t="s">
+      <c r="C24" s="58" t="s">
         <v>128</v>
       </c>
-      <c r="D24" s="59" t="s">
+      <c r="D24" s="58" t="s">
         <v>146</v>
       </c>
-      <c r="E24" s="58">
+      <c r="E24" s="57">
         <v>5.0</v>
       </c>
-      <c r="F24" s="58">
+      <c r="F24" s="57">
         <v>7.0</v>
       </c>
     </row>
@@ -9497,19 +9534,19 @@
       <c r="A25" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="B25" s="57" t="s">
+      <c r="B25" s="56" t="s">
         <v>124</v>
       </c>
-      <c r="C25" s="57" t="s">
+      <c r="C25" s="56" t="s">
         <v>148</v>
       </c>
-      <c r="D25" s="57" t="s">
+      <c r="D25" s="56" t="s">
         <v>59</v>
       </c>
-      <c r="E25" s="58">
+      <c r="E25" s="57">
         <v>5.0</v>
       </c>
-      <c r="F25" s="58">
+      <c r="F25" s="57">
         <v>11.0</v>
       </c>
     </row>
@@ -9517,59 +9554,59 @@
       <c r="A26" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="B26" s="60" t="s">
+      <c r="B26" s="59" t="s">
         <v>130</v>
       </c>
-      <c r="C26" s="60" t="s">
+      <c r="C26" s="59" t="s">
         <v>131</v>
       </c>
-      <c r="D26" s="60" t="s">
+      <c r="D26" s="59" t="s">
         <v>162</v>
       </c>
-      <c r="E26" s="58">
+      <c r="E26" s="57">
         <v>8.0</v>
       </c>
-      <c r="F26" s="58">
+      <c r="F26" s="57">
         <v>7.0</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="64" t="s">
+      <c r="A27" s="63" t="s">
         <v>168</v>
       </c>
-      <c r="B27" s="62" t="s">
+      <c r="B27" s="61" t="s">
         <v>137</v>
       </c>
-      <c r="C27" s="62" t="s">
+      <c r="C27" s="61" t="s">
         <v>138</v>
       </c>
-      <c r="D27" s="62" t="s">
+      <c r="D27" s="61" t="s">
         <v>150</v>
       </c>
-      <c r="E27" s="58">
+      <c r="E27" s="57">
         <v>8.0</v>
       </c>
-      <c r="F27" s="58">
+      <c r="F27" s="57">
         <v>3.0</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="64" t="s">
+      <c r="A28" s="63" t="s">
         <v>169</v>
       </c>
-      <c r="B28" s="62" t="s">
+      <c r="B28" s="61" t="s">
         <v>137</v>
       </c>
-      <c r="C28" s="62" t="s">
+      <c r="C28" s="61" t="s">
         <v>63</v>
       </c>
-      <c r="D28" s="62" t="s">
+      <c r="D28" s="61" t="s">
         <v>139</v>
       </c>
-      <c r="E28" s="58">
+      <c r="E28" s="57">
         <v>9.0</v>
       </c>
-      <c r="F28" s="58">
+      <c r="F28" s="57">
         <v>0.0</v>
       </c>
     </row>
@@ -9582,19 +9619,19 @@
       <c r="A30" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="B30" s="59" t="s">
+      <c r="B30" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="C30" s="59" t="s">
+      <c r="C30" s="58" t="s">
         <v>127</v>
       </c>
-      <c r="D30" s="59" t="s">
+      <c r="D30" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="E30" s="58">
+      <c r="E30" s="57">
         <v>12.0</v>
       </c>
-      <c r="F30" s="58">
+      <c r="F30" s="57">
         <v>1.0</v>
       </c>
     </row>
@@ -9602,19 +9639,19 @@
       <c r="A31" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="B31" s="61" t="s">
+      <c r="B31" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="C31" s="61" t="s">
+      <c r="C31" s="60" t="s">
         <v>76</v>
       </c>
-      <c r="D31" s="61" t="s">
+      <c r="D31" s="60" t="s">
         <v>135</v>
       </c>
-      <c r="E31" s="58">
+      <c r="E31" s="57">
         <v>5.0</v>
       </c>
-      <c r="F31" s="58">
+      <c r="F31" s="57">
         <v>4.0</v>
       </c>
     </row>
@@ -9622,19 +9659,19 @@
       <c r="A32" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="B32" s="60" t="s">
+      <c r="B32" s="59" t="s">
         <v>130</v>
       </c>
-      <c r="C32" s="60" t="s">
+      <c r="C32" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="60" t="s">
+      <c r="D32" s="59" t="s">
         <v>160</v>
       </c>
-      <c r="E32" s="58">
+      <c r="E32" s="57">
         <v>5.0</v>
       </c>
-      <c r="F32" s="58">
+      <c r="F32" s="57">
         <v>4.0</v>
       </c>
     </row>
@@ -9642,19 +9679,19 @@
       <c r="A33" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="B33" s="65" t="s">
+      <c r="B33" s="64" t="s">
         <v>152</v>
       </c>
-      <c r="C33" s="65" t="s">
+      <c r="C33" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="D33" s="65" t="s">
+      <c r="D33" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="E33" s="58">
+      <c r="E33" s="57">
         <v>8.0</v>
       </c>
-      <c r="F33" s="58">
+      <c r="F33" s="57">
         <v>6.0</v>
       </c>
     </row>
@@ -9662,19 +9699,19 @@
       <c r="A34" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="B34" s="61" t="s">
+      <c r="B34" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="C34" s="61" t="s">
+      <c r="C34" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="D34" s="61" t="s">
+      <c r="D34" s="60" t="s">
         <v>141</v>
       </c>
-      <c r="E34" s="58">
+      <c r="E34" s="57">
         <v>9.0</v>
       </c>
-      <c r="F34" s="58">
+      <c r="F34" s="57">
         <v>3.0</v>
       </c>
     </row>
@@ -9682,19 +9719,19 @@
       <c r="A35" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="B35" s="65" t="s">
+      <c r="B35" s="64" t="s">
         <v>152</v>
       </c>
-      <c r="C35" s="65" t="s">
+      <c r="C35" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="D35" s="65" t="s">
+      <c r="D35" s="64" t="s">
         <v>154</v>
       </c>
-      <c r="E35" s="58">
+      <c r="E35" s="57">
         <v>2.0</v>
       </c>
-      <c r="F35" s="58">
+      <c r="F35" s="57">
         <v>10.0</v>
       </c>
     </row>
@@ -9707,55 +9744,55 @@
       <c r="A37" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="B37" s="66" t="s">
+      <c r="B37" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="C37" s="66" t="s">
+      <c r="C37" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="D37" s="66" t="s">
+      <c r="D37" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="E37" s="33"/>
-      <c r="F37" s="33"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="B38" s="62" t="s">
+      <c r="B38" s="61" t="s">
         <v>137</v>
       </c>
-      <c r="C38" s="62" t="s">
+      <c r="C38" s="61" t="s">
         <v>150</v>
       </c>
-      <c r="D38" s="62" t="s">
+      <c r="D38" s="61" t="s">
         <v>139</v>
       </c>
-      <c r="E38" s="58">
+      <c r="E38" s="57">
         <v>8.0</v>
       </c>
-      <c r="F38" s="58">
+      <c r="F38" s="57">
         <v>3.0</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="64" t="s">
+      <c r="A39" s="63" t="s">
         <v>178</v>
       </c>
-      <c r="B39" s="65" t="s">
+      <c r="B39" s="64" t="s">
         <v>152</v>
       </c>
-      <c r="C39" s="65" t="s">
+      <c r="C39" s="64" t="s">
         <v>154</v>
       </c>
-      <c r="D39" s="65" t="s">
+      <c r="D39" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="E39" s="58">
+      <c r="E39" s="57">
         <v>7.0</v>
       </c>
-      <c r="F39" s="58">
+      <c r="F39" s="57">
         <v>8.0</v>
       </c>
     </row>
@@ -9763,19 +9800,19 @@
       <c r="A40" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="B40" s="57" t="s">
+      <c r="B40" s="56" t="s">
         <v>124</v>
       </c>
-      <c r="C40" s="57" t="s">
+      <c r="C40" s="56" t="s">
         <v>144</v>
       </c>
-      <c r="D40" s="57" t="s">
+      <c r="D40" s="56" t="s">
         <v>148</v>
       </c>
-      <c r="E40" s="58">
+      <c r="E40" s="57">
         <v>1.0</v>
       </c>
-      <c r="F40" s="58">
+      <c r="F40" s="57">
         <v>10.0</v>
       </c>
     </row>
@@ -9783,19 +9820,19 @@
       <c r="A41" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="B41" s="59" t="s">
+      <c r="B41" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="C41" s="59" t="s">
+      <c r="C41" s="58" t="s">
         <v>128</v>
       </c>
-      <c r="D41" s="59" t="s">
+      <c r="D41" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="E41" s="58">
+      <c r="E41" s="57">
         <v>6.0</v>
       </c>
-      <c r="F41" s="58">
+      <c r="F41" s="57">
         <v>7.0</v>
       </c>
     </row>
@@ -9803,17 +9840,17 @@
       <c r="A42" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="B42" s="66" t="s">
+      <c r="B42" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="C42" s="66" t="s">
+      <c r="C42" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="D42" s="66" t="s">
+      <c r="D42" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="E42" s="33"/>
-      <c r="F42" s="33"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="32"/>
     </row>
     <row r="43">
       <c r="A43" s="14"/>
@@ -9824,51 +9861,51 @@
       <c r="A44" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="B44" s="66" t="s">
+      <c r="B44" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="C44" s="66" t="s">
+      <c r="C44" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="D44" s="66" t="s">
+      <c r="D44" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="E44" s="33"/>
-      <c r="F44" s="33"/>
+      <c r="E44" s="32"/>
+      <c r="F44" s="32"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="B45" s="66" t="s">
+      <c r="B45" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="C45" s="66" t="s">
+      <c r="C45" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="D45" s="66" t="s">
+      <c r="D45" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="E45" s="33"/>
-      <c r="F45" s="33"/>
+      <c r="E45" s="32"/>
+      <c r="F45" s="32"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="B46" s="62" t="s">
+      <c r="B46" s="61" t="s">
         <v>137</v>
       </c>
-      <c r="C46" s="62" t="s">
+      <c r="C46" s="61" t="s">
         <v>63</v>
       </c>
-      <c r="D46" s="62" t="s">
+      <c r="D46" s="61" t="s">
         <v>138</v>
       </c>
-      <c r="E46" s="58">
+      <c r="E46" s="57">
         <v>7.0</v>
       </c>
-      <c r="F46" s="58">
+      <c r="F46" s="57">
         <v>5.0</v>
       </c>
     </row>
@@ -9876,19 +9913,19 @@
       <c r="A47" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="B47" s="60" t="s">
+      <c r="B47" s="59" t="s">
         <v>130</v>
       </c>
-      <c r="C47" s="60" t="s">
+      <c r="C47" s="59" t="s">
         <v>162</v>
       </c>
-      <c r="D47" s="60" t="s">
+      <c r="D47" s="59" t="s">
         <v>157</v>
       </c>
-      <c r="E47" s="58">
+      <c r="E47" s="57">
         <v>4.0</v>
       </c>
-      <c r="F47" s="58">
+      <c r="F47" s="57">
         <v>6.0</v>
       </c>
     </row>
@@ -9896,19 +9933,19 @@
       <c r="A48" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="B48" s="65" t="s">
+      <c r="B48" s="64" t="s">
         <v>152</v>
       </c>
-      <c r="C48" s="65" t="s">
+      <c r="C48" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="D48" s="65" t="s">
+      <c r="D48" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="E48" s="58">
+      <c r="E48" s="57">
         <v>11.0</v>
       </c>
-      <c r="F48" s="58">
+      <c r="F48" s="57">
         <v>3.0</v>
       </c>
     </row>
@@ -9916,19 +9953,19 @@
       <c r="A49" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="B49" s="61" t="s">
+      <c r="B49" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="C49" s="61" t="s">
+      <c r="C49" s="60" t="s">
         <v>76</v>
       </c>
-      <c r="D49" s="61" t="s">
+      <c r="D49" s="60" t="s">
         <v>141</v>
       </c>
-      <c r="E49" s="58">
+      <c r="E49" s="57">
         <v>6.0</v>
       </c>
-      <c r="F49" s="58">
+      <c r="F49" s="57">
         <v>7.0</v>
       </c>
     </row>
@@ -9941,97 +9978,97 @@
       <c r="A51" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="B51" s="60" t="s">
+      <c r="B51" s="59" t="s">
         <v>130</v>
       </c>
-      <c r="C51" s="60" t="s">
+      <c r="C51" s="59" t="s">
         <v>131</v>
       </c>
-      <c r="D51" s="60" t="s">
+      <c r="D51" s="59" t="s">
         <v>157</v>
       </c>
-      <c r="E51" s="33"/>
-      <c r="F51" s="33"/>
+      <c r="E51" s="32"/>
+      <c r="F51" s="32"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="B52" s="59" t="s">
+      <c r="B52" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="C52" s="59" t="s">
+      <c r="C52" s="58" t="s">
         <v>127</v>
       </c>
-      <c r="D52" s="59" t="s">
+      <c r="D52" s="58" t="s">
         <v>146</v>
       </c>
-      <c r="E52" s="33"/>
-      <c r="F52" s="33"/>
+      <c r="E52" s="32"/>
+      <c r="F52" s="32"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="B53" s="60" t="s">
+      <c r="B53" s="59" t="s">
         <v>130</v>
       </c>
-      <c r="C53" s="60" t="s">
+      <c r="C53" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="D53" s="60" t="s">
+      <c r="D53" s="59" t="s">
         <v>162</v>
       </c>
-      <c r="E53" s="33"/>
-      <c r="F53" s="33"/>
+      <c r="E53" s="32"/>
+      <c r="F53" s="32"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="B54" s="61" t="s">
+      <c r="B54" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="C54" s="61" t="s">
+      <c r="C54" s="60" t="s">
         <v>76</v>
       </c>
-      <c r="D54" s="61" t="s">
+      <c r="D54" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="E54" s="33"/>
-      <c r="F54" s="33"/>
+      <c r="E54" s="32"/>
+      <c r="F54" s="32"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="B55" s="66" t="s">
+      <c r="B55" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="C55" s="66" t="s">
+      <c r="C55" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="D55" s="66" t="s">
+      <c r="D55" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="E55" s="33"/>
-      <c r="F55" s="33"/>
+      <c r="E55" s="32"/>
+      <c r="F55" s="32"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="s">
         <v>193</v>
       </c>
-      <c r="B56" s="66" t="s">
+      <c r="B56" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="C56" s="66" t="s">
+      <c r="C56" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="D56" s="66" t="s">
+      <c r="D56" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="E56" s="33"/>
-      <c r="F56" s="33"/>
+      <c r="E56" s="32"/>
+      <c r="F56" s="32"/>
     </row>
     <row r="57">
       <c r="A57" s="14"/>
@@ -10042,97 +10079,97 @@
       <c r="A58" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="B58" s="66" t="s">
+      <c r="B58" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="C58" s="66" t="s">
+      <c r="C58" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="D58" s="66" t="s">
+      <c r="D58" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="E58" s="33"/>
-      <c r="F58" s="33"/>
+      <c r="E58" s="32"/>
+      <c r="F58" s="32"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="B59" s="57" t="s">
+      <c r="B59" s="56" t="s">
         <v>124</v>
       </c>
-      <c r="C59" s="57" t="s">
+      <c r="C59" s="56" t="s">
         <v>144</v>
       </c>
-      <c r="D59" s="57" t="s">
+      <c r="D59" s="56" t="s">
         <v>59</v>
       </c>
-      <c r="E59" s="33"/>
-      <c r="F59" s="33"/>
+      <c r="E59" s="32"/>
+      <c r="F59" s="32"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="B60" s="61" t="s">
+      <c r="B60" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="C60" s="61" t="s">
+      <c r="C60" s="60" t="s">
         <v>135</v>
       </c>
-      <c r="D60" s="61" t="s">
+      <c r="D60" s="60" t="s">
         <v>141</v>
       </c>
-      <c r="E60" s="33"/>
-      <c r="F60" s="33"/>
+      <c r="E60" s="32"/>
+      <c r="F60" s="32"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="B61" s="60" t="s">
+      <c r="B61" s="59" t="s">
         <v>130</v>
       </c>
-      <c r="C61" s="60" t="s">
+      <c r="C61" s="59" t="s">
         <v>160</v>
       </c>
-      <c r="D61" s="60" t="s">
+      <c r="D61" s="59" t="s">
         <v>157</v>
       </c>
-      <c r="E61" s="33"/>
-      <c r="F61" s="33"/>
+      <c r="E61" s="32"/>
+      <c r="F61" s="32"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="B62" s="66" t="s">
+      <c r="B62" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="C62" s="66" t="s">
+      <c r="C62" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="D62" s="66" t="s">
+      <c r="D62" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="E62" s="33"/>
-      <c r="F62" s="33"/>
+      <c r="E62" s="32"/>
+      <c r="F62" s="32"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="s">
         <v>199</v>
       </c>
-      <c r="B63" s="66" t="s">
+      <c r="B63" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="C63" s="66" t="s">
+      <c r="C63" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="D63" s="66" t="s">
+      <c r="D63" s="65" t="s">
         <v>164</v>
       </c>
-      <c r="E63" s="33"/>
-      <c r="F63" s="33"/>
+      <c r="E63" s="32"/>
+      <c r="F63" s="32"/>
     </row>
     <row r="64">
       <c r="E64" s="29"/>
@@ -10142,70 +10179,70 @@
       <c r="A65" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="B65" s="31" t="s">
+      <c r="B65" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C65" s="61" t="s">
+      <c r="C65" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="D65" s="61" t="s">
+      <c r="D65" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="E65" s="33"/>
-      <c r="F65" s="33"/>
+      <c r="E65" s="32"/>
+      <c r="F65" s="32"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="B66" s="31" t="s">
+      <c r="B66" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C66" s="60" t="s">
+      <c r="C66" s="59" t="s">
         <v>134</v>
       </c>
-      <c r="D66" s="60" t="s">
+      <c r="D66" s="59" t="s">
         <v>59</v>
       </c>
-      <c r="E66" s="33"/>
-      <c r="F66" s="33"/>
+      <c r="E66" s="32"/>
+      <c r="F66" s="32"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="B67" s="31" t="s">
+      <c r="B67" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C67" s="60" t="s">
+      <c r="C67" s="59" t="s">
         <v>141</v>
       </c>
-      <c r="D67" s="60" t="s">
+      <c r="D67" s="59" t="s">
         <v>63</v>
       </c>
-      <c r="E67" s="33"/>
-      <c r="F67" s="33"/>
+      <c r="E67" s="32"/>
+      <c r="F67" s="32"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="B68" s="31" t="s">
+      <c r="B68" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C68" s="59" t="s">
+      <c r="C68" s="58" t="s">
         <v>204</v>
       </c>
-      <c r="D68" s="59" t="s">
+      <c r="D68" s="58" t="s">
         <v>150</v>
       </c>
-      <c r="E68" s="33"/>
-      <c r="F68" s="33"/>
+      <c r="E68" s="32"/>
+      <c r="F68" s="32"/>
     </row>
     <row r="69">
-      <c r="B69" s="35"/>
-      <c r="C69" s="67"/>
-      <c r="D69" s="67"/>
+      <c r="B69" s="34"/>
+      <c r="C69" s="66"/>
+      <c r="D69" s="66"/>
       <c r="E69" s="29"/>
       <c r="F69" s="29"/>
     </row>
@@ -10213,65 +10250,65 @@
       <c r="A70" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="B70" s="31" t="s">
+      <c r="B70" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C70" s="59" t="s">
+      <c r="C70" s="58" t="s">
         <v>127</v>
       </c>
-      <c r="D70" s="59" t="s">
+      <c r="D70" s="58" t="s">
         <v>51</v>
       </c>
-      <c r="E70" s="36"/>
-      <c r="F70" s="36"/>
+      <c r="E70" s="35"/>
+      <c r="F70" s="35"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="B71" s="31" t="s">
+      <c r="B71" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C71" s="65" t="s">
+      <c r="C71" s="64" t="s">
         <v>207</v>
       </c>
-      <c r="D71" s="65" t="s">
+      <c r="D71" s="64" t="s">
         <v>53</v>
       </c>
-      <c r="E71" s="36"/>
-      <c r="F71" s="36"/>
+      <c r="E71" s="35"/>
+      <c r="F71" s="35"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="B72" s="31" t="s">
+      <c r="B72" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C72" s="65" t="s">
+      <c r="C72" s="64" t="s">
         <v>209</v>
       </c>
-      <c r="D72" s="65" t="s">
+      <c r="D72" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="E72" s="36"/>
-      <c r="F72" s="36"/>
+      <c r="E72" s="35"/>
+      <c r="F72" s="35"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="B73" s="31" t="s">
+      <c r="B73" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C73" s="61" t="s">
+      <c r="C73" s="60" t="s">
         <v>157</v>
       </c>
-      <c r="D73" s="61" t="s">
+      <c r="D73" s="60" t="s">
         <v>138</v>
       </c>
-      <c r="E73" s="36"/>
-      <c r="F73" s="36"/>
+      <c r="E73" s="35"/>
+      <c r="F73" s="35"/>
     </row>
     <row r="74">
       <c r="B74" s="27"/>
@@ -10282,49 +10319,49 @@
       <c r="A75" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="B75" s="38" t="s">
+      <c r="B75" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="C75" s="61"/>
-      <c r="D75" s="61"/>
-      <c r="E75" s="39"/>
-      <c r="F75" s="39"/>
+      <c r="C75" s="60"/>
+      <c r="D75" s="60"/>
+      <c r="E75" s="38"/>
+      <c r="F75" s="38"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="B76" s="38" t="s">
+      <c r="B76" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="C76" s="60"/>
-      <c r="D76" s="60"/>
-      <c r="E76" s="39"/>
-      <c r="F76" s="39"/>
+      <c r="C76" s="59"/>
+      <c r="D76" s="59"/>
+      <c r="E76" s="38"/>
+      <c r="F76" s="38"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="B77" s="38" t="s">
+      <c r="B77" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="C77" s="59"/>
-      <c r="D77" s="59"/>
-      <c r="E77" s="39"/>
-      <c r="F77" s="39"/>
+      <c r="C77" s="58"/>
+      <c r="D77" s="58"/>
+      <c r="E77" s="38"/>
+      <c r="F77" s="38"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="B78" s="38" t="s">
+      <c r="B78" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="C78" s="65"/>
-      <c r="D78" s="65"/>
-      <c r="E78" s="39"/>
-      <c r="F78" s="39"/>
+      <c r="C78" s="64"/>
+      <c r="D78" s="64"/>
+      <c r="E78" s="38"/>
+      <c r="F78" s="38"/>
     </row>
     <row r="79">
       <c r="E79" s="29"/>
@@ -10334,25 +10371,25 @@
       <c r="A80" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="B80" s="38" t="s">
+      <c r="B80" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="C80" s="60"/>
-      <c r="D80" s="68"/>
-      <c r="E80" s="39"/>
-      <c r="F80" s="39"/>
+      <c r="C80" s="59"/>
+      <c r="D80" s="67"/>
+      <c r="E80" s="38"/>
+      <c r="F80" s="38"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="B81" s="38" t="s">
+      <c r="B81" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="C81" s="65"/>
-      <c r="D81" s="61"/>
-      <c r="E81" s="39"/>
-      <c r="F81" s="39"/>
+      <c r="C81" s="64"/>
+      <c r="D81" s="60"/>
+      <c r="E81" s="38"/>
+      <c r="F81" s="38"/>
     </row>
     <row r="82">
       <c r="E82" s="29"/>
@@ -14062,110 +14099,110 @@
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="68" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="C1" s="43" t="s">
+      <c r="C1" s="42" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="43" t="s">
         <v>137</v>
       </c>
-      <c r="E1" s="45" t="s">
+      <c r="E1" s="44" t="s">
         <v>152</v>
       </c>
-      <c r="F1" s="46" t="s">
+      <c r="F1" s="45" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="61" t="s">
+      <c r="A2" s="60" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="60" t="s">
+      <c r="B2" s="59" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="57" t="s">
+      <c r="C2" s="56" t="s">
         <v>219</v>
       </c>
-      <c r="D2" s="70" t="s">
+      <c r="D2" s="69" t="s">
         <v>220</v>
       </c>
-      <c r="E2" s="65" t="s">
+      <c r="E2" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="71" t="s">
+      <c r="F2" s="70" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="B3" s="60" t="s">
+      <c r="B3" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="57">
+      <c r="C3" s="56">
         <v>104.0</v>
       </c>
-      <c r="D3" s="70" t="s">
+      <c r="D3" s="69" t="s">
         <v>138</v>
       </c>
-      <c r="E3" s="65" t="s">
+      <c r="E3" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="F3" s="71" t="s">
+      <c r="F3" s="70" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="61" t="s">
+      <c r="A4" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="B4" s="60" t="s">
+      <c r="B4" s="59" t="s">
         <v>162</v>
       </c>
-      <c r="C4" s="57" t="s">
+      <c r="C4" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="70" t="s">
+      <c r="D4" s="69" t="s">
         <v>150</v>
       </c>
-      <c r="E4" s="65" t="s">
+      <c r="E4" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="71" t="s">
+      <c r="F4" s="70" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="61" t="s">
+      <c r="A5" s="60" t="s">
         <v>135</v>
       </c>
-      <c r="B5" s="60" t="s">
+      <c r="B5" s="59" t="s">
         <v>160</v>
       </c>
-      <c r="C5" s="57" t="s">
+      <c r="C5" s="56" t="s">
         <v>59</v>
       </c>
-      <c r="D5" s="70" t="s">
+      <c r="D5" s="69" t="s">
         <v>139</v>
       </c>
-      <c r="E5" s="65" t="s">
+      <c r="E5" s="64" t="s">
         <v>154</v>
       </c>
-      <c r="F5" s="71" t="s">
+      <c r="F5" s="70" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="s">
+      <c r="A6" s="60" t="s">
         <v>141</v>
       </c>
-      <c r="B6" s="60" t="s">
+      <c r="B6" s="59" t="s">
         <v>157</v>
       </c>
       <c r="C6" s="12"/>

</xml_diff>

<commit_message>
Dati: 3 spostamenti di calendario (25/06 e 30/06)
Rigenerato da Calend Bocce 2026 (1).xlsx via tools/build_data.py.

Calendario:
- G: I Masalen vs Gli Hummarell: mar 30/06 22:30 -> gio 25/06 23:00
- C: La Coppia vs I Cugini: lun 29/06 20:30 -> mar 30/06 22:00
- F: T alla seconda vs I Cavalli: mar 30/06 22:00 -> mar 30/06 22:30

Risultati e classifiche invariati. Nessuna sovrapposizione di slot.
Nota: La Coppia gioca due volte il 30/06 a 30 min (21:30 e 22:00), accettato.
Cache-busting v=202606251751.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -2148,12 +2148,18 @@
       <c r="F50" s="6"/>
     </row>
     <row r="51">
-      <c r="A51" s="25" t="s">
+      <c r="A51" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B51" s="23"/>
-      <c r="C51" s="23"/>
-      <c r="D51" s="23"/>
+      <c r="B51" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C51" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D51" s="19" t="s">
+        <v>56</v>
+      </c>
       <c r="E51" s="6"/>
       <c r="F51" s="6"/>
     </row>
@@ -2166,18 +2172,12 @@
       <c r="F52" s="20"/>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="s">
+      <c r="A53" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="B53" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C53" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="D53" s="21" t="s">
-        <v>51</v>
-      </c>
+      <c r="B53" s="23"/>
+      <c r="C53" s="23"/>
+      <c r="D53" s="23"/>
       <c r="E53" s="26"/>
       <c r="F53" s="26"/>
     </row>
@@ -2315,14 +2315,14 @@
       <c r="A63" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B63" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="C63" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="D63" s="17" t="s">
-        <v>44</v>
+      <c r="B63" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C63" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="D63" s="21" t="s">
+        <v>51</v>
       </c>
       <c r="E63" s="26"/>
       <c r="F63" s="26"/>
@@ -2331,14 +2331,14 @@
       <c r="A64" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="B64" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="C64" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="D64" s="19" t="s">
-        <v>56</v>
+      <c r="B64" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C64" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D64" s="17" t="s">
+        <v>44</v>
       </c>
       <c r="E64" s="26"/>
       <c r="F64" s="26"/>

</xml_diff>

<commit_message>
Dati: 6 risultati; baseline classifiche aggiornato (G, H)
Rigenerato da Calend Bocce 2026 (1).xlsx via tools/build_data.py.

Risultati (giocate 32 -> 38):
- B: Apostadores 3-6 The Doctors; Apostadores 0-9 Lord&Chri
- C: 0Sbat 2-7 I Cugini
- E: Le Cognate 3-10 Bad Boys
- G: I Masalen 1-10 Gli Hummarell
- H: Le Sbocciate 1-9 Team Rocket

Ordine cambiato: G, H -> baseline 'expected' aggiornato in build_data.py.
Nessuna modifica di calendario. Nessuna sovrapposizione di slot (campo unico).
Cache-busting v=202606260859.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="225">
   <si>
     <t>data e ora</t>
   </si>
@@ -322,24 +322,12 @@
     <t>martedì 30/06 23:00</t>
   </si>
   <si>
-    <t>mercoledì 01/07 20:30</t>
+    <t>giovedì 02/07 20:30</t>
   </si>
   <si>
     <t>OTT</t>
   </si>
   <si>
-    <t>mercoledì 01/07 21:15</t>
-  </si>
-  <si>
-    <t>mercoledì 01/07 22:00</t>
-  </si>
-  <si>
-    <t>mercoledì 01/07 22:45</t>
-  </si>
-  <si>
-    <t>giovedì 02/07 20:30</t>
-  </si>
-  <si>
     <t>giovedì 02/07 21:15</t>
   </si>
   <si>
@@ -349,7 +337,31 @@
     <t>giovedì 02/07 22:45</t>
   </si>
   <si>
+    <t>martedì 07/07 20:30</t>
+  </si>
+  <si>
+    <t>martedì 07/07 21:15</t>
+  </si>
+  <si>
+    <t>martedì 07/07 22:00</t>
+  </si>
+  <si>
+    <t>martedì 07/07 22:45</t>
+  </si>
+  <si>
+    <t>giovedì 09/07 20:30</t>
+  </si>
+  <si>
     <t>QUAR</t>
+  </si>
+  <si>
+    <t>giovedì 09/07 21:15</t>
+  </si>
+  <si>
+    <t>giovedì 09/07 22:00</t>
+  </si>
+  <si>
+    <t>giovedì 09/07 22:45</t>
   </si>
   <si>
     <t>SEMI</t>
@@ -2080,8 +2092,12 @@
       <c r="D46" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="E46" s="26"/>
-      <c r="F46" s="26"/>
+      <c r="E46" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="F46" s="6">
+        <v>6.0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="s">
@@ -2096,8 +2112,12 @@
       <c r="D47" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="E47" s="26"/>
-      <c r="F47" s="26"/>
+      <c r="E47" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="F47" s="6">
+        <v>7.0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="s">
@@ -2112,8 +2132,12 @@
       <c r="D48" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E48" s="6"/>
-      <c r="F48" s="6"/>
+      <c r="E48" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="F48" s="6">
+        <v>10.0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="s">
@@ -2128,8 +2152,12 @@
       <c r="D49" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E49" s="6"/>
-      <c r="F49" s="6"/>
+      <c r="E49" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="F49" s="6">
+        <v>9.0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="s">
@@ -2144,8 +2172,12 @@
       <c r="D50" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E50" s="6"/>
-      <c r="F50" s="6"/>
+      <c r="E50" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="F50" s="6">
+        <v>9.0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="s">
@@ -2160,8 +2192,12 @@
       <c r="D51" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="E51" s="6"/>
-      <c r="F51" s="6"/>
+      <c r="E51" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="F51" s="6">
+        <v>10.0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="14"/>
@@ -2468,9 +2504,11 @@
       <c r="F79" s="29"/>
     </row>
     <row r="80">
-      <c r="A80" s="4"/>
+      <c r="A80" s="4" t="s">
+        <v>111</v>
+      </c>
       <c r="B80" s="37" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C80" s="31"/>
       <c r="D80" s="31"/>
@@ -2478,9 +2516,11 @@
       <c r="F80" s="38"/>
     </row>
     <row r="81">
-      <c r="A81" s="4"/>
+      <c r="A81" s="4" t="s">
+        <v>113</v>
+      </c>
       <c r="B81" s="37" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C81" s="31"/>
       <c r="D81" s="31"/>
@@ -2488,9 +2528,11 @@
       <c r="F81" s="38"/>
     </row>
     <row r="82">
-      <c r="A82" s="4"/>
+      <c r="A82" s="4" t="s">
+        <v>114</v>
+      </c>
       <c r="B82" s="37" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C82" s="33"/>
       <c r="D82" s="33"/>
@@ -2498,9 +2540,11 @@
       <c r="F82" s="38"/>
     </row>
     <row r="83">
-      <c r="A83" s="4"/>
+      <c r="A83" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="B83" s="37" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C83" s="31"/>
       <c r="D83" s="31"/>
@@ -2517,7 +2561,7 @@
     <row r="85">
       <c r="A85" s="4"/>
       <c r="B85" s="37" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C85" s="31"/>
       <c r="D85" s="31"/>
@@ -2527,7 +2571,7 @@
     <row r="86">
       <c r="A86" s="4"/>
       <c r="B86" s="37" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C86" s="31"/>
       <c r="D86" s="31"/>
@@ -2544,7 +2588,7 @@
     <row r="88">
       <c r="A88" s="4"/>
       <c r="B88" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C88" s="39"/>
       <c r="D88" s="39"/>
@@ -2554,7 +2598,7 @@
     <row r="89">
       <c r="A89" s="4"/>
       <c r="B89" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C89" s="39"/>
       <c r="D89" s="39"/>
@@ -8933,28 +8977,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="40" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B1" s="41" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C1" s="42" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D1" s="43" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E1" s="44" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F1" s="45" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G1" s="46" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H1" s="47" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2">
@@ -9117,10 +9161,10 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B2" s="56" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C2" s="56" t="s">
         <v>21</v>
@@ -9137,16 +9181,16 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B3" s="58" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C3" s="58" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D3" s="58" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E3" s="57">
         <v>9.0</v>
@@ -9157,13 +9201,13 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B4" s="59" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C4" s="59" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D4" s="59" t="s">
         <v>40</v>
@@ -9177,16 +9221,16 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B5" s="60" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C5" s="60" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D5" s="60" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E5" s="57">
         <v>11.0</v>
@@ -9197,16 +9241,16 @@
     </row>
     <row r="6">
       <c r="A6" s="11" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B6" s="61" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C6" s="61" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D6" s="61" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E6" s="57">
         <v>4.0</v>
@@ -9218,16 +9262,16 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B7" s="60" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C7" s="60" t="s">
         <v>47</v>
       </c>
       <c r="D7" s="60" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E7" s="57">
         <v>11.0</v>
@@ -9243,16 +9287,16 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B9" s="60" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C9" s="60" t="s">
         <v>76</v>
       </c>
       <c r="D9" s="60" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E9" s="57">
         <v>6.0</v>
@@ -9263,13 +9307,13 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B10" s="56" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C10" s="56" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D10" s="56" t="s">
         <v>21</v>
@@ -9284,16 +9328,16 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B11" s="58" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C11" s="58" t="s">
         <v>37</v>
       </c>
       <c r="D11" s="58" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E11" s="57">
         <v>10.0</v>
@@ -9304,13 +9348,13 @@
     </row>
     <row r="12">
       <c r="A12" s="11" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B12" s="56" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C12" s="56" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D12" s="56" t="s">
         <v>21</v>
@@ -9324,16 +9368,16 @@
     </row>
     <row r="13">
       <c r="A13" s="63" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B13" s="61" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C13" s="61" t="s">
         <v>63</v>
       </c>
       <c r="D13" s="61" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="E13" s="57">
         <v>6.0</v>
@@ -9344,10 +9388,10 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B14" s="64" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C14" s="64" t="s">
         <v>30</v>
@@ -9371,16 +9415,16 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B16" s="64" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C16" s="64" t="s">
         <v>30</v>
       </c>
       <c r="D16" s="64" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="E16" s="57">
         <v>8.0</v>
@@ -9391,16 +9435,16 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B17" s="60" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C17" s="60" t="s">
         <v>47</v>
       </c>
       <c r="D17" s="60" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E17" s="57">
         <v>7.0</v>
@@ -9411,16 +9455,16 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B18" s="59" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C18" s="59" t="s">
         <v>40</v>
       </c>
       <c r="D18" s="59" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E18" s="57">
         <v>7.0</v>
@@ -9431,16 +9475,16 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B19" s="60" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C19" s="60" t="s">
         <v>47</v>
       </c>
       <c r="D19" s="60" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E19" s="57">
         <v>9.0</v>
@@ -9451,16 +9495,16 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B20" s="59" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C20" s="59" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D20" s="59" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="E20" s="57">
         <v>6.0</v>
@@ -9471,16 +9515,16 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B21" s="59" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C21" s="59" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D21" s="59" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="E21" s="57">
         <v>7.0</v>
@@ -9496,32 +9540,32 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B23" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C23" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D23" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E23" s="32"/>
       <c r="F23" s="32"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B24" s="58" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C24" s="58" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D24" s="58" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E24" s="57">
         <v>5.0</v>
@@ -9532,13 +9576,13 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B25" s="56" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C25" s="56" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D25" s="56" t="s">
         <v>59</v>
@@ -9552,16 +9596,16 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B26" s="59" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C26" s="59" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D26" s="59" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="E26" s="57">
         <v>8.0</v>
@@ -9572,16 +9616,16 @@
     </row>
     <row r="27">
       <c r="A27" s="63" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B27" s="61" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C27" s="61" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D27" s="61" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="E27" s="57">
         <v>8.0</v>
@@ -9592,16 +9636,16 @@
     </row>
     <row r="28">
       <c r="A28" s="63" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B28" s="61" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C28" s="61" t="s">
         <v>63</v>
       </c>
       <c r="D28" s="61" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E28" s="57">
         <v>9.0</v>
@@ -9617,13 +9661,13 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B30" s="58" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C30" s="58" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D30" s="58" t="s">
         <v>37</v>
@@ -9637,16 +9681,16 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B31" s="60" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C31" s="60" t="s">
         <v>76</v>
       </c>
       <c r="D31" s="60" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E31" s="57">
         <v>5.0</v>
@@ -9657,16 +9701,16 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B32" s="59" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C32" s="59" t="s">
         <v>40</v>
       </c>
       <c r="D32" s="59" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="E32" s="57">
         <v>5.0</v>
@@ -9677,10 +9721,10 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B33" s="64" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C33" s="64" t="s">
         <v>30</v>
@@ -9697,16 +9741,16 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B34" s="60" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C34" s="60" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D34" s="60" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E34" s="57">
         <v>9.0</v>
@@ -9717,16 +9761,16 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B35" s="64" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C35" s="64" t="s">
         <v>27</v>
       </c>
       <c r="D35" s="64" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="E35" s="57">
         <v>2.0</v>
@@ -9742,32 +9786,32 @@
     </row>
     <row r="37">
       <c r="A37" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B37" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C37" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D37" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E37" s="32"/>
       <c r="F37" s="32"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B38" s="61" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C38" s="61" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="D38" s="61" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E38" s="57">
         <v>8.0</v>
@@ -9778,13 +9822,13 @@
     </row>
     <row r="39">
       <c r="A39" s="63" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B39" s="64" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C39" s="64" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D39" s="64" t="s">
         <v>51</v>
@@ -9798,16 +9842,16 @@
     </row>
     <row r="40">
       <c r="A40" s="4" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B40" s="56" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C40" s="56" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D40" s="56" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E40" s="57">
         <v>1.0</v>
@@ -9818,13 +9862,13 @@
     </row>
     <row r="41">
       <c r="A41" s="11" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B41" s="58" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C41" s="58" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D41" s="58" t="s">
         <v>37</v>
@@ -9838,16 +9882,16 @@
     </row>
     <row r="42">
       <c r="A42" s="11" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B42" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C42" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D42" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E42" s="32"/>
       <c r="F42" s="32"/>
@@ -9859,48 +9903,48 @@
     </row>
     <row r="44">
       <c r="A44" s="4" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B44" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C44" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D44" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E44" s="32"/>
       <c r="F44" s="32"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B45" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C45" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D45" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E45" s="32"/>
       <c r="F45" s="32"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B46" s="61" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C46" s="61" t="s">
         <v>63</v>
       </c>
       <c r="D46" s="61" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="E46" s="57">
         <v>7.0</v>
@@ -9911,16 +9955,16 @@
     </row>
     <row r="47">
       <c r="A47" s="4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B47" s="59" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C47" s="59" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D47" s="59" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E47" s="57">
         <v>4.0</v>
@@ -9931,10 +9975,10 @@
     </row>
     <row r="48">
       <c r="A48" s="4" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B48" s="64" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C48" s="64" t="s">
         <v>51</v>
@@ -9951,16 +9995,16 @@
     </row>
     <row r="49">
       <c r="A49" s="11" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B49" s="60" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C49" s="60" t="s">
         <v>76</v>
       </c>
       <c r="D49" s="60" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E49" s="57">
         <v>6.0</v>
@@ -9976,58 +10020,58 @@
     </row>
     <row r="51">
       <c r="A51" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B51" s="59" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C51" s="59" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D51" s="59" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E51" s="32"/>
       <c r="F51" s="32"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B52" s="58" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C52" s="58" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D52" s="58" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E52" s="32"/>
       <c r="F52" s="32"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B53" s="59" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C53" s="59" t="s">
         <v>40</v>
       </c>
       <c r="D53" s="59" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="E53" s="32"/>
       <c r="F53" s="32"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B54" s="60" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C54" s="60" t="s">
         <v>76</v>
@@ -10040,32 +10084,32 @@
     </row>
     <row r="55">
       <c r="A55" s="11" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B55" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C55" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D55" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E55" s="32"/>
       <c r="F55" s="32"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B56" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C56" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D56" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E56" s="32"/>
       <c r="F56" s="32"/>
@@ -10077,29 +10121,29 @@
     </row>
     <row r="58">
       <c r="A58" s="4" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B58" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C58" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D58" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E58" s="32"/>
       <c r="F58" s="32"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B59" s="56" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C59" s="56" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D59" s="56" t="s">
         <v>59</v>
@@ -10109,64 +10153,64 @@
     </row>
     <row r="60">
       <c r="A60" s="4" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B60" s="60" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C60" s="60" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D60" s="60" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E60" s="32"/>
       <c r="F60" s="32"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B61" s="59" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C61" s="59" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="D61" s="59" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E61" s="32"/>
       <c r="F61" s="32"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B62" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C62" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D62" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E62" s="32"/>
       <c r="F62" s="32"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B63" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C63" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D63" s="65" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E63" s="32"/>
       <c r="F63" s="32"/>
@@ -10177,7 +10221,7 @@
     </row>
     <row r="65">
       <c r="A65" s="4" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B65" s="30" t="s">
         <v>103</v>
@@ -10193,13 +10237,13 @@
     </row>
     <row r="66">
       <c r="A66" s="4" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B66" s="30" t="s">
         <v>103</v>
       </c>
       <c r="C66" s="59" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D66" s="59" t="s">
         <v>59</v>
@@ -10209,13 +10253,13 @@
     </row>
     <row r="67">
       <c r="A67" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B67" s="30" t="s">
         <v>103</v>
       </c>
       <c r="C67" s="59" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D67" s="59" t="s">
         <v>63</v>
@@ -10225,16 +10269,16 @@
     </row>
     <row r="68">
       <c r="A68" s="4" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B68" s="30" t="s">
         <v>103</v>
       </c>
       <c r="C68" s="58" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D68" s="58" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="E68" s="32"/>
       <c r="F68" s="32"/>
@@ -10248,13 +10292,13 @@
     </row>
     <row r="70">
       <c r="A70" s="4" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B70" s="30" t="s">
         <v>103</v>
       </c>
       <c r="C70" s="58" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D70" s="58" t="s">
         <v>51</v>
@@ -10264,13 +10308,13 @@
     </row>
     <row r="71">
       <c r="A71" s="4" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B71" s="30" t="s">
         <v>103</v>
       </c>
       <c r="C71" s="64" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="D71" s="64" t="s">
         <v>53</v>
@@ -10280,13 +10324,13 @@
     </row>
     <row r="72">
       <c r="A72" s="4" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B72" s="30" t="s">
         <v>103</v>
       </c>
       <c r="C72" s="64" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D72" s="64" t="s">
         <v>30</v>
@@ -10296,16 +10340,16 @@
     </row>
     <row r="73">
       <c r="A73" s="4" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B73" s="30" t="s">
         <v>103</v>
       </c>
       <c r="C73" s="60" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D73" s="60" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="E73" s="35"/>
       <c r="F73" s="35"/>
@@ -10317,10 +10361,10 @@
     </row>
     <row r="75">
       <c r="A75" s="4" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B75" s="37" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C75" s="60"/>
       <c r="D75" s="60"/>
@@ -10329,10 +10373,10 @@
     </row>
     <row r="76">
       <c r="A76" s="4" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B76" s="37" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C76" s="59"/>
       <c r="D76" s="59"/>
@@ -10341,10 +10385,10 @@
     </row>
     <row r="77">
       <c r="A77" s="4" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="B77" s="37" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C77" s="58"/>
       <c r="D77" s="58"/>
@@ -10353,10 +10397,10 @@
     </row>
     <row r="78">
       <c r="A78" s="4" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B78" s="37" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C78" s="64"/>
       <c r="D78" s="64"/>
@@ -10369,10 +10413,10 @@
     </row>
     <row r="80">
       <c r="A80" s="4" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="B80" s="37" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C80" s="59"/>
       <c r="D80" s="67"/>
@@ -10381,10 +10425,10 @@
     </row>
     <row r="81">
       <c r="A81" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B81" s="37" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C81" s="64"/>
       <c r="D81" s="60"/>
@@ -10397,10 +10441,10 @@
     </row>
     <row r="83">
       <c r="A83" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C83" s="4"/>
       <c r="D83" s="4"/>
@@ -10409,10 +10453,10 @@
     </row>
     <row r="84">
       <c r="A84" s="4" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C84" s="4"/>
       <c r="D84" s="4"/>
@@ -14100,22 +14144,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="68" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B1" s="41" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" s="42" t="s">
+        <v>128</v>
+      </c>
+      <c r="D1" s="43" t="s">
+        <v>141</v>
+      </c>
+      <c r="E1" s="44" t="s">
+        <v>156</v>
+      </c>
+      <c r="F1" s="45" t="s">
         <v>130</v>
-      </c>
-      <c r="C1" s="42" t="s">
-        <v>124</v>
-      </c>
-      <c r="D1" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="E1" s="44" t="s">
-        <v>152</v>
-      </c>
-      <c r="F1" s="45" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="2">
@@ -14123,19 +14167,19 @@
         <v>76</v>
       </c>
       <c r="B2" s="59" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C2" s="56" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="D2" s="69" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="E2" s="64" t="s">
         <v>30</v>
       </c>
       <c r="F2" s="70" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3">
@@ -14149,27 +14193,27 @@
         <v>104.0</v>
       </c>
       <c r="D3" s="69" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="E3" s="64" t="s">
         <v>51</v>
       </c>
       <c r="F3" s="70" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="60" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B4" s="59" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C4" s="56" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="69" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="E4" s="64" t="s">
         <v>27</v>
@@ -14180,30 +14224,30 @@
     </row>
     <row r="5">
       <c r="A5" s="60" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B5" s="59" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C5" s="56" t="s">
         <v>59</v>
       </c>
       <c r="D5" s="69" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E5" s="64" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="F5" s="70" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="60" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B6" s="59" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>

</xml_diff>

<commit_message>
Dati: recupero Bad Boys-Ricci di Mare al 30/06
Rigenerato da Calend Bocce 2026 (1).xlsx via tools/build_data.py.

Calendario:
- E: Bad Boys vs Ricci di Mare: lun 22/06 23:00 -> mar 30/06 20:30 (recupero)

Risultati e classifiche invariati. Nessuna sovrapposizione di slot (campo unico).
Cache-busting v=202606260903.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -1803,15 +1803,9 @@
       <c r="A28" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>63</v>
-      </c>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
       <c r="E28" s="6"/>
       <c r="F28" s="6"/>
     </row>
@@ -2306,12 +2300,18 @@
       <c r="F59" s="29"/>
     </row>
     <row r="60">
-      <c r="A60" s="22" t="s">
+      <c r="A60" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B60" s="23"/>
-      <c r="C60" s="23"/>
-      <c r="D60" s="23"/>
+      <c r="B60" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="E60" s="26"/>
       <c r="F60" s="26"/>
     </row>

</xml_diff>

<commit_message>
Dati: 2 anticipi di calendario (29/06)
Rigenerato da Calend Bocce 2026 (1).xlsx via tools/build_data.py.

Calendario (anticipi lun 29/06, serata ora 20:30->22:30 compatta):
- H: Ghirarda vs Le Sbocciate: 22:30 -> 20:30
- B: I Toghini vs Lord&Chri: 23:00 -> 22:30

Risultati e classifiche invariati. Nessuna sovrapposizione di slot (campo unico).
Cache-busting v=202606261129.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -2202,12 +2202,18 @@
       <c r="F52" s="20"/>
     </row>
     <row r="53">
-      <c r="A53" s="22" t="s">
+      <c r="A53" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B53" s="23"/>
-      <c r="C53" s="23"/>
-      <c r="D53" s="23"/>
+      <c r="B53" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>24</v>
+      </c>
       <c r="E53" s="26"/>
       <c r="F53" s="26"/>
     </row>
@@ -2263,31 +2269,25 @@
       <c r="A57" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="B57" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>24</v>
+      <c r="B57" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C57" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D57" s="13" t="s">
+        <v>40</v>
       </c>
       <c r="E57" s="26"/>
       <c r="F57" s="26"/>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="s">
+      <c r="A58" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="B58" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C58" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D58" s="13" t="s">
-        <v>40</v>
-      </c>
+      <c r="B58" s="23"/>
+      <c r="C58" s="23"/>
+      <c r="D58" s="23"/>
       <c r="E58" s="26"/>
       <c r="F58" s="26"/>
     </row>

</xml_diff>

<commit_message>
Dati: rimescolamento orari 30/06
Rigenerato da Calend Bocce 2026 (1).xlsx via tools/build_data.py.

Calendario (mar 30/06):
- F: T alla seconda vs I Cavalli: 22:30 -> 21:30
- C: Chocolate Starfishes vs La Coppia: 21:30 -> 22:00
- C: La Coppia vs I Cugini: 22:00 -> 22:30

Risultati e classifiche invariati. Nessuna sovrapposizione di slot (campo unico).
Nota: La Coppia resta con due gare consecutive (22:00 e 22:30, 30 min), accettato.
Cache-busting v=202606261144.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -2335,14 +2335,14 @@
       <c r="A62" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B62" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C62" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="D62" s="21" t="s">
-        <v>78</v>
+      <c r="B62" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C62" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D62" s="17" t="s">
+        <v>44</v>
       </c>
       <c r="E62" s="26"/>
       <c r="F62" s="26"/>
@@ -2355,10 +2355,10 @@
         <v>49</v>
       </c>
       <c r="C63" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D63" s="21" t="s">
         <v>78</v>
-      </c>
-      <c r="D63" s="21" t="s">
-        <v>51</v>
       </c>
       <c r="E63" s="26"/>
       <c r="F63" s="26"/>
@@ -2367,14 +2367,14 @@
       <c r="A64" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="B64" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="C64" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="D64" s="17" t="s">
-        <v>44</v>
+      <c r="B64" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C64" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="D64" s="21" t="s">
+        <v>51</v>
       </c>
       <c r="E64" s="26"/>
       <c r="F64" s="26"/>

</xml_diff>

<commit_message>
Dati: rinvio Beverly INPS-Wood&Beton al 30/06
Rigenerato da Calend Bocce 2026 (1).xlsx via tools/build_data.py.

Calendario:
- A: Beverly INPS vs Wood&Beton: lun 29/06 21:00 -> mar 30/06 23:00 (rinvio)

Risultati e classifiche invariati. Nessuna sovrapposizione di slot (campo unico).
Effetti: buco alle 21:00 del 29/06; 30/06 ora 6 gare fino alle 23:00.
Cache-busting v=202606291014.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -2218,18 +2218,12 @@
       <c r="F53" s="26"/>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="s">
+      <c r="A54" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="B54" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C54" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D54" s="10" t="s">
-        <v>76</v>
-      </c>
+      <c r="B54" s="23"/>
+      <c r="C54" s="23"/>
+      <c r="D54" s="23"/>
       <c r="E54" s="26"/>
       <c r="F54" s="26"/>
     </row>
@@ -2380,12 +2374,18 @@
       <c r="F64" s="26"/>
     </row>
     <row r="65">
-      <c r="A65" s="25" t="s">
+      <c r="A65" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="B65" s="9"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="9"/>
+      <c r="B65" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C65" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65" s="10" t="s">
+        <v>76</v>
+      </c>
       <c r="E65" s="26"/>
       <c r="F65" s="26"/>
     </row>

</xml_diff>

<commit_message>
Classifiche: pareggi a 3 con classifica avulsa (+ 5 risultati)
compute_standings: per i pari-merito a 3+ squadre (triangolo 1-1-1) lo scontro
diretto a coppie e' non transitivo e dava ordini errati (Girone H metteva
Atletico in testa invece di Team Rocket). Ora si usa la classifica avulsa:
vittorie negli scontri diretti -> differenza generale -> punti fatti -> alfabetico.
TDD: aggiunti 2 test sul triangolo; baseline 'expected' aggiornato (B, E, G, H).

Risultati (giocate 38 -> 43):
- B: I Toghini 4-7 Lord&Chri
- E: Bad Boys 7-6 Ricci di Mare; Gnammestrazzi 3-6 Ricci di Mare
- G: Gli Hummarell 11-3 Bocce da Urlo
- H: Ghirarda 10-3 Le Sbocciate

Calendario:
- E: Bad Boys vs Ricci di Mare: mar 30/06 20:30 -> lun 29/06 21:00

Effetto: H -> Team Rocket primo (avulsa); B -> Lord&Chri secondo (diff +7).
Nessuna sovrapposizione di slot (campo unico). Cache-busting v=202606300947.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -2214,18 +2214,32 @@
       <c r="D53" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E53" s="26"/>
-      <c r="F53" s="26"/>
+      <c r="E53" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="F53" s="6">
+        <v>3.0</v>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="22" t="s">
+      <c r="A54" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B54" s="23"/>
-      <c r="C54" s="23"/>
-      <c r="D54" s="23"/>
-      <c r="E54" s="26"/>
-      <c r="F54" s="26"/>
+      <c r="B54" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E54" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="F54" s="6">
+        <v>6.0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="s">
@@ -2240,8 +2254,12 @@
       <c r="D55" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E55" s="26"/>
-      <c r="F55" s="26"/>
+      <c r="E55" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="F55" s="6">
+        <v>6.0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="s">
@@ -2256,8 +2274,12 @@
       <c r="D56" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="E56" s="26"/>
-      <c r="F56" s="26"/>
+      <c r="E56" s="6">
+        <v>11.0</v>
+      </c>
+      <c r="F56" s="6">
+        <v>3.0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="s">
@@ -2272,8 +2294,12 @@
       <c r="D57" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E57" s="26"/>
-      <c r="F57" s="26"/>
+      <c r="E57" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="F57" s="6">
+        <v>7.0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="25" t="s">
@@ -2294,18 +2320,12 @@
       <c r="F59" s="29"/>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="s">
+      <c r="A60" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="B60" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C60" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D60" s="5" t="s">
-        <v>63</v>
-      </c>
+      <c r="B60" s="23"/>
+      <c r="C60" s="23"/>
+      <c r="D60" s="23"/>
       <c r="E60" s="26"/>
       <c r="F60" s="26"/>
     </row>

</xml_diff>

<commit_message>
Dati: chiusa la fase a gironi (5 risultati)
Risultati inseriti (48/48 partite giocate):
- [A] Beverly INPS-Wood&Beton 4-7
- [C] Chocolate Starfishes-La Coppia 9-1
- [C] La Coppia-I Cugini 3-9
- [F] T alla seconda-I Cavalli 5-8
- [G] I Masalen-Bocce da Urlo 3-9

Classifiche aggiornate nei gironi A, C, F, G (baseline expected
in build_data.py allineato di conseguenza). Check campo unico:
nessuna sovrapposizione di slot.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -322,31 +322,31 @@
     <t>martedì 30/06 23:00</t>
   </si>
   <si>
-    <t>giovedì 02/07 20:30</t>
+    <t>giovedì 02/07 21:00</t>
   </si>
   <si>
     <t>OTT</t>
   </si>
   <si>
-    <t>giovedì 02/07 21:15</t>
+    <t>giovedì 02/07 21:30</t>
   </si>
   <si>
     <t>giovedì 02/07 22:00</t>
   </si>
   <si>
-    <t>giovedì 02/07 22:45</t>
-  </si>
-  <si>
-    <t>martedì 07/07 20:30</t>
-  </si>
-  <si>
-    <t>martedì 07/07 21:15</t>
+    <t>giovedì 02/07 22:30</t>
+  </si>
+  <si>
+    <t>martedì 07/07 21:00</t>
+  </si>
+  <si>
+    <t>martedì 07/07 21:30</t>
   </si>
   <si>
     <t>martedì 07/07 22:00</t>
   </si>
   <si>
-    <t>martedì 07/07 22:45</t>
+    <t>mercoledì 08/07 21:00</t>
   </si>
   <si>
     <t>giovedì 09/07 20:30</t>
@@ -2342,8 +2342,12 @@
       <c r="D61" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="E61" s="26"/>
-      <c r="F61" s="26"/>
+      <c r="E61" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="F61" s="6">
+        <v>9.0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="s">
@@ -2358,8 +2362,12 @@
       <c r="D62" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="E62" s="26"/>
-      <c r="F62" s="26"/>
+      <c r="E62" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="F62" s="6">
+        <v>8.0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="s">
@@ -2374,8 +2382,12 @@
       <c r="D63" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="E63" s="26"/>
-      <c r="F63" s="26"/>
+      <c r="E63" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="F63" s="6">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="11" t="s">
@@ -2390,8 +2402,12 @@
       <c r="D64" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="E64" s="26"/>
-      <c r="F64" s="26"/>
+      <c r="E64" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="F64" s="6">
+        <v>9.0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="s">
@@ -2406,8 +2422,12 @@
       <c r="D65" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="E65" s="26"/>
-      <c r="F65" s="26"/>
+      <c r="E65" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="F65" s="6">
+        <v>7.0</v>
+      </c>
     </row>
     <row r="66"/>
     <row r="67"/>
@@ -2505,39 +2525,28 @@
       <c r="F77" s="35"/>
     </row>
     <row r="78">
-      <c r="A78" s="4" t="s">
+      <c r="B78" s="27"/>
+      <c r="C78" s="36"/>
+      <c r="D78" s="36"/>
+      <c r="E78" s="29"/>
+      <c r="F78" s="29"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B78" s="30" t="s">
+      <c r="B79" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C78" s="31"/>
-      <c r="D78" s="31"/>
-      <c r="E78" s="35"/>
-      <c r="F78" s="35"/>
-    </row>
-    <row r="79">
-      <c r="B79" s="27"/>
-      <c r="C79" s="36"/>
-      <c r="D79" s="36"/>
-      <c r="E79" s="29"/>
-      <c r="F79" s="29"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B80" s="37" t="s">
-        <v>112</v>
-      </c>
-      <c r="C80" s="31"/>
-      <c r="D80" s="31"/>
-      <c r="E80" s="38"/>
-      <c r="F80" s="38"/>
-    </row>
+      <c r="C79" s="31"/>
+      <c r="D79" s="31"/>
+      <c r="E79" s="35"/>
+      <c r="F79" s="35"/>
+    </row>
+    <row r="80"/>
     <row r="81">
       <c r="A81" s="4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B81" s="37" t="s">
         <v>112</v>
@@ -2549,44 +2558,46 @@
     </row>
     <row r="82">
       <c r="A82" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B82" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="C82" s="33"/>
-      <c r="D82" s="33"/>
+      <c r="C82" s="31"/>
+      <c r="D82" s="31"/>
       <c r="E82" s="38"/>
       <c r="F82" s="38"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B83" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="C83" s="31"/>
-      <c r="D83" s="31"/>
+      <c r="C83" s="33"/>
+      <c r="D83" s="33"/>
       <c r="E83" s="38"/>
       <c r="F83" s="38"/>
     </row>
     <row r="84">
-      <c r="B84" s="27"/>
-      <c r="C84" s="36"/>
-      <c r="D84" s="36"/>
-      <c r="E84" s="29"/>
-      <c r="F84" s="29"/>
+      <c r="A84" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B84" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="C84" s="31"/>
+      <c r="D84" s="31"/>
+      <c r="E84" s="38"/>
+      <c r="F84" s="38"/>
     </row>
     <row r="85">
-      <c r="A85" s="4"/>
-      <c r="B85" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="C85" s="31"/>
-      <c r="D85" s="31"/>
-      <c r="E85" s="38"/>
-      <c r="F85" s="38"/>
+      <c r="B85" s="27"/>
+      <c r="C85" s="36"/>
+      <c r="D85" s="36"/>
+      <c r="E85" s="29"/>
+      <c r="F85" s="29"/>
     </row>
     <row r="86">
       <c r="A86" s="4"/>
@@ -2599,26 +2610,26 @@
       <c r="F86" s="38"/>
     </row>
     <row r="87">
-      <c r="B87" s="27"/>
-      <c r="C87" s="36"/>
-      <c r="D87" s="36"/>
-      <c r="E87" s="29"/>
-      <c r="F87" s="29"/>
+      <c r="A87" s="4"/>
+      <c r="B87" s="37" t="s">
+        <v>116</v>
+      </c>
+      <c r="C87" s="31"/>
+      <c r="D87" s="31"/>
+      <c r="E87" s="38"/>
+      <c r="F87" s="38"/>
     </row>
     <row r="88">
-      <c r="A88" s="4"/>
-      <c r="B88" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="C88" s="39"/>
-      <c r="D88" s="39"/>
-      <c r="E88" s="4"/>
-      <c r="F88" s="4"/>
+      <c r="B88" s="27"/>
+      <c r="C88" s="36"/>
+      <c r="D88" s="36"/>
+      <c r="E88" s="29"/>
+      <c r="F88" s="29"/>
     </row>
     <row r="89">
       <c r="A89" s="4"/>
       <c r="B89" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C89" s="39"/>
       <c r="D89" s="39"/>
@@ -2626,11 +2637,14 @@
       <c r="F89" s="4"/>
     </row>
     <row r="90">
-      <c r="B90" s="27"/>
-      <c r="C90" s="27"/>
-      <c r="D90" s="27"/>
-      <c r="E90" s="29"/>
-      <c r="F90" s="29"/>
+      <c r="A90" s="4"/>
+      <c r="B90" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C90" s="39"/>
+      <c r="D90" s="39"/>
+      <c r="E90" s="4"/>
+      <c r="F90" s="4"/>
     </row>
     <row r="91">
       <c r="B91" s="27"/>
@@ -8966,13 +8980,6 @@
       <c r="D995" s="27"/>
       <c r="E995" s="29"/>
       <c r="F995" s="29"/>
-    </row>
-    <row r="996">
-      <c r="B996" s="27"/>
-      <c r="C996" s="27"/>
-      <c r="D996" s="27"/>
-      <c r="E996" s="29"/>
-      <c r="F996" s="29"/>
     </row>
   </sheetData>
   <printOptions/>

</xml_diff>

<commit_message>
Dati: ottavo I Toghini-Gli Zebis spostato a gio 09/07 20:00
Unico ottavo fuori dal blocco 02-07/07: si gioca la stessa serata
dei quarti (campo unico, nessuna sovrapposizione di slot). Il vincente
entra nel quarto Q2 delle 21:15.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -364,7 +364,7 @@
     <t>OTT8</t>
   </si>
   <si>
-    <t>mercoledì 08/07 21:00</t>
+    <t>giovedì 09/07 20:00</t>
   </si>
   <si>
     <t>OTT4</t>
@@ -2656,15 +2656,20 @@
       <c r="F79" s="49"/>
     </row>
     <row r="80">
-      <c r="B80" s="43"/>
-      <c r="C80" s="20"/>
-      <c r="D80" s="20"/>
-      <c r="E80" s="20"/>
-      <c r="F80" s="20"/>
+      <c r="A80" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B80" s="51" t="s">
+        <v>119</v>
+      </c>
+      <c r="C80" s="48"/>
+      <c r="D80" s="48"/>
+      <c r="E80" s="52"/>
+      <c r="F80" s="52"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B81" s="51" t="s">
         <v>119</v>
@@ -2676,7 +2681,7 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B82" s="51" t="s">
         <v>119</v>
@@ -2688,7 +2693,7 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B83" s="51" t="s">
         <v>119</v>
@@ -2699,23 +2704,21 @@
       <c r="F83" s="52"/>
     </row>
     <row r="84">
-      <c r="A84" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="B84" s="51" t="s">
-        <v>119</v>
-      </c>
-      <c r="C84" s="48"/>
-      <c r="D84" s="48"/>
-      <c r="E84" s="52"/>
-      <c r="F84" s="52"/>
+      <c r="B84" s="39"/>
+      <c r="C84" s="22"/>
+      <c r="D84" s="22"/>
+      <c r="E84" s="50"/>
+      <c r="F84" s="50"/>
     </row>
     <row r="85">
-      <c r="B85" s="39"/>
-      <c r="C85" s="22"/>
-      <c r="D85" s="22"/>
-      <c r="E85" s="50"/>
-      <c r="F85" s="50"/>
+      <c r="A85" s="5"/>
+      <c r="B85" s="51" t="s">
+        <v>123</v>
+      </c>
+      <c r="C85" s="48"/>
+      <c r="D85" s="48"/>
+      <c r="E85" s="52"/>
+      <c r="F85" s="52"/>
     </row>
     <row r="86">
       <c r="A86" s="5"/>
@@ -2728,26 +2731,26 @@
       <c r="F86" s="52"/>
     </row>
     <row r="87">
-      <c r="A87" s="5"/>
-      <c r="B87" s="51" t="s">
-        <v>123</v>
-      </c>
-      <c r="C87" s="48"/>
-      <c r="D87" s="48"/>
-      <c r="E87" s="52"/>
-      <c r="F87" s="52"/>
+      <c r="B87" s="39"/>
+      <c r="C87" s="22"/>
+      <c r="D87" s="22"/>
+      <c r="E87" s="50"/>
+      <c r="F87" s="50"/>
     </row>
     <row r="88">
-      <c r="B88" s="39"/>
-      <c r="C88" s="22"/>
-      <c r="D88" s="22"/>
-      <c r="E88" s="50"/>
-      <c r="F88" s="50"/>
+      <c r="A88" s="5"/>
+      <c r="B88" s="53" t="s">
+        <v>124</v>
+      </c>
+      <c r="C88" s="48"/>
+      <c r="D88" s="48"/>
+      <c r="E88" s="5"/>
+      <c r="F88" s="5"/>
     </row>
     <row r="89">
       <c r="A89" s="5"/>
       <c r="B89" s="53" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C89" s="48"/>
       <c r="D89" s="48"/>
@@ -2755,14 +2758,11 @@
       <c r="F89" s="5"/>
     </row>
     <row r="90">
-      <c r="A90" s="5"/>
-      <c r="B90" s="53" t="s">
-        <v>125</v>
-      </c>
-      <c r="C90" s="48"/>
-      <c r="D90" s="48"/>
-      <c r="E90" s="5"/>
-      <c r="F90" s="5"/>
+      <c r="B90" s="39"/>
+      <c r="C90" s="40"/>
+      <c r="D90" s="40"/>
+      <c r="E90" s="42"/>
+      <c r="F90" s="42"/>
     </row>
     <row r="91">
       <c r="B91" s="39"/>
@@ -9091,13 +9091,6 @@
       <c r="D994" s="40"/>
       <c r="E994" s="42"/>
       <c r="F994" s="42"/>
-    </row>
-    <row r="995">
-      <c r="B995" s="39"/>
-      <c r="C995" s="40"/>
-      <c r="D995" s="40"/>
-      <c r="E995" s="42"/>
-      <c r="F995" s="42"/>
     </row>
   </sheetData>
   <printOptions/>

</xml_diff>

<commit_message>
Dati: risultati ottavi 02/07 (I Cugini e Gli Hummarell ai quarti)
OTT2 I Cugini 9-2 Ghirarda; OTT3 Team Rocket 5-6 Gli Hummarell. Quarti
numerati QUAR1..QUAR4 nel foglio. Campo unico: nessuna sovrapposizione
(anche il 09/07, con OTT4 alle 20:00 prima dei quarti).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="237">
   <si>
     <t>data e ora</t>
   </si>
@@ -373,319 +373,331 @@
     <t>giovedì 09/07 20:30</t>
   </si>
   <si>
+    <t>QUAR1</t>
+  </si>
+  <si>
+    <t>giovedì 09/07 21:15</t>
+  </si>
+  <si>
+    <t>QUAR2</t>
+  </si>
+  <si>
+    <t>giovedì 09/07 22:00</t>
+  </si>
+  <si>
+    <t>QUAR3</t>
+  </si>
+  <si>
+    <t>giovedì 09/07 22:45</t>
+  </si>
+  <si>
+    <t>QUAR4</t>
+  </si>
+  <si>
+    <t>SEMI</t>
+  </si>
+  <si>
+    <t>FIN 3°</t>
+  </si>
+  <si>
+    <t>FIN 1°</t>
+  </si>
+  <si>
+    <t>Girone A</t>
+  </si>
+  <si>
+    <t>Girone B</t>
+  </si>
+  <si>
+    <t>Girone C</t>
+  </si>
+  <si>
+    <t>Girone D</t>
+  </si>
+  <si>
+    <t>Girone E</t>
+  </si>
+  <si>
+    <t>Girone F</t>
+  </si>
+  <si>
+    <t>Girone G</t>
+  </si>
+  <si>
+    <t>Girone H</t>
+  </si>
+  <si>
+    <t>giovedì 19/06 20:30</t>
+  </si>
+  <si>
+    <t>Girone 3</t>
+  </si>
+  <si>
+    <t>giovedì 19/06 21:00</t>
+  </si>
+  <si>
+    <t>Girone 6</t>
+  </si>
+  <si>
+    <t>Pit e Loki</t>
+  </si>
+  <si>
+    <t>Gemelli Diversi</t>
+  </si>
+  <si>
+    <t>giovedì 19/06 21:30</t>
+  </si>
+  <si>
+    <t>Girone 2</t>
+  </si>
+  <si>
+    <t>Gli Umarells</t>
+  </si>
+  <si>
+    <t>giovedì 19/06 22:00</t>
+  </si>
+  <si>
+    <t>Girone 1</t>
+  </si>
+  <si>
+    <t>Zaccarini</t>
+  </si>
+  <si>
+    <t>AC Picchia</t>
+  </si>
+  <si>
+    <t>giovedì 19/06 22:30</t>
+  </si>
+  <si>
+    <t>Girone 4</t>
+  </si>
+  <si>
+    <t>Sardine e Cipolle</t>
+  </si>
+  <si>
+    <t>Alice e Alex</t>
+  </si>
+  <si>
+    <t>giovedì 19/06 23:00</t>
+  </si>
+  <si>
+    <t>T alla Seconda</t>
+  </si>
+  <si>
+    <t>lunedì 23/06 20:30</t>
+  </si>
+  <si>
+    <t>lunedì 23/06 21:00</t>
+  </si>
+  <si>
+    <t>Salseritos</t>
+  </si>
+  <si>
+    <t>lunedì 23/06 21:30</t>
+  </si>
+  <si>
+    <t>Boaretti</t>
+  </si>
+  <si>
+    <t>lunedì 23/06 22:00</t>
+  </si>
+  <si>
+    <t>104</t>
+  </si>
+  <si>
+    <t>lunedì 23/06 22:30</t>
+  </si>
+  <si>
+    <t>Narcos Ardola</t>
+  </si>
+  <si>
+    <t>lunedì 23/06 23:00</t>
+  </si>
+  <si>
+    <t>Girone 5</t>
+  </si>
+  <si>
+    <t>martedì 24/06 20:30</t>
+  </si>
+  <si>
+    <t>I Bad Boys</t>
+  </si>
+  <si>
+    <t>martedì 24/06 21:00</t>
+  </si>
+  <si>
+    <t>martedì 24/06 21:30</t>
+  </si>
+  <si>
+    <t>I Barsai</t>
+  </si>
+  <si>
+    <t>martedì 24/06 22:00</t>
+  </si>
+  <si>
+    <t>martedì 24/06 22:30</t>
+  </si>
+  <si>
+    <t>Gianni e Pinotto</t>
+  </si>
+  <si>
+    <t>martedì 24/06 23:00</t>
+  </si>
+  <si>
+    <t>I Belli Addormentati</t>
+  </si>
+  <si>
+    <t>mercoledì 25/06 20:30</t>
+  </si>
+  <si>
+    <t>---</t>
+  </si>
+  <si>
+    <t>mercoledì 25/06 21:00</t>
+  </si>
+  <si>
+    <t>mercoledì 25/06 21:30</t>
+  </si>
+  <si>
+    <t>mercoledì 25/06 22:00</t>
+  </si>
+  <si>
+    <t>mercoledì 25/06 22:30</t>
+  </si>
+  <si>
+    <t>mercoledì 25/06 23:00</t>
+  </si>
+  <si>
+    <t>giovedì 26/06 20:30</t>
+  </si>
+  <si>
+    <t>giovedì 26/06 21:00</t>
+  </si>
+  <si>
+    <t>giovedì 26/06 21:30</t>
+  </si>
+  <si>
+    <t>giovedì 26/06 22:00</t>
+  </si>
+  <si>
+    <t>giovedì 26/06 22:30</t>
+  </si>
+  <si>
+    <t>giovedì 26/06 23:00</t>
+  </si>
+  <si>
+    <t>lunedì 30/06 20:30</t>
+  </si>
+  <si>
+    <t>lunedì 30/06 21:00</t>
+  </si>
+  <si>
+    <t>lunedì 30/06 21:30</t>
+  </si>
+  <si>
+    <t>lunedì 30/06 22:00</t>
+  </si>
+  <si>
+    <t>lunedì 30/06 22:30</t>
+  </si>
+  <si>
+    <t>lunedì 30/06 23:00</t>
+  </si>
+  <si>
+    <t>martedì 01/07 20:30</t>
+  </si>
+  <si>
+    <t>martedì 01/07 21:00</t>
+  </si>
+  <si>
+    <t>martedì 01/07 21:30</t>
+  </si>
+  <si>
+    <t>martedì 01/07 22:00</t>
+  </si>
+  <si>
+    <t>martedì 01/07 22:30</t>
+  </si>
+  <si>
+    <t>martedì 01/07 23:00</t>
+  </si>
+  <si>
+    <t>mercoledì 02/07 20:30</t>
+  </si>
+  <si>
+    <t>mercoledì 02/07 21:00</t>
+  </si>
+  <si>
+    <t>mercoledì 02/07 21:30</t>
+  </si>
+  <si>
+    <t>mercoledì 02/07 22:00</t>
+  </si>
+  <si>
+    <t>mercoledì 02/07 22:30</t>
+  </si>
+  <si>
+    <t>mercoledì 02/07 23:00</t>
+  </si>
+  <si>
+    <t>giovedì 03/07 20:30</t>
+  </si>
+  <si>
+    <t>giovedì 03/07 21:00</t>
+  </si>
+  <si>
+    <t>giovedì 03/07 21:30</t>
+  </si>
+  <si>
+    <t>giovedì 03/07 22:00</t>
+  </si>
+  <si>
+    <t>giovedì 03/07 22:30</t>
+  </si>
+  <si>
+    <t>giovedì 03/07 23:00</t>
+  </si>
+  <si>
+    <t>lunedì 07/07 20:30</t>
+  </si>
+  <si>
+    <t>OTT</t>
+  </si>
+  <si>
+    <t>lunedì 07/07 21:15</t>
+  </si>
+  <si>
+    <t>lunedì 07/07 22:00</t>
+  </si>
+  <si>
+    <t>lunedì 07/07 22:45</t>
+  </si>
+  <si>
+    <t>Lord &amp; Chri</t>
+  </si>
+  <si>
+    <t>martedì 08/07 20:30</t>
+  </si>
+  <si>
+    <t>martedì 08/07 21:15</t>
+  </si>
+  <si>
+    <t>Tironi di bocce</t>
+  </si>
+  <si>
+    <t>martedì 08/07 22:00</t>
+  </si>
+  <si>
+    <t>Belli Addormentati</t>
+  </si>
+  <si>
+    <t>martedì 08/07 22:45</t>
+  </si>
+  <si>
+    <t>giovedì 10/07 20:30</t>
+  </si>
+  <si>
     <t>QUAR</t>
-  </si>
-  <si>
-    <t>giovedì 09/07 21:15</t>
-  </si>
-  <si>
-    <t>giovedì 09/07 22:00</t>
-  </si>
-  <si>
-    <t>giovedì 09/07 22:45</t>
-  </si>
-  <si>
-    <t>SEMI</t>
-  </si>
-  <si>
-    <t>FIN 3°</t>
-  </si>
-  <si>
-    <t>FIN 1°</t>
-  </si>
-  <si>
-    <t>Girone A</t>
-  </si>
-  <si>
-    <t>Girone B</t>
-  </si>
-  <si>
-    <t>Girone C</t>
-  </si>
-  <si>
-    <t>Girone D</t>
-  </si>
-  <si>
-    <t>Girone E</t>
-  </si>
-  <si>
-    <t>Girone F</t>
-  </si>
-  <si>
-    <t>Girone G</t>
-  </si>
-  <si>
-    <t>Girone H</t>
-  </si>
-  <si>
-    <t>giovedì 19/06 20:30</t>
-  </si>
-  <si>
-    <t>Girone 3</t>
-  </si>
-  <si>
-    <t>giovedì 19/06 21:00</t>
-  </si>
-  <si>
-    <t>Girone 6</t>
-  </si>
-  <si>
-    <t>Pit e Loki</t>
-  </si>
-  <si>
-    <t>Gemelli Diversi</t>
-  </si>
-  <si>
-    <t>giovedì 19/06 21:30</t>
-  </si>
-  <si>
-    <t>Girone 2</t>
-  </si>
-  <si>
-    <t>Gli Umarells</t>
-  </si>
-  <si>
-    <t>giovedì 19/06 22:00</t>
-  </si>
-  <si>
-    <t>Girone 1</t>
-  </si>
-  <si>
-    <t>Zaccarini</t>
-  </si>
-  <si>
-    <t>AC Picchia</t>
-  </si>
-  <si>
-    <t>giovedì 19/06 22:30</t>
-  </si>
-  <si>
-    <t>Girone 4</t>
-  </si>
-  <si>
-    <t>Sardine e Cipolle</t>
-  </si>
-  <si>
-    <t>Alice e Alex</t>
-  </si>
-  <si>
-    <t>giovedì 19/06 23:00</t>
-  </si>
-  <si>
-    <t>T alla Seconda</t>
-  </si>
-  <si>
-    <t>lunedì 23/06 20:30</t>
-  </si>
-  <si>
-    <t>lunedì 23/06 21:00</t>
-  </si>
-  <si>
-    <t>Salseritos</t>
-  </si>
-  <si>
-    <t>lunedì 23/06 21:30</t>
-  </si>
-  <si>
-    <t>Boaretti</t>
-  </si>
-  <si>
-    <t>lunedì 23/06 22:00</t>
-  </si>
-  <si>
-    <t>104</t>
-  </si>
-  <si>
-    <t>lunedì 23/06 22:30</t>
-  </si>
-  <si>
-    <t>Narcos Ardola</t>
-  </si>
-  <si>
-    <t>lunedì 23/06 23:00</t>
-  </si>
-  <si>
-    <t>Girone 5</t>
-  </si>
-  <si>
-    <t>martedì 24/06 20:30</t>
-  </si>
-  <si>
-    <t>I Bad Boys</t>
-  </si>
-  <si>
-    <t>martedì 24/06 21:00</t>
-  </si>
-  <si>
-    <t>martedì 24/06 21:30</t>
-  </si>
-  <si>
-    <t>I Barsai</t>
-  </si>
-  <si>
-    <t>martedì 24/06 22:00</t>
-  </si>
-  <si>
-    <t>martedì 24/06 22:30</t>
-  </si>
-  <si>
-    <t>Gianni e Pinotto</t>
-  </si>
-  <si>
-    <t>martedì 24/06 23:00</t>
-  </si>
-  <si>
-    <t>I Belli Addormentati</t>
-  </si>
-  <si>
-    <t>mercoledì 25/06 20:30</t>
-  </si>
-  <si>
-    <t>---</t>
-  </si>
-  <si>
-    <t>mercoledì 25/06 21:00</t>
-  </si>
-  <si>
-    <t>mercoledì 25/06 21:30</t>
-  </si>
-  <si>
-    <t>mercoledì 25/06 22:00</t>
-  </si>
-  <si>
-    <t>mercoledì 25/06 22:30</t>
-  </si>
-  <si>
-    <t>mercoledì 25/06 23:00</t>
-  </si>
-  <si>
-    <t>giovedì 26/06 20:30</t>
-  </si>
-  <si>
-    <t>giovedì 26/06 21:00</t>
-  </si>
-  <si>
-    <t>giovedì 26/06 21:30</t>
-  </si>
-  <si>
-    <t>giovedì 26/06 22:00</t>
-  </si>
-  <si>
-    <t>giovedì 26/06 22:30</t>
-  </si>
-  <si>
-    <t>giovedì 26/06 23:00</t>
-  </si>
-  <si>
-    <t>lunedì 30/06 20:30</t>
-  </si>
-  <si>
-    <t>lunedì 30/06 21:00</t>
-  </si>
-  <si>
-    <t>lunedì 30/06 21:30</t>
-  </si>
-  <si>
-    <t>lunedì 30/06 22:00</t>
-  </si>
-  <si>
-    <t>lunedì 30/06 22:30</t>
-  </si>
-  <si>
-    <t>lunedì 30/06 23:00</t>
-  </si>
-  <si>
-    <t>martedì 01/07 20:30</t>
-  </si>
-  <si>
-    <t>martedì 01/07 21:00</t>
-  </si>
-  <si>
-    <t>martedì 01/07 21:30</t>
-  </si>
-  <si>
-    <t>martedì 01/07 22:00</t>
-  </si>
-  <si>
-    <t>martedì 01/07 22:30</t>
-  </si>
-  <si>
-    <t>martedì 01/07 23:00</t>
-  </si>
-  <si>
-    <t>mercoledì 02/07 20:30</t>
-  </si>
-  <si>
-    <t>mercoledì 02/07 21:00</t>
-  </si>
-  <si>
-    <t>mercoledì 02/07 21:30</t>
-  </si>
-  <si>
-    <t>mercoledì 02/07 22:00</t>
-  </si>
-  <si>
-    <t>mercoledì 02/07 22:30</t>
-  </si>
-  <si>
-    <t>mercoledì 02/07 23:00</t>
-  </si>
-  <si>
-    <t>giovedì 03/07 20:30</t>
-  </si>
-  <si>
-    <t>giovedì 03/07 21:00</t>
-  </si>
-  <si>
-    <t>giovedì 03/07 21:30</t>
-  </si>
-  <si>
-    <t>giovedì 03/07 22:00</t>
-  </si>
-  <si>
-    <t>giovedì 03/07 22:30</t>
-  </si>
-  <si>
-    <t>giovedì 03/07 23:00</t>
-  </si>
-  <si>
-    <t>lunedì 07/07 20:30</t>
-  </si>
-  <si>
-    <t>OTT</t>
-  </si>
-  <si>
-    <t>lunedì 07/07 21:15</t>
-  </si>
-  <si>
-    <t>lunedì 07/07 22:00</t>
-  </si>
-  <si>
-    <t>lunedì 07/07 22:45</t>
-  </si>
-  <si>
-    <t>Lord &amp; Chri</t>
-  </si>
-  <si>
-    <t>martedì 08/07 20:30</t>
-  </si>
-  <si>
-    <t>martedì 08/07 21:15</t>
-  </si>
-  <si>
-    <t>Tironi di bocce</t>
-  </si>
-  <si>
-    <t>martedì 08/07 22:00</t>
-  </si>
-  <si>
-    <t>Belli Addormentati</t>
-  </si>
-  <si>
-    <t>martedì 08/07 22:45</t>
-  </si>
-  <si>
-    <t>giovedì 10/07 20:30</t>
   </si>
   <si>
     <t>giovedì 10/07 21:15</t>
@@ -1015,7 +1027,7 @@
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="49" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1083,9 +1095,6 @@
     <xf borderId="1" fillId="10" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
     <xf borderId="1" fillId="11" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
@@ -1105,6 +1114,9 @@
     </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -2526,8 +2538,12 @@
       <c r="D70" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="E70" s="46"/>
-      <c r="F70" s="46"/>
+      <c r="E70" s="46">
+        <v>9.0</v>
+      </c>
+      <c r="F70" s="46">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="s">
@@ -2542,8 +2558,12 @@
       <c r="D71" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E71" s="46"/>
-      <c r="F71" s="46"/>
+      <c r="E71" s="46">
+        <v>5.0</v>
+      </c>
+      <c r="F71" s="46">
+        <v>6.0</v>
+      </c>
     </row>
     <row r="72">
       <c r="B72" s="47"/>
@@ -2662,7 +2682,9 @@
       <c r="B80" s="51" t="s">
         <v>119</v>
       </c>
-      <c r="C80" s="48"/>
+      <c r="C80" s="45" t="s">
+        <v>51</v>
+      </c>
       <c r="D80" s="48"/>
       <c r="E80" s="52"/>
       <c r="F80" s="52"/>
@@ -2672,19 +2694,21 @@
         <v>120</v>
       </c>
       <c r="B81" s="51" t="s">
-        <v>119</v>
-      </c>
-      <c r="C81" s="48"/>
+        <v>121</v>
+      </c>
+      <c r="C81" s="45" t="s">
+        <v>56</v>
+      </c>
       <c r="D81" s="48"/>
       <c r="E81" s="52"/>
       <c r="F81" s="52"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B82" s="51" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C82" s="48"/>
       <c r="D82" s="48"/>
@@ -2693,10 +2717,10 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B83" s="51" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C83" s="48"/>
       <c r="D83" s="48"/>
@@ -2713,7 +2737,7 @@
     <row r="85">
       <c r="A85" s="5"/>
       <c r="B85" s="51" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C85" s="48"/>
       <c r="D85" s="48"/>
@@ -2723,7 +2747,7 @@
     <row r="86">
       <c r="A86" s="5"/>
       <c r="B86" s="51" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C86" s="48"/>
       <c r="D86" s="48"/>
@@ -2740,7 +2764,7 @@
     <row r="88">
       <c r="A88" s="5"/>
       <c r="B88" s="53" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C88" s="48"/>
       <c r="D88" s="48"/>
@@ -2750,7 +2774,7 @@
     <row r="89">
       <c r="A89" s="5"/>
       <c r="B89" s="53" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C89" s="48"/>
       <c r="D89" s="48"/>
@@ -9115,28 +9139,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="54" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B1" s="55" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C1" s="56" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D1" s="57" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E1" s="58" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="F1" s="59" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="G1" s="60" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="H1" s="61" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2">
@@ -9299,10 +9323,10 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B2" s="70" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C2" s="70" t="s">
         <v>21</v>
@@ -9310,237 +9334,237 @@
       <c r="D2" s="70" t="s">
         <v>59</v>
       </c>
-      <c r="E2" s="71">
+      <c r="E2" s="46">
         <v>10.0</v>
       </c>
-      <c r="F2" s="71">
+      <c r="F2" s="46">
         <v>2.0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="B3" s="72" t="s">
-        <v>137</v>
-      </c>
-      <c r="C3" s="72" t="s">
-        <v>138</v>
-      </c>
-      <c r="D3" s="72" t="s">
         <v>139</v>
       </c>
-      <c r="E3" s="71">
+      <c r="B3" s="71" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="71" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="E3" s="46">
         <v>9.0</v>
       </c>
-      <c r="F3" s="71">
+      <c r="F3" s="46">
         <v>3.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B4" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="C4" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="D4" s="73" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" s="72" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4" s="72" t="s">
+        <v>145</v>
+      </c>
+      <c r="D4" s="72" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="71">
+      <c r="E4" s="46">
         <v>2.0</v>
       </c>
-      <c r="F4" s="71">
+      <c r="F4" s="46">
         <v>10.0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="B5" s="74" t="s">
-        <v>144</v>
-      </c>
-      <c r="C5" s="74" t="s">
-        <v>145</v>
-      </c>
-      <c r="D5" s="74" t="s">
         <v>146</v>
       </c>
-      <c r="E5" s="71">
+      <c r="B5" s="73" t="s">
+        <v>147</v>
+      </c>
+      <c r="C5" s="73" t="s">
+        <v>148</v>
+      </c>
+      <c r="D5" s="73" t="s">
+        <v>149</v>
+      </c>
+      <c r="E5" s="46">
         <v>11.0</v>
       </c>
-      <c r="F5" s="71">
+      <c r="F5" s="46">
         <v>0.0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="s">
-        <v>147</v>
-      </c>
-      <c r="B6" s="75" t="s">
-        <v>148</v>
-      </c>
-      <c r="C6" s="75" t="s">
-        <v>149</v>
-      </c>
-      <c r="D6" s="75" t="s">
         <v>150</v>
       </c>
-      <c r="E6" s="71">
+      <c r="B6" s="74" t="s">
+        <v>151</v>
+      </c>
+      <c r="C6" s="74" t="s">
+        <v>152</v>
+      </c>
+      <c r="D6" s="74" t="s">
+        <v>153</v>
+      </c>
+      <c r="E6" s="46">
         <v>4.0</v>
       </c>
-      <c r="F6" s="71">
+      <c r="F6" s="46">
         <v>5.0</v>
       </c>
       <c r="N6" s="17"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="B7" s="74" t="s">
-        <v>144</v>
-      </c>
-      <c r="C7" s="74" t="s">
+        <v>154</v>
+      </c>
+      <c r="B7" s="73" t="s">
+        <v>147</v>
+      </c>
+      <c r="C7" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="74" t="s">
-        <v>152</v>
-      </c>
-      <c r="E7" s="71">
+      <c r="D7" s="73" t="s">
+        <v>155</v>
+      </c>
+      <c r="E7" s="46">
         <v>11.0</v>
       </c>
-      <c r="F7" s="71">
+      <c r="F7" s="46">
         <v>3.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="20"/>
-      <c r="E8" s="76"/>
-      <c r="F8" s="76"/>
+      <c r="E8" s="75"/>
+      <c r="F8" s="75"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="B9" s="74" t="s">
-        <v>144</v>
-      </c>
-      <c r="C9" s="74" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="73" t="s">
+        <v>147</v>
+      </c>
+      <c r="C9" s="73" t="s">
         <v>76</v>
       </c>
-      <c r="D9" s="74" t="s">
-        <v>145</v>
-      </c>
-      <c r="E9" s="71">
+      <c r="D9" s="73" t="s">
+        <v>148</v>
+      </c>
+      <c r="E9" s="46">
         <v>6.0</v>
       </c>
-      <c r="F9" s="71">
+      <c r="F9" s="46">
         <v>7.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B10" s="70" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C10" s="70" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D10" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="71">
+      <c r="E10" s="46">
         <v>4.0</v>
       </c>
-      <c r="F10" s="71">
+      <c r="F10" s="46">
         <v>11.0</v>
       </c>
       <c r="H10" s="26"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="B11" s="72" t="s">
-        <v>137</v>
-      </c>
-      <c r="C11" s="72" t="s">
+        <v>159</v>
+      </c>
+      <c r="B11" s="71" t="s">
+        <v>140</v>
+      </c>
+      <c r="C11" s="71" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="72" t="s">
-        <v>157</v>
-      </c>
-      <c r="E11" s="71">
+      <c r="D11" s="71" t="s">
+        <v>160</v>
+      </c>
+      <c r="E11" s="46">
         <v>10.0</v>
       </c>
-      <c r="F11" s="71">
+      <c r="F11" s="46">
         <v>0.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B12" s="70" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C12" s="70" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D12" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="71">
+      <c r="E12" s="46">
         <v>2.0</v>
       </c>
-      <c r="F12" s="71">
+      <c r="F12" s="46">
         <v>11.0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="77" t="s">
-        <v>160</v>
-      </c>
-      <c r="B13" s="75" t="s">
-        <v>148</v>
-      </c>
-      <c r="C13" s="75" t="s">
+      <c r="A13" s="76" t="s">
+        <v>163</v>
+      </c>
+      <c r="B13" s="74" t="s">
+        <v>151</v>
+      </c>
+      <c r="C13" s="74" t="s">
         <v>63</v>
       </c>
-      <c r="D13" s="75" t="s">
-        <v>161</v>
-      </c>
-      <c r="E13" s="71">
+      <c r="D13" s="74" t="s">
+        <v>164</v>
+      </c>
+      <c r="E13" s="46">
         <v>6.0</v>
       </c>
-      <c r="F13" s="71">
+      <c r="F13" s="46">
         <v>5.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="B14" s="78" t="s">
-        <v>163</v>
-      </c>
-      <c r="C14" s="78" t="s">
+        <v>165</v>
+      </c>
+      <c r="B14" s="77" t="s">
+        <v>166</v>
+      </c>
+      <c r="C14" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="78" t="s">
+      <c r="D14" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="71">
+      <c r="E14" s="46">
         <v>10.0</v>
       </c>
-      <c r="F14" s="71">
+      <c r="F14" s="46">
         <v>3.0</v>
       </c>
       <c r="H14" s="26"/>
@@ -9553,121 +9577,121 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="B16" s="78" t="s">
-        <v>163</v>
-      </c>
-      <c r="C16" s="78" t="s">
+        <v>167</v>
+      </c>
+      <c r="B16" s="77" t="s">
+        <v>166</v>
+      </c>
+      <c r="C16" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="78" t="s">
-        <v>165</v>
-      </c>
-      <c r="E16" s="71">
+      <c r="D16" s="77" t="s">
+        <v>168</v>
+      </c>
+      <c r="E16" s="46">
         <v>8.0</v>
       </c>
-      <c r="F16" s="71">
+      <c r="F16" s="46">
         <v>5.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="B17" s="74" t="s">
-        <v>144</v>
-      </c>
-      <c r="C17" s="74" t="s">
+        <v>169</v>
+      </c>
+      <c r="B17" s="73" t="s">
+        <v>147</v>
+      </c>
+      <c r="C17" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="74" t="s">
-        <v>146</v>
-      </c>
-      <c r="E17" s="71">
+      <c r="D17" s="73" t="s">
+        <v>149</v>
+      </c>
+      <c r="E17" s="46">
         <v>7.0</v>
       </c>
-      <c r="F17" s="71">
+      <c r="F17" s="46">
         <v>4.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="B18" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="C18" s="73" t="s">
+        <v>170</v>
+      </c>
+      <c r="B18" s="72" t="s">
+        <v>144</v>
+      </c>
+      <c r="C18" s="72" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="73" t="s">
-        <v>168</v>
-      </c>
-      <c r="E18" s="71">
+      <c r="D18" s="72" t="s">
+        <v>171</v>
+      </c>
+      <c r="E18" s="46">
         <v>7.0</v>
       </c>
-      <c r="F18" s="71">
+      <c r="F18" s="46">
         <v>5.0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="B19" s="74" t="s">
-        <v>144</v>
-      </c>
-      <c r="C19" s="74" t="s">
+        <v>172</v>
+      </c>
+      <c r="B19" s="73" t="s">
+        <v>147</v>
+      </c>
+      <c r="C19" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="74" t="s">
-        <v>145</v>
-      </c>
-      <c r="E19" s="71">
+      <c r="D19" s="73" t="s">
+        <v>148</v>
+      </c>
+      <c r="E19" s="46">
         <v>9.0</v>
       </c>
-      <c r="F19" s="71">
+      <c r="F19" s="46">
         <v>5.0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B20" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="C20" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="D20" s="73" t="s">
-        <v>171</v>
-      </c>
-      <c r="E20" s="71">
+        <v>173</v>
+      </c>
+      <c r="B20" s="72" t="s">
+        <v>144</v>
+      </c>
+      <c r="C20" s="72" t="s">
+        <v>145</v>
+      </c>
+      <c r="D20" s="72" t="s">
+        <v>174</v>
+      </c>
+      <c r="E20" s="46">
         <v>6.0</v>
       </c>
-      <c r="F20" s="71">
+      <c r="F20" s="46">
         <v>8.0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="B21" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="C21" s="73" t="s">
-        <v>173</v>
-      </c>
-      <c r="D21" s="73" t="s">
-        <v>171</v>
-      </c>
-      <c r="E21" s="71">
+        <v>175</v>
+      </c>
+      <c r="B21" s="72" t="s">
+        <v>144</v>
+      </c>
+      <c r="C21" s="72" t="s">
+        <v>176</v>
+      </c>
+      <c r="D21" s="72" t="s">
+        <v>174</v>
+      </c>
+      <c r="E21" s="46">
         <v>7.0</v>
       </c>
-      <c r="F21" s="71">
+      <c r="F21" s="46">
         <v>3.0</v>
       </c>
     </row>
@@ -9678,117 +9702,117 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="B23" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="C23" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="D23" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
+        <v>177</v>
+      </c>
+      <c r="B23" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="C23" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="D23" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="E23" s="79"/>
+      <c r="F23" s="79"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="B24" s="72" t="s">
-        <v>137</v>
-      </c>
-      <c r="C24" s="72" t="s">
-        <v>139</v>
-      </c>
-      <c r="D24" s="72" t="s">
-        <v>157</v>
-      </c>
-      <c r="E24" s="71">
+        <v>179</v>
+      </c>
+      <c r="B24" s="71" t="s">
+        <v>140</v>
+      </c>
+      <c r="C24" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="D24" s="71" t="s">
+        <v>160</v>
+      </c>
+      <c r="E24" s="46">
         <v>5.0</v>
       </c>
-      <c r="F24" s="71">
+      <c r="F24" s="46">
         <v>7.0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B25" s="70" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C25" s="70" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D25" s="70" t="s">
         <v>59</v>
       </c>
-      <c r="E25" s="71">
+      <c r="E25" s="46">
         <v>5.0</v>
       </c>
-      <c r="F25" s="71">
+      <c r="F25" s="46">
         <v>11.0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="B26" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="C26" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="D26" s="73" t="s">
-        <v>173</v>
-      </c>
-      <c r="E26" s="71">
+        <v>181</v>
+      </c>
+      <c r="B26" s="72" t="s">
+        <v>144</v>
+      </c>
+      <c r="C26" s="72" t="s">
+        <v>145</v>
+      </c>
+      <c r="D26" s="72" t="s">
+        <v>176</v>
+      </c>
+      <c r="E26" s="46">
         <v>8.0</v>
       </c>
-      <c r="F26" s="71">
+      <c r="F26" s="46">
         <v>7.0</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="77" t="s">
-        <v>179</v>
-      </c>
-      <c r="B27" s="75" t="s">
-        <v>148</v>
-      </c>
-      <c r="C27" s="75" t="s">
-        <v>149</v>
-      </c>
-      <c r="D27" s="75" t="s">
-        <v>161</v>
-      </c>
-      <c r="E27" s="71">
+      <c r="A27" s="76" t="s">
+        <v>182</v>
+      </c>
+      <c r="B27" s="74" t="s">
+        <v>151</v>
+      </c>
+      <c r="C27" s="74" t="s">
+        <v>152</v>
+      </c>
+      <c r="D27" s="74" t="s">
+        <v>164</v>
+      </c>
+      <c r="E27" s="46">
         <v>8.0</v>
       </c>
-      <c r="F27" s="71">
+      <c r="F27" s="46">
         <v>3.0</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="77" t="s">
-        <v>180</v>
-      </c>
-      <c r="B28" s="75" t="s">
-        <v>148</v>
-      </c>
-      <c r="C28" s="75" t="s">
+      <c r="A28" s="76" t="s">
+        <v>183</v>
+      </c>
+      <c r="B28" s="74" t="s">
+        <v>151</v>
+      </c>
+      <c r="C28" s="74" t="s">
         <v>63</v>
       </c>
-      <c r="D28" s="75" t="s">
-        <v>150</v>
-      </c>
-      <c r="E28" s="71">
+      <c r="D28" s="74" t="s">
+        <v>153</v>
+      </c>
+      <c r="E28" s="46">
         <v>9.0</v>
       </c>
-      <c r="F28" s="71">
+      <c r="F28" s="46">
         <v>0.0</v>
       </c>
     </row>
@@ -9799,121 +9823,121 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="B30" s="72" t="s">
-        <v>137</v>
-      </c>
-      <c r="C30" s="72" t="s">
-        <v>138</v>
-      </c>
-      <c r="D30" s="72" t="s">
+        <v>184</v>
+      </c>
+      <c r="B30" s="71" t="s">
+        <v>140</v>
+      </c>
+      <c r="C30" s="71" t="s">
+        <v>141</v>
+      </c>
+      <c r="D30" s="71" t="s">
         <v>37</v>
       </c>
-      <c r="E30" s="71">
+      <c r="E30" s="46">
         <v>12.0</v>
       </c>
-      <c r="F30" s="71">
+      <c r="F30" s="46">
         <v>1.0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="B31" s="74" t="s">
-        <v>144</v>
-      </c>
-      <c r="C31" s="74" t="s">
+        <v>185</v>
+      </c>
+      <c r="B31" s="73" t="s">
+        <v>147</v>
+      </c>
+      <c r="C31" s="73" t="s">
         <v>76</v>
       </c>
-      <c r="D31" s="74" t="s">
-        <v>146</v>
-      </c>
-      <c r="E31" s="71">
+      <c r="D31" s="73" t="s">
+        <v>149</v>
+      </c>
+      <c r="E31" s="46">
         <v>5.0</v>
       </c>
-      <c r="F31" s="71">
+      <c r="F31" s="46">
         <v>4.0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="B32" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="C32" s="73" t="s">
+        <v>186</v>
+      </c>
+      <c r="B32" s="72" t="s">
+        <v>144</v>
+      </c>
+      <c r="C32" s="72" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="73" t="s">
-        <v>171</v>
-      </c>
-      <c r="E32" s="71">
+      <c r="D32" s="72" t="s">
+        <v>174</v>
+      </c>
+      <c r="E32" s="46">
         <v>5.0</v>
       </c>
-      <c r="F32" s="71">
+      <c r="F32" s="46">
         <v>4.0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="B33" s="78" t="s">
-        <v>163</v>
-      </c>
-      <c r="C33" s="78" t="s">
+        <v>187</v>
+      </c>
+      <c r="B33" s="77" t="s">
+        <v>166</v>
+      </c>
+      <c r="C33" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="D33" s="78" t="s">
+      <c r="D33" s="77" t="s">
         <v>51</v>
       </c>
-      <c r="E33" s="71">
+      <c r="E33" s="46">
         <v>8.0</v>
       </c>
-      <c r="F33" s="71">
+      <c r="F33" s="46">
         <v>6.0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="B34" s="74" t="s">
-        <v>144</v>
-      </c>
-      <c r="C34" s="74" t="s">
-        <v>145</v>
-      </c>
-      <c r="D34" s="74" t="s">
-        <v>152</v>
-      </c>
-      <c r="E34" s="71">
+        <v>188</v>
+      </c>
+      <c r="B34" s="73" t="s">
+        <v>147</v>
+      </c>
+      <c r="C34" s="73" t="s">
+        <v>148</v>
+      </c>
+      <c r="D34" s="73" t="s">
+        <v>155</v>
+      </c>
+      <c r="E34" s="46">
         <v>9.0</v>
       </c>
-      <c r="F34" s="71">
+      <c r="F34" s="46">
         <v>3.0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="B35" s="78" t="s">
-        <v>163</v>
-      </c>
-      <c r="C35" s="78" t="s">
+        <v>189</v>
+      </c>
+      <c r="B35" s="77" t="s">
+        <v>166</v>
+      </c>
+      <c r="C35" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="D35" s="78" t="s">
-        <v>165</v>
-      </c>
-      <c r="E35" s="71">
+      <c r="D35" s="77" t="s">
+        <v>168</v>
+      </c>
+      <c r="E35" s="46">
         <v>2.0</v>
       </c>
-      <c r="F35" s="71">
+      <c r="F35" s="46">
         <v>10.0</v>
       </c>
     </row>
@@ -9924,115 +9948,115 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="B37" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="C37" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="D37" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="E37" s="46"/>
-      <c r="F37" s="46"/>
+        <v>190</v>
+      </c>
+      <c r="B37" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="C37" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="D37" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="E37" s="79"/>
+      <c r="F37" s="79"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="B38" s="75" t="s">
-        <v>148</v>
-      </c>
-      <c r="C38" s="75" t="s">
-        <v>161</v>
-      </c>
-      <c r="D38" s="75" t="s">
-        <v>150</v>
-      </c>
-      <c r="E38" s="71">
+        <v>191</v>
+      </c>
+      <c r="B38" s="74" t="s">
+        <v>151</v>
+      </c>
+      <c r="C38" s="74" t="s">
+        <v>164</v>
+      </c>
+      <c r="D38" s="74" t="s">
+        <v>153</v>
+      </c>
+      <c r="E38" s="46">
         <v>8.0</v>
       </c>
-      <c r="F38" s="71">
+      <c r="F38" s="46">
         <v>3.0</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="77" t="s">
-        <v>189</v>
-      </c>
-      <c r="B39" s="78" t="s">
-        <v>163</v>
-      </c>
-      <c r="C39" s="78" t="s">
-        <v>165</v>
-      </c>
-      <c r="D39" s="78" t="s">
+      <c r="A39" s="76" t="s">
+        <v>192</v>
+      </c>
+      <c r="B39" s="77" t="s">
+        <v>166</v>
+      </c>
+      <c r="C39" s="77" t="s">
+        <v>168</v>
+      </c>
+      <c r="D39" s="77" t="s">
         <v>51</v>
       </c>
-      <c r="E39" s="71">
+      <c r="E39" s="46">
         <v>7.0</v>
       </c>
-      <c r="F39" s="71">
+      <c r="F39" s="46">
         <v>8.0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B40" s="70" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C40" s="70" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D40" s="70" t="s">
-        <v>159</v>
-      </c>
-      <c r="E40" s="71">
+        <v>162</v>
+      </c>
+      <c r="E40" s="46">
         <v>1.0</v>
       </c>
-      <c r="F40" s="71">
+      <c r="F40" s="46">
         <v>10.0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="B41" s="72" t="s">
-        <v>137</v>
-      </c>
-      <c r="C41" s="72" t="s">
-        <v>139</v>
-      </c>
-      <c r="D41" s="72" t="s">
+        <v>194</v>
+      </c>
+      <c r="B41" s="71" t="s">
+        <v>140</v>
+      </c>
+      <c r="C41" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="D41" s="71" t="s">
         <v>37</v>
       </c>
-      <c r="E41" s="71">
+      <c r="E41" s="46">
         <v>6.0</v>
       </c>
-      <c r="F41" s="71">
+      <c r="F41" s="46">
         <v>7.0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="16" t="s">
-        <v>192</v>
-      </c>
-      <c r="B42" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="C42" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="D42" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="E42" s="46"/>
-      <c r="F42" s="46"/>
+        <v>195</v>
+      </c>
+      <c r="B42" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="C42" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="D42" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="E42" s="79"/>
+      <c r="F42" s="79"/>
     </row>
     <row r="43">
       <c r="A43" s="20"/>
@@ -10041,113 +10065,113 @@
     </row>
     <row r="44">
       <c r="A44" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="B44" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="C44" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="D44" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="E44" s="46"/>
-      <c r="F44" s="46"/>
+        <v>196</v>
+      </c>
+      <c r="B44" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="C44" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="D44" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="E44" s="79"/>
+      <c r="F44" s="79"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="B45" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="C45" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="D45" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="E45" s="46"/>
-      <c r="F45" s="46"/>
+        <v>197</v>
+      </c>
+      <c r="B45" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="C45" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="D45" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="E45" s="79"/>
+      <c r="F45" s="79"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="B46" s="75" t="s">
-        <v>148</v>
-      </c>
-      <c r="C46" s="75" t="s">
+        <v>198</v>
+      </c>
+      <c r="B46" s="74" t="s">
+        <v>151</v>
+      </c>
+      <c r="C46" s="74" t="s">
         <v>63</v>
       </c>
-      <c r="D46" s="75" t="s">
-        <v>149</v>
-      </c>
-      <c r="E46" s="71">
+      <c r="D46" s="74" t="s">
+        <v>152</v>
+      </c>
+      <c r="E46" s="46">
         <v>7.0</v>
       </c>
-      <c r="F46" s="71">
+      <c r="F46" s="46">
         <v>5.0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="B47" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="C47" s="73" t="s">
-        <v>173</v>
-      </c>
-      <c r="D47" s="73" t="s">
-        <v>168</v>
-      </c>
-      <c r="E47" s="71">
+        <v>199</v>
+      </c>
+      <c r="B47" s="72" t="s">
+        <v>144</v>
+      </c>
+      <c r="C47" s="72" t="s">
+        <v>176</v>
+      </c>
+      <c r="D47" s="72" t="s">
+        <v>171</v>
+      </c>
+      <c r="E47" s="46">
         <v>4.0</v>
       </c>
-      <c r="F47" s="71">
+      <c r="F47" s="46">
         <v>6.0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="B48" s="78" t="s">
-        <v>163</v>
-      </c>
-      <c r="C48" s="78" t="s">
+        <v>200</v>
+      </c>
+      <c r="B48" s="77" t="s">
+        <v>166</v>
+      </c>
+      <c r="C48" s="77" t="s">
         <v>51</v>
       </c>
-      <c r="D48" s="78" t="s">
+      <c r="D48" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="E48" s="71">
+      <c r="E48" s="46">
         <v>11.0</v>
       </c>
-      <c r="F48" s="71">
+      <c r="F48" s="46">
         <v>3.0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="s">
-        <v>198</v>
-      </c>
-      <c r="B49" s="74" t="s">
-        <v>144</v>
-      </c>
-      <c r="C49" s="74" t="s">
+        <v>201</v>
+      </c>
+      <c r="B49" s="73" t="s">
+        <v>147</v>
+      </c>
+      <c r="C49" s="73" t="s">
         <v>76</v>
       </c>
-      <c r="D49" s="74" t="s">
-        <v>152</v>
-      </c>
-      <c r="E49" s="71">
+      <c r="D49" s="73" t="s">
+        <v>155</v>
+      </c>
+      <c r="E49" s="46">
         <v>6.0</v>
       </c>
-      <c r="F49" s="71">
+      <c r="F49" s="46">
         <v>7.0</v>
       </c>
     </row>
@@ -10158,99 +10182,99 @@
     </row>
     <row r="51">
       <c r="A51" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="B51" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="C51" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="D51" s="73" t="s">
-        <v>168</v>
-      </c>
-      <c r="E51" s="46"/>
-      <c r="F51" s="46"/>
+        <v>202</v>
+      </c>
+      <c r="B51" s="72" t="s">
+        <v>144</v>
+      </c>
+      <c r="C51" s="72" t="s">
+        <v>145</v>
+      </c>
+      <c r="D51" s="72" t="s">
+        <v>171</v>
+      </c>
+      <c r="E51" s="79"/>
+      <c r="F51" s="79"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="B52" s="72" t="s">
-        <v>137</v>
-      </c>
-      <c r="C52" s="72" t="s">
-        <v>138</v>
-      </c>
-      <c r="D52" s="72" t="s">
-        <v>157</v>
-      </c>
-      <c r="E52" s="46"/>
-      <c r="F52" s="46"/>
+        <v>203</v>
+      </c>
+      <c r="B52" s="71" t="s">
+        <v>140</v>
+      </c>
+      <c r="C52" s="71" t="s">
+        <v>141</v>
+      </c>
+      <c r="D52" s="71" t="s">
+        <v>160</v>
+      </c>
+      <c r="E52" s="79"/>
+      <c r="F52" s="79"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="B53" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="C53" s="73" t="s">
+        <v>204</v>
+      </c>
+      <c r="B53" s="72" t="s">
+        <v>144</v>
+      </c>
+      <c r="C53" s="72" t="s">
         <v>40</v>
       </c>
-      <c r="D53" s="73" t="s">
-        <v>173</v>
-      </c>
-      <c r="E53" s="46"/>
-      <c r="F53" s="46"/>
+      <c r="D53" s="72" t="s">
+        <v>176</v>
+      </c>
+      <c r="E53" s="79"/>
+      <c r="F53" s="79"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="B54" s="74" t="s">
-        <v>144</v>
-      </c>
-      <c r="C54" s="74" t="s">
+        <v>205</v>
+      </c>
+      <c r="B54" s="73" t="s">
+        <v>147</v>
+      </c>
+      <c r="C54" s="73" t="s">
         <v>76</v>
       </c>
-      <c r="D54" s="74" t="s">
+      <c r="D54" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="E54" s="46"/>
-      <c r="F54" s="46"/>
+      <c r="E54" s="79"/>
+      <c r="F54" s="79"/>
     </row>
     <row r="55">
       <c r="A55" s="16" t="s">
-        <v>203</v>
-      </c>
-      <c r="B55" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="C55" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="D55" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="E55" s="46"/>
-      <c r="F55" s="46"/>
+        <v>206</v>
+      </c>
+      <c r="B55" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="C55" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="D55" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="E55" s="79"/>
+      <c r="F55" s="79"/>
     </row>
     <row r="56">
       <c r="A56" s="16" t="s">
-        <v>204</v>
-      </c>
-      <c r="B56" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="C56" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="D56" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="E56" s="46"/>
-      <c r="F56" s="46"/>
+        <v>207</v>
+      </c>
+      <c r="B56" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="C56" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="D56" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="E56" s="79"/>
+      <c r="F56" s="79"/>
     </row>
     <row r="57">
       <c r="A57" s="20"/>
@@ -10259,99 +10283,99 @@
     </row>
     <row r="58">
       <c r="A58" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="B58" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="C58" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="D58" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="E58" s="46"/>
-      <c r="F58" s="46"/>
+        <v>208</v>
+      </c>
+      <c r="B58" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="C58" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="D58" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="E58" s="79"/>
+      <c r="F58" s="79"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B59" s="70" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C59" s="70" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D59" s="70" t="s">
         <v>59</v>
       </c>
-      <c r="E59" s="46"/>
-      <c r="F59" s="46"/>
+      <c r="E59" s="79"/>
+      <c r="F59" s="79"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B60" s="74" t="s">
-        <v>144</v>
-      </c>
-      <c r="C60" s="74" t="s">
-        <v>146</v>
-      </c>
-      <c r="D60" s="74" t="s">
-        <v>152</v>
-      </c>
-      <c r="E60" s="46"/>
-      <c r="F60" s="46"/>
+        <v>210</v>
+      </c>
+      <c r="B60" s="73" t="s">
+        <v>147</v>
+      </c>
+      <c r="C60" s="73" t="s">
+        <v>149</v>
+      </c>
+      <c r="D60" s="73" t="s">
+        <v>155</v>
+      </c>
+      <c r="E60" s="79"/>
+      <c r="F60" s="79"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B61" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="C61" s="73" t="s">
+        <v>211</v>
+      </c>
+      <c r="B61" s="72" t="s">
+        <v>144</v>
+      </c>
+      <c r="C61" s="72" t="s">
+        <v>174</v>
+      </c>
+      <c r="D61" s="72" t="s">
         <v>171</v>
       </c>
-      <c r="D61" s="73" t="s">
-        <v>168</v>
-      </c>
-      <c r="E61" s="46"/>
-      <c r="F61" s="46"/>
+      <c r="E61" s="79"/>
+      <c r="F61" s="79"/>
     </row>
     <row r="62">
       <c r="A62" s="16" t="s">
-        <v>209</v>
-      </c>
-      <c r="B62" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="C62" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="D62" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="E62" s="46"/>
-      <c r="F62" s="46"/>
+        <v>212</v>
+      </c>
+      <c r="B62" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="C62" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="D62" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="E62" s="79"/>
+      <c r="F62" s="79"/>
     </row>
     <row r="63">
       <c r="A63" s="16" t="s">
-        <v>210</v>
-      </c>
-      <c r="B63" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="C63" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="D63" s="79" t="s">
-        <v>175</v>
-      </c>
-      <c r="E63" s="46"/>
-      <c r="F63" s="46"/>
+        <v>213</v>
+      </c>
+      <c r="B63" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="C63" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="D63" s="78" t="s">
+        <v>178</v>
+      </c>
+      <c r="E63" s="79"/>
+      <c r="F63" s="79"/>
     </row>
     <row r="64">
       <c r="E64" s="42"/>
@@ -10359,67 +10383,67 @@
     </row>
     <row r="65">
       <c r="A65" s="5" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B65" s="80" t="s">
-        <v>212</v>
-      </c>
-      <c r="C65" s="74" t="s">
+        <v>215</v>
+      </c>
+      <c r="C65" s="73" t="s">
         <v>21</v>
       </c>
-      <c r="D65" s="74" t="s">
+      <c r="D65" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="E65" s="46"/>
-      <c r="F65" s="46"/>
+      <c r="E65" s="79"/>
+      <c r="F65" s="79"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B66" s="80" t="s">
-        <v>212</v>
-      </c>
-      <c r="C66" s="73" t="s">
-        <v>145</v>
-      </c>
-      <c r="D66" s="73" t="s">
+        <v>215</v>
+      </c>
+      <c r="C66" s="72" t="s">
+        <v>148</v>
+      </c>
+      <c r="D66" s="72" t="s">
         <v>59</v>
       </c>
-      <c r="E66" s="46"/>
-      <c r="F66" s="46"/>
+      <c r="E66" s="79"/>
+      <c r="F66" s="79"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B67" s="80" t="s">
-        <v>212</v>
-      </c>
-      <c r="C67" s="73" t="s">
-        <v>152</v>
-      </c>
-      <c r="D67" s="73" t="s">
+        <v>215</v>
+      </c>
+      <c r="C67" s="72" t="s">
+        <v>155</v>
+      </c>
+      <c r="D67" s="72" t="s">
         <v>63</v>
       </c>
-      <c r="E67" s="46"/>
-      <c r="F67" s="46"/>
+      <c r="E67" s="79"/>
+      <c r="F67" s="79"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="B68" s="80" t="s">
         <v>215</v>
       </c>
-      <c r="B68" s="80" t="s">
-        <v>212</v>
-      </c>
-      <c r="C68" s="72" t="s">
-        <v>216</v>
-      </c>
-      <c r="D68" s="72" t="s">
-        <v>161</v>
-      </c>
-      <c r="E68" s="46"/>
-      <c r="F68" s="46"/>
+      <c r="C68" s="71" t="s">
+        <v>219</v>
+      </c>
+      <c r="D68" s="71" t="s">
+        <v>164</v>
+      </c>
+      <c r="E68" s="79"/>
+      <c r="F68" s="79"/>
     </row>
     <row r="69">
       <c r="B69" s="81"/>
@@ -10430,15 +10454,15 @@
     </row>
     <row r="70">
       <c r="A70" s="5" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B70" s="80" t="s">
-        <v>212</v>
-      </c>
-      <c r="C70" s="72" t="s">
-        <v>138</v>
-      </c>
-      <c r="D70" s="72" t="s">
+        <v>215</v>
+      </c>
+      <c r="C70" s="71" t="s">
+        <v>141</v>
+      </c>
+      <c r="D70" s="71" t="s">
         <v>51</v>
       </c>
       <c r="E70" s="83"/>
@@ -10446,15 +10470,15 @@
     </row>
     <row r="71">
       <c r="A71" s="5" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B71" s="80" t="s">
-        <v>212</v>
-      </c>
-      <c r="C71" s="78" t="s">
-        <v>219</v>
-      </c>
-      <c r="D71" s="78" t="s">
+        <v>215</v>
+      </c>
+      <c r="C71" s="77" t="s">
+        <v>222</v>
+      </c>
+      <c r="D71" s="77" t="s">
         <v>53</v>
       </c>
       <c r="E71" s="83"/>
@@ -10462,15 +10486,15 @@
     </row>
     <row r="72">
       <c r="A72" s="5" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B72" s="80" t="s">
-        <v>212</v>
-      </c>
-      <c r="C72" s="78" t="s">
-        <v>221</v>
-      </c>
-      <c r="D72" s="78" t="s">
+        <v>215</v>
+      </c>
+      <c r="C72" s="77" t="s">
+        <v>224</v>
+      </c>
+      <c r="D72" s="77" t="s">
         <v>30</v>
       </c>
       <c r="E72" s="83"/>
@@ -10478,16 +10502,16 @@
     </row>
     <row r="73">
       <c r="A73" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B73" s="80" t="s">
-        <v>212</v>
-      </c>
-      <c r="C73" s="74" t="s">
-        <v>168</v>
-      </c>
-      <c r="D73" s="74" t="s">
-        <v>149</v>
+        <v>215</v>
+      </c>
+      <c r="C73" s="73" t="s">
+        <v>171</v>
+      </c>
+      <c r="D73" s="73" t="s">
+        <v>152</v>
       </c>
       <c r="E73" s="83"/>
       <c r="F73" s="83"/>
@@ -10499,49 +10523,49 @@
     </row>
     <row r="75">
       <c r="A75" s="5" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B75" s="84" t="s">
-        <v>119</v>
-      </c>
-      <c r="C75" s="74"/>
-      <c r="D75" s="74"/>
+        <v>227</v>
+      </c>
+      <c r="C75" s="73"/>
+      <c r="D75" s="73"/>
       <c r="E75" s="52"/>
       <c r="F75" s="52"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B76" s="84" t="s">
-        <v>119</v>
-      </c>
-      <c r="C76" s="73"/>
-      <c r="D76" s="73"/>
+        <v>227</v>
+      </c>
+      <c r="C76" s="72"/>
+      <c r="D76" s="72"/>
       <c r="E76" s="52"/>
       <c r="F76" s="52"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B77" s="84" t="s">
-        <v>119</v>
-      </c>
-      <c r="C77" s="72"/>
-      <c r="D77" s="72"/>
+        <v>227</v>
+      </c>
+      <c r="C77" s="71"/>
+      <c r="D77" s="71"/>
       <c r="E77" s="52"/>
       <c r="F77" s="52"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B78" s="84" t="s">
-        <v>119</v>
-      </c>
-      <c r="C78" s="78"/>
-      <c r="D78" s="78"/>
+        <v>227</v>
+      </c>
+      <c r="C78" s="77"/>
+      <c r="D78" s="77"/>
       <c r="E78" s="52"/>
       <c r="F78" s="52"/>
     </row>
@@ -10551,25 +10575,25 @@
     </row>
     <row r="80">
       <c r="A80" s="5" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B80" s="84" t="s">
-        <v>123</v>
-      </c>
-      <c r="C80" s="73"/>
+        <v>126</v>
+      </c>
+      <c r="C80" s="72"/>
       <c r="D80" s="85"/>
       <c r="E80" s="52"/>
       <c r="F80" s="52"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B81" s="84" t="s">
-        <v>123</v>
-      </c>
-      <c r="C81" s="78"/>
-      <c r="D81" s="74"/>
+        <v>126</v>
+      </c>
+      <c r="C81" s="77"/>
+      <c r="D81" s="73"/>
       <c r="E81" s="52"/>
       <c r="F81" s="52"/>
     </row>
@@ -10579,10 +10603,10 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C83" s="5"/>
       <c r="D83" s="5"/>
@@ -10591,10 +10615,10 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C84" s="5"/>
       <c r="D84" s="5"/>
@@ -14282,78 +14306,78 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="86" t="s">
+        <v>147</v>
+      </c>
+      <c r="B1" s="55" t="s">
         <v>144</v>
       </c>
-      <c r="B1" s="55" t="s">
+      <c r="C1" s="56" t="s">
+        <v>138</v>
+      </c>
+      <c r="D1" s="57" t="s">
+        <v>151</v>
+      </c>
+      <c r="E1" s="58" t="s">
+        <v>166</v>
+      </c>
+      <c r="F1" s="59" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="73" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="72" t="s">
+        <v>145</v>
+      </c>
+      <c r="C2" s="70" t="s">
+        <v>235</v>
+      </c>
+      <c r="D2" s="87" t="s">
+        <v>236</v>
+      </c>
+      <c r="E2" s="77" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="88" t="s">
         <v>141</v>
       </c>
-      <c r="C1" s="56" t="s">
-        <v>135</v>
-      </c>
-      <c r="D1" s="57" t="s">
-        <v>148</v>
-      </c>
-      <c r="E1" s="58" t="s">
-        <v>163</v>
-      </c>
-      <c r="F1" s="59" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="74" t="s">
-        <v>76</v>
-      </c>
-      <c r="B2" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="C2" s="70" t="s">
-        <v>231</v>
-      </c>
-      <c r="D2" s="87" t="s">
-        <v>232</v>
-      </c>
-      <c r="E2" s="78" t="s">
-        <v>30</v>
-      </c>
-      <c r="F2" s="88" t="s">
-        <v>138</v>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="B3" s="73" t="s">
+      <c r="B3" s="72" t="s">
         <v>40</v>
       </c>
       <c r="C3" s="70">
         <v>104.0</v>
       </c>
       <c r="D3" s="87" t="s">
-        <v>149</v>
-      </c>
-      <c r="E3" s="78" t="s">
+        <v>152</v>
+      </c>
+      <c r="E3" s="77" t="s">
         <v>51</v>
       </c>
       <c r="F3" s="88" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="74" t="s">
-        <v>145</v>
-      </c>
-      <c r="B4" s="73" t="s">
-        <v>173</v>
+      <c r="A4" s="73" t="s">
+        <v>148</v>
+      </c>
+      <c r="B4" s="72" t="s">
+        <v>176</v>
       </c>
       <c r="C4" s="70" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="87" t="s">
-        <v>161</v>
-      </c>
-      <c r="E4" s="78" t="s">
+        <v>164</v>
+      </c>
+      <c r="E4" s="77" t="s">
         <v>27</v>
       </c>
       <c r="F4" s="88" t="s">
@@ -14361,31 +14385,31 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="74" t="s">
-        <v>146</v>
-      </c>
-      <c r="B5" s="73" t="s">
-        <v>171</v>
+      <c r="A5" s="73" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5" s="72" t="s">
+        <v>174</v>
       </c>
       <c r="C5" s="70" t="s">
         <v>59</v>
       </c>
       <c r="D5" s="87" t="s">
-        <v>150</v>
-      </c>
-      <c r="E5" s="78" t="s">
-        <v>165</v>
+        <v>153</v>
+      </c>
+      <c r="E5" s="77" t="s">
+        <v>168</v>
       </c>
       <c r="F5" s="88" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="74" t="s">
-        <v>152</v>
-      </c>
-      <c r="B6" s="73" t="s">
-        <v>168</v>
+      <c r="A6" s="73" t="s">
+        <v>155</v>
+      </c>
+      <c r="B6" s="72" t="s">
+        <v>171</v>
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>

</xml_diff>

<commit_message>
Dati: orari finali (ven 17/07)
Finale 3°/4° posto ven 17/07 20:45; Finale ven 17/07 21:30. Semifinali ancora
senza orario. Campo unico: nessuna sovrapposizione (finali in giornata a se').

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resources/Calend Bocce 2026 (1).xlsx
+++ b/Resources/Calend Bocce 2026 (1).xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="239">
   <si>
     <t>data e ora</t>
   </si>
@@ -397,7 +397,13 @@
     <t>SEMI</t>
   </si>
   <si>
+    <t>venerdì 17/07 20:45</t>
+  </si>
+  <si>
     <t>FIN 3°</t>
+  </si>
+  <si>
+    <t>venerdì 17/07 21:30</t>
   </si>
   <si>
     <t>FIN 1°</t>
@@ -2682,9 +2688,7 @@
       <c r="B80" s="51" t="s">
         <v>119</v>
       </c>
-      <c r="C80" s="45" t="s">
-        <v>51</v>
-      </c>
+      <c r="C80" s="45"/>
       <c r="D80" s="48"/>
       <c r="E80" s="52"/>
       <c r="F80" s="52"/>
@@ -2696,9 +2700,7 @@
       <c r="B81" s="51" t="s">
         <v>121</v>
       </c>
-      <c r="C81" s="45" t="s">
-        <v>56</v>
-      </c>
+      <c r="C81" s="45"/>
       <c r="D81" s="48"/>
       <c r="E81" s="52"/>
       <c r="F81" s="52"/>
@@ -2762,9 +2764,11 @@
       <c r="F87" s="50"/>
     </row>
     <row r="88">
-      <c r="A88" s="5"/>
+      <c r="A88" s="5" t="s">
+        <v>127</v>
+      </c>
       <c r="B88" s="53" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C88" s="48"/>
       <c r="D88" s="48"/>
@@ -2772,9 +2776,11 @@
       <c r="F88" s="5"/>
     </row>
     <row r="89">
-      <c r="A89" s="5"/>
+      <c r="A89" s="5" t="s">
+        <v>129</v>
+      </c>
       <c r="B89" s="53" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C89" s="48"/>
       <c r="D89" s="48"/>
@@ -9139,28 +9145,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="54" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B1" s="55" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C1" s="56" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D1" s="57" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E1" s="58" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F1" s="59" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G1" s="60" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H1" s="61" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2">
@@ -9323,10 +9329,10 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B2" s="70" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C2" s="70" t="s">
         <v>21</v>
@@ -9343,16 +9349,16 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B3" s="71" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C3" s="71" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D3" s="71" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E3" s="46">
         <v>9.0</v>
@@ -9363,13 +9369,13 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B4" s="72" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C4" s="72" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D4" s="72" t="s">
         <v>40</v>
@@ -9383,16 +9389,16 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B5" s="73" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C5" s="73" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D5" s="73" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E5" s="46">
         <v>11.0</v>
@@ -9403,16 +9409,16 @@
     </row>
     <row r="6">
       <c r="A6" s="16" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B6" s="74" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C6" s="74" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D6" s="74" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E6" s="46">
         <v>4.0</v>
@@ -9424,16 +9430,16 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B7" s="73" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C7" s="73" t="s">
         <v>47</v>
       </c>
       <c r="D7" s="73" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E7" s="46">
         <v>11.0</v>
@@ -9449,16 +9455,16 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B9" s="73" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C9" s="73" t="s">
         <v>76</v>
       </c>
       <c r="D9" s="73" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E9" s="46">
         <v>6.0</v>
@@ -9469,13 +9475,13 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B10" s="70" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C10" s="70" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D10" s="70" t="s">
         <v>21</v>
@@ -9490,16 +9496,16 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B11" s="71" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C11" s="71" t="s">
         <v>37</v>
       </c>
       <c r="D11" s="71" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E11" s="46">
         <v>10.0</v>
@@ -9510,13 +9516,13 @@
     </row>
     <row r="12">
       <c r="A12" s="16" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B12" s="70" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C12" s="70" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D12" s="70" t="s">
         <v>21</v>
@@ -9530,16 +9536,16 @@
     </row>
     <row r="13">
       <c r="A13" s="76" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B13" s="74" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C13" s="74" t="s">
         <v>63</v>
       </c>
       <c r="D13" s="74" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E13" s="46">
         <v>6.0</v>
@@ -9550,10 +9556,10 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B14" s="77" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C14" s="77" t="s">
         <v>30</v>
@@ -9577,16 +9583,16 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B16" s="77" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C16" s="77" t="s">
         <v>30</v>
       </c>
       <c r="D16" s="77" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E16" s="46">
         <v>8.0</v>
@@ -9597,16 +9603,16 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B17" s="73" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C17" s="73" t="s">
         <v>47</v>
       </c>
       <c r="D17" s="73" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E17" s="46">
         <v>7.0</v>
@@ -9617,16 +9623,16 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B18" s="72" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C18" s="72" t="s">
         <v>40</v>
       </c>
       <c r="D18" s="72" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E18" s="46">
         <v>7.0</v>
@@ -9637,16 +9643,16 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B19" s="73" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C19" s="73" t="s">
         <v>47</v>
       </c>
       <c r="D19" s="73" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E19" s="46">
         <v>9.0</v>
@@ -9657,16 +9663,16 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B20" s="72" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C20" s="72" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D20" s="72" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E20" s="46">
         <v>6.0</v>
@@ -9677,16 +9683,16 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B21" s="72" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C21" s="72" t="s">
+        <v>178</v>
+      </c>
+      <c r="D21" s="72" t="s">
         <v>176</v>
-      </c>
-      <c r="D21" s="72" t="s">
-        <v>174</v>
       </c>
       <c r="E21" s="46">
         <v>7.0</v>
@@ -9702,32 +9708,32 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B23" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C23" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D23" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E23" s="79"/>
       <c r="F23" s="79"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B24" s="71" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C24" s="71" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D24" s="71" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E24" s="46">
         <v>5.0</v>
@@ -9738,13 +9744,13 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B25" s="70" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C25" s="70" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D25" s="70" t="s">
         <v>59</v>
@@ -9758,16 +9764,16 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B26" s="72" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C26" s="72" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D26" s="72" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E26" s="46">
         <v>8.0</v>
@@ -9778,16 +9784,16 @@
     </row>
     <row r="27">
       <c r="A27" s="76" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B27" s="74" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C27" s="74" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D27" s="74" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E27" s="46">
         <v>8.0</v>
@@ -9798,16 +9804,16 @@
     </row>
     <row r="28">
       <c r="A28" s="76" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B28" s="74" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C28" s="74" t="s">
         <v>63</v>
       </c>
       <c r="D28" s="74" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E28" s="46">
         <v>9.0</v>
@@ -9823,13 +9829,13 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B30" s="71" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C30" s="71" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D30" s="71" t="s">
         <v>37</v>
@@ -9843,16 +9849,16 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B31" s="73" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C31" s="73" t="s">
         <v>76</v>
       </c>
       <c r="D31" s="73" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E31" s="46">
         <v>5.0</v>
@@ -9863,16 +9869,16 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B32" s="72" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C32" s="72" t="s">
         <v>40</v>
       </c>
       <c r="D32" s="72" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E32" s="46">
         <v>5.0</v>
@@ -9883,10 +9889,10 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B33" s="77" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C33" s="77" t="s">
         <v>30</v>
@@ -9903,16 +9909,16 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B34" s="73" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C34" s="73" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D34" s="73" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E34" s="46">
         <v>9.0</v>
@@ -9923,16 +9929,16 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B35" s="77" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C35" s="77" t="s">
         <v>27</v>
       </c>
       <c r="D35" s="77" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E35" s="46">
         <v>2.0</v>
@@ -9948,32 +9954,32 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B37" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C37" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D37" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E37" s="79"/>
       <c r="F37" s="79"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B38" s="74" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C38" s="74" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D38" s="74" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E38" s="46">
         <v>8.0</v>
@@ -9984,13 +9990,13 @@
     </row>
     <row r="39">
       <c r="A39" s="76" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B39" s="77" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C39" s="77" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D39" s="77" t="s">
         <v>51</v>
@@ -10004,16 +10010,16 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B40" s="70" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C40" s="70" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D40" s="70" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E40" s="46">
         <v>1.0</v>
@@ -10024,13 +10030,13 @@
     </row>
     <row r="41">
       <c r="A41" s="16" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B41" s="71" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C41" s="71" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D41" s="71" t="s">
         <v>37</v>
@@ -10044,16 +10050,16 @@
     </row>
     <row r="42">
       <c r="A42" s="16" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B42" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C42" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D42" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E42" s="79"/>
       <c r="F42" s="79"/>
@@ -10065,48 +10071,48 @@
     </row>
     <row r="44">
       <c r="A44" s="5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B44" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C44" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D44" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E44" s="79"/>
       <c r="F44" s="79"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B45" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C45" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D45" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E45" s="79"/>
       <c r="F45" s="79"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B46" s="74" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C46" s="74" t="s">
         <v>63</v>
       </c>
       <c r="D46" s="74" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E46" s="46">
         <v>7.0</v>
@@ -10117,16 +10123,16 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B47" s="72" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C47" s="72" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D47" s="72" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E47" s="46">
         <v>4.0</v>
@@ -10137,10 +10143,10 @@
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B48" s="77" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C48" s="77" t="s">
         <v>51</v>
@@ -10157,16 +10163,16 @@
     </row>
     <row r="49">
       <c r="A49" s="16" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B49" s="73" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C49" s="73" t="s">
         <v>76</v>
       </c>
       <c r="D49" s="73" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E49" s="46">
         <v>6.0</v>
@@ -10182,58 +10188,58 @@
     </row>
     <row r="51">
       <c r="A51" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B51" s="72" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C51" s="72" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D51" s="72" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E51" s="79"/>
       <c r="F51" s="79"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B52" s="71" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C52" s="71" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D52" s="71" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E52" s="79"/>
       <c r="F52" s="79"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B53" s="72" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C53" s="72" t="s">
         <v>40</v>
       </c>
       <c r="D53" s="72" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E53" s="79"/>
       <c r="F53" s="79"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B54" s="73" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C54" s="73" t="s">
         <v>76</v>
@@ -10246,32 +10252,32 @@
     </row>
     <row r="55">
       <c r="A55" s="16" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B55" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C55" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D55" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E55" s="79"/>
       <c r="F55" s="79"/>
     </row>
     <row r="56">
       <c r="A56" s="16" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B56" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C56" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D56" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E56" s="79"/>
       <c r="F56" s="79"/>
@@ -10283,29 +10289,29 @@
     </row>
     <row r="58">
       <c r="A58" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B58" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C58" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D58" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E58" s="79"/>
       <c r="F58" s="79"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B59" s="70" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C59" s="70" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D59" s="70" t="s">
         <v>59</v>
@@ -10315,64 +10321,64 @@
     </row>
     <row r="60">
       <c r="A60" s="5" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B60" s="73" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C60" s="73" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D60" s="73" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E60" s="79"/>
       <c r="F60" s="79"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B61" s="72" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C61" s="72" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D61" s="72" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E61" s="79"/>
       <c r="F61" s="79"/>
     </row>
     <row r="62">
       <c r="A62" s="16" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B62" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C62" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D62" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E62" s="79"/>
       <c r="F62" s="79"/>
     </row>
     <row r="63">
       <c r="A63" s="16" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B63" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C63" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D63" s="78" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E63" s="79"/>
       <c r="F63" s="79"/>
@@ -10383,10 +10389,10 @@
     </row>
     <row r="65">
       <c r="A65" s="5" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B65" s="80" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C65" s="73" t="s">
         <v>21</v>
@@ -10399,13 +10405,13 @@
     </row>
     <row r="66">
       <c r="A66" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B66" s="80" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C66" s="72" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D66" s="72" t="s">
         <v>59</v>
@@ -10415,13 +10421,13 @@
     </row>
     <row r="67">
       <c r="A67" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B67" s="80" t="s">
         <v>217</v>
       </c>
-      <c r="B67" s="80" t="s">
-        <v>215</v>
-      </c>
       <c r="C67" s="72" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D67" s="72" t="s">
         <v>63</v>
@@ -10431,16 +10437,16 @@
     </row>
     <row r="68">
       <c r="A68" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B68" s="80" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C68" s="71" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D68" s="71" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E68" s="79"/>
       <c r="F68" s="79"/>
@@ -10454,13 +10460,13 @@
     </row>
     <row r="70">
       <c r="A70" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B70" s="80" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C70" s="71" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D70" s="71" t="s">
         <v>51</v>
@@ -10470,13 +10476,13 @@
     </row>
     <row r="71">
       <c r="A71" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B71" s="80" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C71" s="77" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D71" s="77" t="s">
         <v>53</v>
@@ -10486,13 +10492,13 @@
     </row>
     <row r="72">
       <c r="A72" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B72" s="80" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C72" s="77" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D72" s="77" t="s">
         <v>30</v>
@@ -10502,16 +10508,16 @@
     </row>
     <row r="73">
       <c r="A73" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B73" s="80" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C73" s="73" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D73" s="73" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E73" s="83"/>
       <c r="F73" s="83"/>
@@ -10523,10 +10529,10 @@
     </row>
     <row r="75">
       <c r="A75" s="5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B75" s="84" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C75" s="73"/>
       <c r="D75" s="73"/>
@@ -10535,10 +10541,10 @@
     </row>
     <row r="76">
       <c r="A76" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B76" s="84" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C76" s="72"/>
       <c r="D76" s="72"/>
@@ -10547,10 +10553,10 @@
     </row>
     <row r="77">
       <c r="A77" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="B77" s="84" t="s">
         <v>229</v>
-      </c>
-      <c r="B77" s="84" t="s">
-        <v>227</v>
       </c>
       <c r="C77" s="71"/>
       <c r="D77" s="71"/>
@@ -10559,10 +10565,10 @@
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B78" s="84" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C78" s="77"/>
       <c r="D78" s="77"/>
@@ -10575,7 +10581,7 @@
     </row>
     <row r="80">
       <c r="A80" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B80" s="84" t="s">
         <v>126</v>
@@ -10587,7 +10593,7 @@
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B81" s="84" t="s">
         <v>126</v>
@@ -10603,10 +10609,10 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C83" s="5"/>
       <c r="D83" s="5"/>
@@ -10615,10 +10621,10 @@
     </row>
     <row r="84">
       <c r="A84" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C84" s="5"/>
       <c r="D84" s="5"/>
@@ -14306,22 +14312,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="86" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B1" s="55" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C1" s="56" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D1" s="57" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E1" s="58" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F1" s="59" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2">
@@ -14329,19 +14335,19 @@
         <v>76</v>
       </c>
       <c r="B2" s="72" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C2" s="70" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D2" s="87" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E2" s="77" t="s">
         <v>30</v>
       </c>
       <c r="F2" s="88" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3">
@@ -14355,27 +14361,27 @@
         <v>104.0</v>
       </c>
       <c r="D3" s="87" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E3" s="77" t="s">
         <v>51</v>
       </c>
       <c r="F3" s="88" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="73" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B4" s="72" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C4" s="70" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="87" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E4" s="77" t="s">
         <v>27</v>
@@ -14386,30 +14392,30 @@
     </row>
     <row r="5">
       <c r="A5" s="73" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B5" s="72" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C5" s="70" t="s">
         <v>59</v>
       </c>
       <c r="D5" s="87" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E5" s="77" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F5" s="88" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="73" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B6" s="72" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>

</xml_diff>